<commit_message>
docs: UI/UX 追蹤清單 Round 3 補登
既有 4 項標記已修正:
- #23 (row 25) 桌面內容截斷無省略提示 → news .item-info line-clamp 2
- #24 (row 26) 純圖示連結缺 aria-label → news 箭頭加 aria-label
- #26 (row 28) 新增 NEW 標籤 → 7 天內消息橘色 NEW pill
- #44 (row 46) 三大核心圖示靜態 → 包入 Dynamic Island morph 卡片

新增 5 項 (#93-#97):
- #93 About 三大核心 Dynamic Island 互動卡片 (提升/互動/中)
- #94 About 成員照片 hover scale (提升/視覺/低)
- #95 About 底部 CTA hover micro-animation (提升/視覺/低)
- #96 News 列表升級浮起卡片 + 入場動畫 + 日期 pill (提升/視覺/中)
- #97 社群外連結加 target=_blank + rel=noopener (修復/互動/低)

統計同步: V 72→77 (88.5%), 合計 82→87
- 最新消息 5→6, 關於長穩 5→8, 共用元件 16→17
- 中優先 36→38, 低優先 40→43, 高+中+低 = 87 ✓

scripts/update-uiux-tracking.mjs 累積三輪改動 (idempotent)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -83,13 +83,8 @@
       <name val="Calibri"/>
       <color rgb="006100"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="9C5700"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -142,12 +137,6 @@
         <bgColor/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -168,7 +157,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -192,9 +181,6 @@
       <alignment vertical="center" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -252,10 +238,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -287,10 +273,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1760,7 +1746,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P94"/>
+  <dimension ref="A1:P99"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="6"/>
     <col min="2" max="2" customWidth="1" width="6"/>
@@ -2656,45 +2642,45 @@
       </c>
     </row>
     <row r="19" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A19" s="10">
+      <c r="A19" s="8">
         <v>17</v>
       </c>
-      <c r="B19" s="10" t="str">
-        <v>V</v>
-      </c>
-      <c r="C19" s="10" t="str">
+      <c r="B19" s="8" t="str">
+        <v>V</v>
+      </c>
+      <c r="C19" s="8" t="str">
         <v>首頁</v>
       </c>
-      <c r="D19" s="10" t="str">
-        <v/>
-      </c>
-      <c r="E19" s="10" t="str">
+      <c r="D19" s="8" t="str">
+        <v/>
+      </c>
+      <c r="E19" s="8" t="str">
         <v>修復</v>
       </c>
-      <c r="F19" s="10" t="str">
+      <c r="F19" s="8" t="str">
         <v>視覺</v>
       </c>
-      <c r="G19" s="10" t="str">
+      <c r="G19" s="8" t="str">
         <v>中</v>
       </c>
-      <c r="H19" s="10" t="str">
+      <c r="H19" s="8" t="str">
         <v>Footer 社群連結呈現不一致</v>
       </c>
-      <c r="I19" s="10" t="str">
+      <c r="I19" s="8" t="str">
         <v>LINE 用 styled button (.btn-line)，Facebook 用純文字圖示連結 (.ic-facebook-before)</v>
       </c>
-      <c r="J19" s="10" t="str">
+      <c r="J19" s="8" t="str">
         <v>統一為相同呈現方式</v>
       </c>
-      <c r="K19" s="10" t="str">
+      <c r="K19" s="8" t="str">
         <v>components/AppFooter.vue</v>
       </c>
-      <c r="L19" s="10" t="str" xml:space="preserve">
+      <c r="L19" s="8" t="str" xml:space="preserve">
         <v xml:space="preserve">components/AppFooter.vue_x000d_
 assets/style/components/_appFooter.scss_x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M19" s="10" t="str">
+      <c r="M19" s="8" t="str">
         <v>兩個社群連結完全不同的 HTML 結構和樣式</v>
       </c>
       <c r="N19" s="9" t="str">
@@ -2967,105 +2953,105 @@
       </c>
     </row>
     <row r="25" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A25" s="3">
+      <c r="A25" s="10">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="str">
+      <c r="B25" s="10" t="str">
         <v>~</v>
       </c>
-      <c r="C25" s="3" t="str">
+      <c r="C25" s="10" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D25" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E25" s="3" t="str">
+      <c r="D25" s="10" t="str">
+        <v/>
+      </c>
+      <c r="E25" s="10" t="str">
         <v>修復</v>
       </c>
-      <c r="F25" s="3" t="str">
+      <c r="F25" s="10" t="str">
         <v>視覺</v>
       </c>
-      <c r="G25" s="3" t="str">
+      <c r="G25" s="10" t="str">
         <v>低</v>
       </c>
-      <c r="H25" s="3" t="str">
+      <c r="H25" s="10" t="str">
         <v>桌面版內容截斷無省略提示</v>
       </c>
-      <c r="I25" s="3" t="str">
+      <c r="I25" s="10" t="str">
         <v>桌面版 .item-info 無 text-overflow 或 line-clamp</v>
       </c>
-      <c r="J25" s="3" t="str">
+      <c r="J25" s="10" t="str">
         <v>加入 text-overflow: ellipsis 或 line-clamp</v>
       </c>
-      <c r="K25" s="3" t="str">
+      <c r="K25" s="10" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L25" s="3" t="str" xml:space="preserve">
+      <c r="L25" s="10" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/news.vue_x000d_
 assets/style/components/_appBody.scss_x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M25" s="3" t="str">
+      <c r="M25" s="10" t="str">
         <v>桌面無省略確認；手機版已有 textLineClamp(2)</v>
       </c>
-      <c r="N25" s="3" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="O25" s="3" t="str">
-        <v/>
-      </c>
-      <c r="P25" s="3" t="str">
-        <v/>
+      <c r="N25" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O25" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P25" s="9" t="str">
+        <v>pages/news.vue 的 .article-item .item-info 加 line-clamp: 2（桌面）/ line-clamp: 3（手機 ≤1024px），超過行數自動省略結尾。</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="3">
+      <c r="A26" s="10">
         <v>24</v>
       </c>
-      <c r="B26" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C26" s="3" t="str">
+      <c r="B26" s="10" t="str">
+        <v>V</v>
+      </c>
+      <c r="C26" s="10" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D26" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E26" s="3" t="str">
+      <c r="D26" s="10" t="str">
+        <v/>
+      </c>
+      <c r="E26" s="10" t="str">
         <v>修復</v>
       </c>
-      <c r="F26" s="3" t="str">
+      <c r="F26" s="10" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G26" s="3" t="str">
+      <c r="G26" s="10" t="str">
         <v>低</v>
       </c>
-      <c r="H26" s="3" t="str">
+      <c r="H26" s="10" t="str">
         <v>純圖示連結缺少 aria-label</v>
       </c>
-      <c r="I26" s="3" t="str">
+      <c r="I26" s="10" t="str">
         <v>&lt;i class="ic-arrow-right"&gt; 無 aria-label/title/隱藏文字</v>
       </c>
-      <c r="J26" s="3" t="str">
+      <c r="J26" s="10" t="str">
         <v>加入 aria-label</v>
       </c>
-      <c r="K26" s="3" t="str">
+      <c r="K26" s="10" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L26" s="3" t="str">
+      <c r="L26" s="10" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="M26" s="3" t="str">
+      <c r="M26" s="10" t="str">
         <v>grep aria-label 全站回傳 0 筆</v>
       </c>
-      <c r="N26" s="3" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="O26" s="3" t="str">
-        <v/>
-      </c>
-      <c r="P26" s="3" t="str">
-        <v/>
+      <c r="N26" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O26" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P26" s="9" t="str">
+        <v>pages/news.vue 的 &lt;i class="ic-arrow-right"&gt; 加上 aria-label="閱讀全文"，符合無障礙語意要求。</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1" xml:space="preserve">
@@ -3120,55 +3106,55 @@
       </c>
     </row>
     <row r="28" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A28" s="3">
+      <c r="A28" s="10">
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C28" s="3" t="str">
+      <c r="B28" s="10" t="str">
+        <v>V</v>
+      </c>
+      <c r="C28" s="10" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E28" s="3" t="str">
+      <c r="D28" s="10" t="str">
+        <v/>
+      </c>
+      <c r="E28" s="10" t="str">
         <v>提升</v>
       </c>
-      <c r="F28" s="3" t="str">
+      <c r="F28" s="10" t="str">
         <v>視覺</v>
       </c>
-      <c r="G28" s="3" t="str">
+      <c r="G28" s="10" t="str">
         <v>低</v>
       </c>
-      <c r="H28" s="3" t="str">
+      <c r="H28" s="10" t="str">
         <v>新增「NEW」標籤</v>
       </c>
-      <c r="I28" s="3" t="str">
+      <c r="I28" s="10" t="str">
         <v>新消息無醒目標示</v>
       </c>
-      <c r="J28" s="3" t="str">
+      <c r="J28" s="10" t="str">
         <v>7 天內的新消息加上 NEW badge</v>
       </c>
-      <c r="K28" s="3" t="str">
+      <c r="K28" s="10" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L28" s="3" t="str" xml:space="preserve">
+      <c r="L28" s="10" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/news.vue_x000d_
 assets/style/components/_appBody.scss_x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M28" s="3" t="str">
+      <c r="M28" s="10" t="str">
         <v>功能確實不存在</v>
       </c>
-      <c r="N28" s="3" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="O28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="P28" s="3" t="str">
-        <v/>
+      <c r="N28" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O28" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P28" s="9" t="str">
+        <v>pages/news.vue 加 isNewItem(releaseTime) helper（7 天內判斷），對應消息右上角顯示橘色 NEW pill 標籤（_appBody.scss .badge-new）。</v>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1" xml:space="preserve">
@@ -4049,55 +4035,55 @@
       </c>
     </row>
     <row r="46" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A46" s="3">
+      <c r="A46" s="10">
         <v>44</v>
       </c>
-      <c r="B46" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C46" s="3" t="str">
+      <c r="B46" s="10" t="str">
+        <v>V</v>
+      </c>
+      <c r="C46" s="10" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D46" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E46" s="3" t="str">
+      <c r="D46" s="10" t="str">
+        <v/>
+      </c>
+      <c r="E46" s="10" t="str">
         <v>提升</v>
       </c>
-      <c r="F46" s="3" t="str">
+      <c r="F46" s="10" t="str">
         <v>視覺</v>
       </c>
-      <c r="G46" s="3" t="str">
+      <c r="G46" s="10" t="str">
         <v>低</v>
       </c>
-      <c r="H46" s="3" t="str">
+      <c r="H46" s="10" t="str">
         <v>三大核心圖示為靜態 SVG</v>
       </c>
-      <c r="I46" s="3" t="str">
+      <c r="I46" s="10" t="str">
         <v>環境保育/人才培育/社會關懷用靜態 &lt;i class="how-logo"&gt;</v>
       </c>
-      <c r="J46" s="3" t="str">
+      <c r="J46" s="10" t="str">
         <v>加入 SVG 動畫</v>
       </c>
-      <c r="K46" s="3" t="str">
+      <c r="K46" s="10" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L46" s="3" t="str" xml:space="preserve">
+      <c r="L46" s="10" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/about.vue_x000d_
 assets/style/components/_appBody_about.scss_x000d_
 assets/style/_animation.scss</v>
       </c>
-      <c r="M46" s="3" t="str">
+      <c r="M46" s="10" t="str">
         <v>確認無任何動畫 class 或 JS</v>
       </c>
-      <c r="N46" s="3" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="O46" s="3" t="str">
-        <v/>
-      </c>
-      <c r="P46" s="3" t="str">
-        <v/>
+      <c r="N46" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O46" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P46" s="9" t="str">
+        <v>icon SVG 本身仍為靜態，但已包入 Dynamic Island 互動卡片（.how-content）：hover/click toggle 觸發整體 morph 動畫（grid-template-rows 展開、translateY 浮起、background opacity overlay 漸層切換、border 露出青綠光暈）。視覺已不再死板。</v>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1">
@@ -5437,46 +5423,46 @@
       </c>
     </row>
     <row r="73" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A73" s="11">
+      <c r="A73" s="5">
         <v>71</v>
       </c>
-      <c r="B73" s="11" t="str">
-        <v>V</v>
-      </c>
-      <c r="C73" s="11" t="str">
+      <c r="B73" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C73" s="5" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D73" s="11" t="str">
-        <v/>
-      </c>
-      <c r="E73" s="11" t="str">
+      <c r="D73" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E73" s="5" t="str">
         <v>修復</v>
       </c>
-      <c r="F73" s="11" t="str">
+      <c r="F73" s="5" t="str">
         <v>RWD</v>
       </c>
-      <c r="G73" s="11" t="str">
+      <c r="G73" s="5" t="str">
         <v>高</v>
       </c>
-      <c r="H73" s="11" t="str">
+      <c r="H73" s="5" t="str">
         <v>多處觸控目標小於 44x44px</v>
       </c>
-      <c r="I73" s="11" t="str">
+      <c r="I73" s="5" t="str">
         <v>分頁按鈕 30x30px、.btn-reset height:32px、.btn-advance height:40px</v>
       </c>
-      <c r="J73" s="11" t="str">
+      <c r="J73" s="5" t="str">
         <v>確保所有可點擊元素最小 44x44px</v>
       </c>
-      <c r="K73" s="11" t="str">
+      <c r="K73" s="5" t="str">
         <v>全站</v>
       </c>
-      <c r="L73" s="11" t="str" xml:space="preserve">
+      <c r="L73" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">assets/style/components/_compPage.scss_x000d_
 assets/style/components/_button.scss_x000d_
 assets/style/components/_compSelect.scss_x000d_
 assets/style/rwd/_rwd_compPage.scss</v>
       </c>
-      <c r="M73" s="11" t="str">
+      <c r="M73" s="5" t="str">
         <v>確認多處尺寸低於 44px 標準</v>
       </c>
       <c r="N73" s="6" t="str">
@@ -6481,6 +6467,262 @@
       </c>
       <c r="P94" s="9" t="str">
         <v>改版補登；同步修桌面 1025-1280px overflow（加 FB 後 .card-more 內容寬度 ~1300px 會爆）：.card-more 加 flex-wrap: wrap + max-width: calc(100% - 64px)；.info-more 加 max-width: 480px 讓長文字桌面換 2 行</v>
+      </c>
+    </row>
+    <row r="95" xml:space="preserve">
+      <c r="A95" s="9">
+        <v>93</v>
+      </c>
+      <c r="B95" s="9" t="str">
+        <v>V</v>
+      </c>
+      <c r="C95" s="9" t="str">
+        <v>關於長穩</v>
+      </c>
+      <c r="D95" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E95" s="9" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F95" s="9" t="str">
+        <v>互動</v>
+      </c>
+      <c r="G95" s="9" t="str">
+        <v>中</v>
+      </c>
+      <c r="H95" s="9" t="str">
+        <v>About 三大核心介紹缺乏互動性</v>
+      </c>
+      <c r="I95" s="9" t="str">
+        <v>環境保育/人才培育/社會關懷三張卡片原為靜態圖文，使用者掃過無視覺反應，缺乏吸引點擊探索的動機</v>
+      </c>
+      <c r="J95" s="9" t="str">
+        <v>改造為 iOS Dynamic Island 風格 morph 卡片：暖象牙白漸層底 + 圓角 28px + 預設只露 icon+標題 → hover/click toggle 平滑展開內文（grid-template-rows trick）+ translateY 浮起 + 邊框露出青綠光暈</v>
+      </c>
+      <c r="K95" s="9" t="str">
+        <v>pages/about.vue</v>
+      </c>
+      <c r="L95" s="9" t="str" xml:space="preserve">
+        <v xml:space="preserve">iFare_Frontend/pages/about.vue_x000d_
+assets/style/components/_appBody_about.scss_x000d_
+assets/style/rwd/_rwd_about.scss</v>
+      </c>
+      <c r="M95" s="9" t="str">
+        <v>改版補登；HTML 重組（icon+title 合進 .how-top、info 包 .how-info-wrap）；script 加 activeHow ref + toggleHow handler；keyboard a11y (Enter/Space) 與 tabindex；GPU 優化（will-change + ::before opacity overlay 取代 gradient transition）；Apple spring easing cubic-bezier(0.32, 0.72, 0, 1)</v>
+      </c>
+      <c r="N95" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O95" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P95" s="9" t="str">
+        <v>改版補登；對應 #44 三大核心圖示靜態問題已連動修正</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9">
+        <v>94</v>
+      </c>
+      <c r="B96" s="9" t="str">
+        <v>V</v>
+      </c>
+      <c r="C96" s="9" t="str">
+        <v>關於長穩</v>
+      </c>
+      <c r="D96" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E96" s="9" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F96" s="9" t="str">
+        <v>視覺</v>
+      </c>
+      <c r="G96" s="9" t="str">
+        <v>低</v>
+      </c>
+      <c r="H96" s="9" t="str">
+        <v>About 成員照片缺 hover 互動</v>
+      </c>
+      <c r="I96" s="9" t="str">
+        <v>陳進財/鄔筠軒/顏杏蓉三位成員區塊原無 hover 反饋，掃過時視覺無變化</v>
+      </c>
+      <c r="J96" s="9" t="str">
+        <v>陳進財/鄔筠軒整組 hover：照片 scale(1.06) + 白框 scale(1.03) + box-shadow 加深 + 橘色標牌 translateY(-4px)；顏杏蓉（無照片）標牌 hover translateY(-4px) + scale(1.04)</v>
+      </c>
+      <c r="K96" s="9" t="str">
+        <v>pages/about.vue</v>
+      </c>
+      <c r="L96" s="9" t="str">
+        <v>iFare_Frontend/assets/style/components/_appBody_about.scss</v>
+      </c>
+      <c r="M96" s="9" t="str">
+        <v>改版補登；同套 cubic-bezier(0.32, 0.72, 0, 1) easing；will-change: transform 給 .member-photo 預先建 GPU layer</v>
+      </c>
+      <c r="N96" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O96" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P96" s="9" t="str">
+        <v>改版補登</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9">
+        <v>95</v>
+      </c>
+      <c r="B97" s="9" t="str">
+        <v>V</v>
+      </c>
+      <c r="C97" s="9" t="str">
+        <v>關於長穩</v>
+      </c>
+      <c r="D97" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E97" s="9" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F97" s="9" t="str">
+        <v>視覺</v>
+      </c>
+      <c r="G97" s="9" t="str">
+        <v>低</v>
+      </c>
+      <c r="H97" s="9" t="str">
+        <v>About 底部 CTA 連結缺 hover micro-animation</v>
+      </c>
+      <c r="I97" s="9" t="str">
+        <v>「前往 i-Fare」與「查看最新消息」兩個 advance-link 原為靜態，hover 無互動反饋，無法強化「點我前進」訊號</v>
+      </c>
+      <c r="J97" s="9" t="str">
+        <v>連結 hover 時 translateY(-2px) 上浮，箭頭 icon translateX(6px) 向右滑出，引導視線前進</v>
+      </c>
+      <c r="K97" s="9" t="str">
+        <v>pages/about.vue</v>
+      </c>
+      <c r="L97" s="9" t="str">
+        <v>iFare_Frontend/assets/style/components/_appBody_about.scss</v>
+      </c>
+      <c r="M97" s="9" t="str">
+        <v>改版補登；統一 cubic-bezier(0.32, 0.72, 0, 1) easing 0.22s</v>
+      </c>
+      <c r="N97" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O97" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P97" s="9" t="str">
+        <v>改版補登</v>
+      </c>
+    </row>
+    <row r="98" xml:space="preserve">
+      <c r="A98" s="9">
+        <v>96</v>
+      </c>
+      <c r="B98" s="9" t="str">
+        <v>V</v>
+      </c>
+      <c r="C98" s="9" t="str">
+        <v>最新消息</v>
+      </c>
+      <c r="D98" s="9" t="str">
+        <v/>
+      </c>
+      <c r="E98" s="9" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F98" s="9" t="str">
+        <v>視覺</v>
+      </c>
+      <c r="G98" s="9" t="str">
+        <v>中</v>
+      </c>
+      <c r="H98" s="9" t="str">
+        <v>News 列表呈現升級為浮起卡片 + 入場動畫 + 日期 pill</v>
+      </c>
+      <c r="I98" s="9" t="str">
+        <v>原本最新消息為「底線分隔的清單列」，hover 只是淡白底 + 箭頭轉橘，視覺扁平、缺乏互動感、日期不醒目、長內文無截斷</v>
+      </c>
+      <c r="J98" s="9" t="str">
+        <v>列表整體升級：圓角 16px 浮起卡片（white .7 + shadow）+ stagger fade-up 入場動畫（@for 1~12 each +50ms）+ 日期變橘色 pill 標籤（border + 半透明橘底）+ hover translateY(-3px) + 背景變實白 + 箭頭橘色滑右 6px</v>
+      </c>
+      <c r="K98" s="9" t="str">
+        <v>pages/news.vue</v>
+      </c>
+      <c r="L98" s="9" t="str" xml:space="preserve">
+        <v xml:space="preserve">iFare_Frontend/pages/news.vue_x000d_
+assets/style/components/_appBody.scss_x000d_
+assets/style/_animation.scss_x000d_
+assets/style/rwd/_rwd.scss</v>
+      </c>
+      <c r="M98" s="9" t="str">
+        <v>改版補登；@keyframes newsItemEnter 放 _animation.scss；統一 cubic-bezier(0.32, 0.72, 0, 1) easing；配色全用既有 token 沒引入新色</v>
+      </c>
+      <c r="N98" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O98" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P98" s="9" t="str">
+        <v>改版補登；同次改動連帶解決 #23 (line-clamp 2)、#24 (aria-label)、#26 (NEW badge)</v>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
+      <c r="A99" s="9">
+        <v>97</v>
+      </c>
+      <c r="B99" s="9" t="str">
+        <v>V</v>
+      </c>
+      <c r="C99" s="9" t="str">
+        <v>共用元件</v>
+      </c>
+      <c r="D99" s="9" t="str">
+        <v>AppFooter / AppHeader</v>
+      </c>
+      <c r="E99" s="9" t="str">
+        <v>修復</v>
+      </c>
+      <c r="F99" s="9" t="str">
+        <v>互動</v>
+      </c>
+      <c r="G99" s="9" t="str">
+        <v>低</v>
+      </c>
+      <c r="H99" s="9" t="str">
+        <v>社群外連結未開新分頁，可能丟失當前頁狀態</v>
+      </c>
+      <c r="I99" s="9" t="str">
+        <v>AppFooter LINE/Facebook 與 AppHeader 手機版社群 icon 連結原為一般 &lt;a href&gt;，點擊會在當前分頁導向，使用者離開站內後返回成本高</v>
+      </c>
+      <c r="J99" s="9" t="str">
+        <v>4 個社群連結都加 target="_blank" + rel="noopener noreferrer"：開新分頁、避免反向 tabnabbing、不洩漏 referrer</v>
+      </c>
+      <c r="K99" s="9" t="str">
+        <v>components/AppFooter.vue components/AppHeader.vue</v>
+      </c>
+      <c r="L99" s="9" t="str" xml:space="preserve">
+        <v xml:space="preserve">iFare_Frontend/components/AppFooter.vue_x000d_
+iFare_Frontend/components/AppHeader.vue</v>
+      </c>
+      <c r="M99" s="9" t="str">
+        <v>改版補登；rel="noopener" 是 W3C 安全建議</v>
+      </c>
+      <c r="N99" s="9" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O99" s="9" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="P99" s="9" t="str">
+        <v>改版補登</v>
       </c>
     </row>
   </sheetData>
@@ -6490,7 +6732,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P99"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6529,10 +6771,10 @@
         <v>V 確認</v>
       </c>
       <c r="B3" s="2">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C3" s="2" t="str">
-        <v>87.8%</v>
+        <v>88.5%</v>
       </c>
       <c r="D3" s="3" t="str">
         <v>經程式碼驗證確認問題存在</v>
@@ -6546,7 +6788,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="2" t="str">
-        <v>12.2%</v>
+        <v>11.5%</v>
       </c>
       <c r="D4" s="3" t="str">
         <v>問題存在但原描述部分不正確，已修正描述</v>
@@ -6557,13 +6799,13 @@
         <v>合計</v>
       </c>
       <c r="B5" s="2">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C5" s="3" t="str">
         <v>100%</v>
       </c>
       <c r="D5" s="2" t="str">
-        <v>已移除 8 項原始盤點中不正確的項目；2026-04-28 補登 5 項改版實作項目（#88/#89/#90/#91/#92）</v>
+        <v>已移除 8 項原始盤點中不正確的項目；2026-04-28 補登 10 項改版實作項目（#88-#97）</v>
       </c>
     </row>
     <row r="7" ht="16.2" customHeight="1">
@@ -6620,11 +6862,11 @@
       <c r="B11" s="3">
         <v>3</v>
       </c>
-      <c r="C11" s="3">
-        <v>2</v>
-      </c>
-      <c r="D11" s="3">
-        <v>5</v>
+      <c r="C11" s="2">
+        <v>3</v>
+      </c>
+      <c r="D11" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="12" ht="16.2" customHeight="1">
@@ -6662,25 +6904,25 @@
       <c r="B14" s="3">
         <v>2</v>
       </c>
-      <c r="C14" s="3">
-        <v>3</v>
-      </c>
-      <c r="D14" s="3">
-        <v>5</v>
+      <c r="C14" s="2">
+        <v>6</v>
+      </c>
+      <c r="D14" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="16.2" customHeight="1">
       <c r="A15" s="3" t="str">
         <v>共用元件</v>
       </c>
-      <c r="B15" s="3">
-        <v>14</v>
+      <c r="B15" s="2">
+        <v>15</v>
       </c>
       <c r="C15" s="2">
         <v>2</v>
       </c>
       <c r="D15" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" ht="16.2" customHeight="1">
@@ -6730,13 +6972,13 @@
         <v>合計</v>
       </c>
       <c r="B19" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C19" s="2">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D19" s="2">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" ht="16.2" customHeight="1">
@@ -6780,10 +7022,10 @@
         <v>27</v>
       </c>
       <c r="C24" s="2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D24" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" ht="16.2" customHeight="1">
@@ -6791,13 +7033,13 @@
         <v>低</v>
       </c>
       <c r="B25" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D25" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(xlsx): 清掉壞掉的 _xlnm._FilterDatabase 範圍 (UIUX sheet 看起來空白的根因)
之前 round 2 時 xlsx 內被自動產生 _xlnm._FilterDatabase Name
指向 'UIUX問題追蹤清單'!A2:O79，但後續 round 5/8/9 擴展到 P133，
這個 stale filter 範圍讓 Excel 開檔時部分 row 不顯示。

修復:
- 清空 wb.Workbook.Names
- 清空各 sheet !autofilter
- repair-xlsx-bloat.mjs 加上同樣邏輯，未來自動處理

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -8,9 +8,6 @@
     <sheet name="UIUX問題追蹤清單" sheetId="3" r:id="rId3"/>
     <sheet name="統計摘要" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'UIUX問題追蹤清單'!A2:O79</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -39,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -48,8 +45,28 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="9C5700"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="9C5700"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="006100"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="006100"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -57,6 +74,30 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -80,16 +121,23 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -145,10 +193,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -180,10 +228,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -4054,53 +4102,53 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="str">
+      <c r="B3" s="5" t="str">
         <v>~</v>
       </c>
-      <c r="C3" s="3" t="str">
+      <c r="C3" s="5" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D3" s="3" t="str">
+      <c r="D3" s="5" t="str">
         <v>搜尋介面</v>
       </c>
-      <c r="E3" s="3" t="str">
+      <c r="E3" s="5" t="str">
         <v>修復</v>
       </c>
-      <c r="F3" s="3" t="str">
+      <c r="F3" s="5" t="str">
         <v>互動</v>
       </c>
-      <c r="G3" s="3" t="str">
+      <c r="G3" s="5" t="str">
         <v>高</v>
       </c>
-      <c r="H3" s="3" t="str">
+      <c r="H3" s="5" t="str">
         <v>篩選條件不完整時無錯誤訊息</v>
       </c>
-      <c r="I3" s="3" t="str">
+      <c r="I3" s="5" t="str">
         <v>按鈕變灰(disabled)但使用者不知道缺哪個欄位，Search()直接 return false 無任何提示</v>
       </c>
-      <c r="J3" s="3" t="str">
+      <c r="J3" s="5" t="str">
         <v>加入未填欄位紅框提示 + 錯誤文字</v>
       </c>
-      <c r="K3" s="3" t="str">
+      <c r="K3" s="5" t="str">
         <v>pages/ifare.vue</v>
       </c>
-      <c r="L3" s="3" t="str" xml:space="preserve">
+      <c r="L3" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/ifare.vue_x000d__x000d__x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M3" s="3" t="str">
+      <c r="M3" s="5" t="str">
         <v>無錯誤訊息確認；但「(必填)」標示已存在於 _font.scss</v>
       </c>
-      <c r="N3" s="3" t="str">
+      <c r="N3" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O3" s="3" t="str">
+      <c r="O3" s="5" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P3" s="3" t="str">
+      <c r="P3" s="5" t="str">
         <v>已移除三項都空時的 disabled 條件（pages/ifare.vue:75 + pages/ifare/result.vue 三處），改用 hasAnyCondition 顯示「未填條件將顯示最新福利」提示。改採「不阻擋 + 引導文案」策略，與原建議「未填欄位紅框 + 錯誤文字」方向不同。</v>
       </c>
     </row>
@@ -4463,54 +4511,54 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A11" s="3">
+      <c r="A11" s="5">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C11" s="3" t="str">
+      <c r="B11" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C11" s="5" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D11" s="3" t="str">
+      <c r="D11" s="5" t="str">
         <v>查詢結果</v>
       </c>
-      <c r="E11" s="3" t="str">
+      <c r="E11" s="5" t="str">
         <v>提升</v>
       </c>
-      <c r="F11" s="3" t="str">
+      <c r="F11" s="5" t="str">
         <v>視覺</v>
       </c>
-      <c r="G11" s="3" t="str">
+      <c r="G11" s="5" t="str">
         <v>低</v>
       </c>
-      <c r="H11" s="3" t="str">
+      <c r="H11" s="5" t="str">
         <v>搜尋結果數量不夠醒目</v>
       </c>
-      <c r="I11" s="3" t="str">
+      <c r="I11" s="5" t="str">
         <v>結果數量 font-size:14px font-weight:400，周圍文字 opacity:0.5</v>
       </c>
-      <c r="J11" s="3" t="str">
+      <c r="J11" s="5" t="str">
         <v>頂部大字顯示 + 計數動畫</v>
       </c>
-      <c r="K11" s="3" t="str">
+      <c r="K11" s="5" t="str">
         <v>pages/ifare/result.vue</v>
       </c>
-      <c r="L11" s="3" t="str" xml:space="preserve">
+      <c r="L11" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/ifare/result.vue_x000d__x000d__x000d_
 assets/style/components/_appBodyChild_ifare.scss_x000d__x000d__x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M11" s="3" t="str">
+      <c r="M11" s="5" t="str">
         <v>確認字體小且無強調</v>
       </c>
-      <c r="N11" s="3" t="str">
+      <c r="N11" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O11" s="3" t="str">
+      <c r="O11" s="5" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P11" s="3" t="str">
+      <c r="P11" s="5" t="str">
         <v>結果摘要從「{{count}}」改寫為「共找到 X 項，僅顯示前 X 筆」(pages/ifare/result.vue)；.result-total 從 inline-flex + ::before 結構簡化為 inline；新增 .result-summary-note 樣式。原訴求「頂部大字 + 計數動畫」尚未做。</v>
       </c>
     </row>
@@ -4822,106 +4870,106 @@
       </c>
     </row>
     <row r="18" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A18" s="3">
+      <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C18" s="3" t="str">
+      <c r="B18" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C18" s="7" t="str">
         <v>首頁</v>
       </c>
-      <c r="D18" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E18" s="3" t="str">
+      <c r="D18" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E18" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F18" s="3" t="str">
+      <c r="F18" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G18" s="3" t="str">
+      <c r="G18" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H18" s="3" t="str">
+      <c r="H18" s="7" t="str">
         <v>頁面切換無轉場動畫</v>
       </c>
-      <c r="I18" s="3" t="str">
+      <c r="I18" s="7" t="str">
         <v>layouts/default.vue 用 &lt;slot /&gt; 無 &lt;Transition&gt;，nuxt.config 無 pageTransition</v>
       </c>
-      <c r="J18" s="3" t="str">
+      <c r="J18" s="7" t="str">
         <v>加入 Nuxt &lt;transition&gt; 過場效果</v>
       </c>
-      <c r="K18" s="3" t="str">
+      <c r="K18" s="7" t="str">
         <v>layouts/default.vue</v>
       </c>
-      <c r="L18" s="3" t="str" xml:space="preserve">
+      <c r="L18" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">layouts/default.vue_x000d__x000d__x000d_
 nuxt.config.ts_x000d__x000d__x000d_
 assets/style/_transition.scss</v>
       </c>
-      <c r="M18" s="3" t="str">
+      <c r="M18" s="7" t="str">
         <v>確認無任何 transition 設定</v>
       </c>
-      <c r="N18" s="3" t="str">
+      <c r="N18" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O18" s="3" t="str">
+      <c r="O18" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P18" s="3" t="str">
+      <c r="P18" s="7" t="str">
         <v>app.vue 加 &lt;NuxtPage :transition="{ name: 'page', mode: 'out-in' }" /&gt;；_animation.scss 新增 .page-enter/leave-active 與 .layout-enter/leave-active keyframes（opacity + translateY，純 GPU 屬性）。</v>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A19" s="3">
+      <c r="A19" s="7">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C19" s="3" t="str">
+      <c r="B19" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C19" s="7" t="str">
         <v>首頁</v>
       </c>
-      <c r="D19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E19" s="3" t="str">
+      <c r="D19" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E19" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F19" s="3" t="str">
+      <c r="F19" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G19" s="3" t="str">
+      <c r="G19" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H19" s="3" t="str">
+      <c r="H19" s="7" t="str">
         <v>Footer 社群連結呈現不一致</v>
       </c>
-      <c r="I19" s="3" t="str">
+      <c r="I19" s="7" t="str">
         <v>LINE 用 styled button (.btn-line)，Facebook 用純文字圖示連結 (.ic-facebook-before)</v>
       </c>
-      <c r="J19" s="3" t="str">
+      <c r="J19" s="7" t="str">
         <v>統一為相同呈現方式</v>
       </c>
-      <c r="K19" s="3" t="str">
+      <c r="K19" s="7" t="str">
         <v>components/AppFooter.vue</v>
       </c>
-      <c r="L19" s="3" t="str" xml:space="preserve">
+      <c r="L19" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">components/AppFooter.vue_x000d__x000d__x000d_
 assets/style/components/_appFooter.scss_x000d__x000d__x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M19" s="3" t="str">
+      <c r="M19" s="7" t="str">
         <v>兩個社群連結完全不同的 HTML 結構和樣式</v>
       </c>
-      <c r="N19" s="3" t="str">
+      <c r="N19" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O19" s="3" t="str">
+      <c r="O19" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P19" s="3" t="str">
+      <c r="P19" s="7" t="str">
         <v>LINE 與 Facebook 統一為 .btn-social 白底按鈕（含 icon + 深綠字），Facebook 從 .ic-facebook-before 文字連結改為 button 結構並與 LINE 並排。LINE icon 修正為品牌綠 #06C755（Line-Logo.svg fill），Facebook 改用品牌藍 #1877F2（新增 Facebook-Logo-color.svg）。</v>
       </c>
     </row>
@@ -5134,155 +5182,155 @@
       </c>
     </row>
     <row r="24" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A24" s="3">
+      <c r="A24" s="7">
         <v>22</v>
       </c>
-      <c r="B24" s="3" t="str">
+      <c r="B24" s="7" t="str">
         <v>~</v>
       </c>
-      <c r="C24" s="3" t="str">
+      <c r="C24" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D24" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E24" s="3" t="str">
+      <c r="D24" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E24" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F24" s="3" t="str">
+      <c r="F24" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G24" s="3" t="str">
+      <c r="G24" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H24" s="3" t="str">
+      <c r="H24" s="7" t="str">
         <v>缺少 Loading 骨架畫面</v>
       </c>
-      <c r="I24" s="3" t="str">
+      <c r="I24" s="7" t="str">
         <v>API 載入期間無骨架或 loading 指示</v>
       </c>
-      <c r="J24" s="3" t="str">
+      <c r="J24" s="7" t="str">
         <v>新增 skeleton loader</v>
       </c>
-      <c r="K24" s="3" t="str">
+      <c r="K24" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L24" s="3" t="str" xml:space="preserve">
+      <c r="L24" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/news.vue_x000d__x000d__x000d_
 assets/style/components/_appBody.scss</v>
       </c>
-      <c r="M24" s="3" t="str">
+      <c r="M24" s="7" t="str">
         <v>無骨架確認；但有 CSS :empty 空狀態（「目前沒有相關資料哦！」）</v>
       </c>
-      <c r="N24" s="3" t="str">
+      <c r="N24" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O24" s="3" t="str">
+      <c r="O24" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P24" s="3" t="str">
+      <c r="P24" s="7" t="str">
         <v>pages/news.vue 加 isLoading/hasError，分四分支渲染（4 條 skeleton-line 骨架／錯誤+重試／空狀態／正常列表）；LoadNews() 重構並加 .catch()；_animation.scss 加 @keyframes skeletonShimmer 與 .skeleton-line 樣式。</v>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A25" s="3">
+      <c r="A25" s="7">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="str">
+      <c r="B25" s="7" t="str">
         <v>~</v>
       </c>
-      <c r="C25" s="3" t="str">
+      <c r="C25" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D25" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E25" s="3" t="str">
+      <c r="D25" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E25" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F25" s="3" t="str">
+      <c r="F25" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G25" s="3" t="str">
+      <c r="G25" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H25" s="3" t="str">
+      <c r="H25" s="7" t="str">
         <v>桌面版內容截斷無省略提示</v>
       </c>
-      <c r="I25" s="3" t="str">
+      <c r="I25" s="7" t="str">
         <v>桌面版 .item-info 無 text-overflow 或 line-clamp</v>
       </c>
-      <c r="J25" s="3" t="str">
+      <c r="J25" s="7" t="str">
         <v>加入 text-overflow: ellipsis 或 line-clamp</v>
       </c>
-      <c r="K25" s="3" t="str">
+      <c r="K25" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L25" s="3" t="str" xml:space="preserve">
+      <c r="L25" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/news.vue_x000d__x000d__x000d_
 assets/style/components/_appBody.scss_x000d__x000d__x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M25" s="3" t="str">
+      <c r="M25" s="7" t="str">
         <v>桌面無省略確認；手機版已有 textLineClamp(2)</v>
       </c>
-      <c r="N25" s="3" t="str">
+      <c r="N25" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O25" s="3" t="str">
+      <c r="O25" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P25" s="3" t="str">
+      <c r="P25" s="7" t="str">
         <v>pages/news.vue 的 .article-item .item-info 加 line-clamp: 2（桌面）/ line-clamp: 3（手機 ≤1024px），超過行數自動省略結尾。</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="3">
+      <c r="A26" s="7">
         <v>24</v>
       </c>
-      <c r="B26" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C26" s="3" t="str">
+      <c r="B26" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C26" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D26" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E26" s="3" t="str">
+      <c r="D26" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E26" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F26" s="3" t="str">
+      <c r="F26" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G26" s="3" t="str">
+      <c r="G26" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H26" s="3" t="str">
+      <c r="H26" s="7" t="str">
         <v>純圖示連結缺少 aria-label</v>
       </c>
-      <c r="I26" s="3" t="str">
+      <c r="I26" s="7" t="str">
         <v>&lt;i class="ic-arrow-right"&gt; 無 aria-label/title/隱藏文字</v>
       </c>
-      <c r="J26" s="3" t="str">
+      <c r="J26" s="7" t="str">
         <v>加入 aria-label</v>
       </c>
-      <c r="K26" s="3" t="str">
+      <c r="K26" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L26" s="3" t="str">
+      <c r="L26" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="M26" s="3" t="str">
+      <c r="M26" s="7" t="str">
         <v>grep aria-label 全站回傳 0 筆</v>
       </c>
-      <c r="N26" s="3" t="str">
+      <c r="N26" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O26" s="3" t="str">
+      <c r="O26" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P26" s="3" t="str">
+      <c r="P26" s="7" t="str">
         <v>pages/news.vue 的 &lt;i class="ic-arrow-right"&gt; 加上 aria-label="閱讀全文"，符合無障礙語意要求。</v>
       </c>
     </row>
@@ -5338,54 +5386,54 @@
       </c>
     </row>
     <row r="28" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A28" s="3">
+      <c r="A28" s="7">
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C28" s="3" t="str">
+      <c r="B28" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C28" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E28" s="3" t="str">
+      <c r="D28" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E28" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F28" s="3" t="str">
+      <c r="F28" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G28" s="3" t="str">
+      <c r="G28" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H28" s="3" t="str">
+      <c r="H28" s="7" t="str">
         <v>新增「NEW」標籤</v>
       </c>
-      <c r="I28" s="3" t="str">
+      <c r="I28" s="7" t="str">
         <v>新消息無醒目標示</v>
       </c>
-      <c r="J28" s="3" t="str">
+      <c r="J28" s="7" t="str">
         <v>7 天內的新消息加上 NEW badge</v>
       </c>
-      <c r="K28" s="3" t="str">
+      <c r="K28" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L28" s="3" t="str" xml:space="preserve">
+      <c r="L28" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/news.vue_x000d__x000d__x000d_
 assets/style/components/_appBody.scss_x000d__x000d__x000d_
 assets/style/_font.scss</v>
       </c>
-      <c r="M28" s="3" t="str">
+      <c r="M28" s="7" t="str">
         <v>功能確實不存在</v>
       </c>
-      <c r="N28" s="3" t="str">
+      <c r="N28" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O28" s="3" t="str">
+      <c r="O28" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P28" s="3" t="str">
+      <c r="P28" s="7" t="str">
         <v>pages/news.vue 加 isNewItem(releaseTime) helper（7 天內判斷），對應消息右上角顯示橘色 NEW pill 標籤（_appBody.scss .badge-new）。</v>
       </c>
     </row>
@@ -6267,54 +6315,54 @@
       </c>
     </row>
     <row r="46" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A46" s="3">
+      <c r="A46" s="7">
         <v>44</v>
       </c>
-      <c r="B46" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C46" s="3" t="str">
+      <c r="B46" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C46" s="7" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D46" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E46" s="3" t="str">
+      <c r="D46" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E46" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F46" s="3" t="str">
+      <c r="F46" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G46" s="3" t="str">
+      <c r="G46" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H46" s="3" t="str">
+      <c r="H46" s="7" t="str">
         <v>三大核心圖示為靜態 SVG</v>
       </c>
-      <c r="I46" s="3" t="str">
+      <c r="I46" s="7" t="str">
         <v>環境保育/人才培育/社會關懷用靜態 &lt;i class="how-logo"&gt;</v>
       </c>
-      <c r="J46" s="3" t="str">
+      <c r="J46" s="7" t="str">
         <v>加入 SVG 動畫</v>
       </c>
-      <c r="K46" s="3" t="str">
+      <c r="K46" s="7" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L46" s="3" t="str" xml:space="preserve">
+      <c r="L46" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/about.vue_x000d__x000d__x000d_
 assets/style/components/_appBody_about.scss_x000d__x000d__x000d_
 assets/style/_animation.scss</v>
       </c>
-      <c r="M46" s="3" t="str">
+      <c r="M46" s="7" t="str">
         <v>確認無任何動畫 class 或 JS</v>
       </c>
-      <c r="N46" s="3" t="str">
+      <c r="N46" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O46" s="3" t="str">
+      <c r="O46" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P46" s="3" t="str">
+      <c r="P46" s="7" t="str">
         <v>icon SVG 本身仍為靜態，但已包入 Dynamic Island 互動卡片（.how-content）：hover/click toggle 觸發整體 morph 動畫（grid-template-rows 展開、translateY 浮起、background opacity overlay 漸層切換、border 露出青綠光暈）。視覺已不再死板。</v>
       </c>
     </row>
@@ -7040,106 +7088,106 @@
       </c>
     </row>
     <row r="61" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A61" s="3">
+      <c r="A61" s="7">
         <v>59</v>
       </c>
-      <c r="B61" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C61" s="3" t="str">
+      <c r="B61" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C61" s="7" t="str">
         <v>全站微互動</v>
       </c>
-      <c r="D61" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E61" s="3" t="str">
+      <c r="D61" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E61" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F61" s="3" t="str">
+      <c r="F61" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G61" s="3" t="str">
+      <c r="G61" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H61" s="3" t="str">
+      <c r="H61" s="7" t="str">
         <v>卡片 hover 效果升級</v>
       </c>
-      <c r="I61" s="3" t="str">
+      <c r="I61" s="7" t="str">
         <v>目前卡片 hover 效果單調</v>
       </c>
-      <c r="J61" s="3" t="str">
+      <c r="J61" s="7" t="str">
         <v>上浮 4px + 陰影加深</v>
       </c>
-      <c r="K61" s="3" t="str">
+      <c r="K61" s="7" t="str">
         <v>全站</v>
       </c>
-      <c r="L61" s="3" t="str" xml:space="preserve">
+      <c r="L61" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">assets/style/components/_appBody.scss_x000d__x000d__x000d_
 assets/style/components/_appBody_index.scss_x000d__x000d__x000d_
 assets/style/components/_appBodyChild_ifare.scss</v>
       </c>
-      <c r="M61" s="3" t="str">
+      <c r="M61" s="7" t="str">
         <v>功能確實不存在（待實測確認現有 hover）</v>
       </c>
-      <c r="N61" s="3" t="str">
+      <c r="N61" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O61" s="3" t="str">
+      <c r="O61" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P61" s="3" t="str">
+      <c r="P61" s="7" t="str">
         <v>_main.scss 為 .result-item / .article-item / .agency-item 加 hover translateY(-3px) + box-shadow，active translateY(-1px) 回彈。純 GPU 屬性，不觸發 layout 重繪。</v>
       </c>
     </row>
     <row r="62" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A62" s="3">
+      <c r="A62" s="5">
         <v>60</v>
       </c>
-      <c r="B62" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C62" s="3" t="str">
+      <c r="B62" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C62" s="5" t="str">
         <v>全站微互動</v>
       </c>
-      <c r="D62" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E62" s="3" t="str">
+      <c r="D62" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E62" s="5" t="str">
         <v>提升</v>
       </c>
-      <c r="F62" s="3" t="str">
+      <c r="F62" s="5" t="str">
         <v>視覺</v>
       </c>
-      <c r="G62" s="3" t="str">
+      <c r="G62" s="5" t="str">
         <v>低</v>
       </c>
-      <c r="H62" s="3" t="str">
+      <c r="H62" s="5" t="str">
         <v>CTA 按鈕互動效果</v>
       </c>
-      <c r="I62" s="3" t="str">
+      <c r="I62" s="5" t="str">
         <v>按鈕缺乏觸覺回饋</v>
       </c>
-      <c r="J62" s="3" t="str">
+      <c r="J62" s="5" t="str">
         <v>hover 按壓回彈 + 點擊漣漪效果</v>
       </c>
-      <c r="K62" s="3" t="str">
+      <c r="K62" s="5" t="str">
         <v>全站</v>
       </c>
-      <c r="L62" s="3" t="str" xml:space="preserve">
+      <c r="L62" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">assets/style/components/_button.scss_x000d__x000d__x000d_
 assets/style/_font.scss_x000d__x000d__x000d_
 assets/style/rwd/_rwd_button.scss</v>
       </c>
-      <c r="M62" s="3" t="str">
+      <c r="M62" s="5" t="str">
         <v>功能確實不存在</v>
       </c>
-      <c r="N62" s="3" t="str">
+      <c r="N62" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O62" s="3" t="str">
+      <c r="O62" s="5" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P62" s="3" t="str">
+      <c r="P62" s="5" t="str">
         <v>_main.scss 為 .btn-filter / .btn-tag / .btn-retry 加 hover translateY(-1px) + active scale(0.97) 按壓回彈。原訴求「點擊漣漪效果」尚未做。</v>
       </c>
     </row>
@@ -7655,55 +7703,55 @@
       </c>
     </row>
     <row r="73" ht="45" customHeight="1" xml:space="preserve">
-      <c r="A73" s="3">
+      <c r="A73" s="5">
         <v>71</v>
       </c>
-      <c r="B73" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C73" s="3" t="str">
+      <c r="B73" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C73" s="5" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D73" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E73" s="3" t="str">
+      <c r="D73" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E73" s="5" t="str">
         <v>修復</v>
       </c>
-      <c r="F73" s="3" t="str">
+      <c r="F73" s="5" t="str">
         <v>RWD</v>
       </c>
-      <c r="G73" s="3" t="str">
+      <c r="G73" s="5" t="str">
         <v>高</v>
       </c>
-      <c r="H73" s="3" t="str">
+      <c r="H73" s="5" t="str">
         <v>多處觸控目標小於 44x44px</v>
       </c>
-      <c r="I73" s="3" t="str">
+      <c r="I73" s="5" t="str">
         <v>分頁按鈕 30x30px、.btn-reset height:32px、.btn-advance height:40px</v>
       </c>
-      <c r="J73" s="3" t="str">
+      <c r="J73" s="5" t="str">
         <v>確保所有可點擊元素最小 44x44px</v>
       </c>
-      <c r="K73" s="3" t="str">
+      <c r="K73" s="5" t="str">
         <v>全站</v>
       </c>
-      <c r="L73" s="3" t="str" xml:space="preserve">
+      <c r="L73" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">assets/style/components/_compPage.scss_x000d__x000d__x000d_
 assets/style/components/_button.scss_x000d__x000d__x000d_
 assets/style/components/_compSelect.scss_x000d__x000d__x000d_
 assets/style/rwd/_rwd_compPage.scss</v>
       </c>
-      <c r="M73" s="3" t="str">
+      <c r="M73" s="5" t="str">
         <v>確認多處尺寸低於 44px 標準</v>
       </c>
-      <c r="N73" s="3" t="str">
+      <c r="N73" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O73" s="3" t="str">
+      <c r="O73" s="5" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P73" s="3" t="str">
+      <c r="P73" s="5" t="str">
         <v>footer .btn-social 高度從 40px 提升到 44px（LINE / Facebook 兩按鈕符合 iOS HIG 觸控標準）。CompPage 分頁箭頭、btn-reset、btn-advance、CompSelect 等其他元件尚未套用 44px 標準。</v>
       </c>
     </row>
@@ -8100,52 +8148,52 @@
       </c>
     </row>
     <row r="82" ht="45" customHeight="1">
-      <c r="A82" s="3">
+      <c r="A82" s="5">
         <v>80</v>
       </c>
-      <c r="B82" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C82" s="3" t="str">
+      <c r="B82" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C82" s="5" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D82" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E82" s="3" t="str">
+      <c r="D82" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E82" s="5" t="str">
         <v>修復</v>
       </c>
-      <c r="F82" s="3" t="str">
+      <c r="F82" s="5" t="str">
         <v>互動</v>
       </c>
-      <c r="G82" s="3" t="str">
+      <c r="G82" s="5" t="str">
         <v>高</v>
       </c>
-      <c r="H82" s="3" t="str">
+      <c r="H82" s="5" t="str">
         <v>缺少載入失敗與重試機制</v>
       </c>
-      <c r="I82" s="3" t="str">
+      <c r="I82" s="5" t="str">
         <v>目前清單有 loading / skeleton / toast，但尚未明確區分 API 載入失敗狀態與重試機制。</v>
       </c>
-      <c r="J82" s="3" t="str">
+      <c r="J82" s="5" t="str">
         <v>建立統一錯誤狀態元件，針對 API 失敗提供錯誤訊息、retry 按鈕，並區分空資料與載入失敗。</v>
       </c>
-      <c r="K82" s="3" t="str">
+      <c r="K82" s="5" t="str">
         <v>全站</v>
       </c>
-      <c r="L82" s="3" t="str">
+      <c r="L82" s="5" t="str">
         <v>pages/news.vue pages/articles.vue pages/collaborator.vue pages/ifare/result.vue layouts/default.vue components/</v>
       </c>
-      <c r="M82" s="3" t="str">
+      <c r="M82" s="5" t="str">
         <v>現有清單多著重 loading 與空狀態，未明列 error state。</v>
       </c>
-      <c r="N82" s="3" t="str">
+      <c r="N82" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O82" s="3" t="str">
+      <c r="O82" s="5" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P82" s="3" t="str">
+      <c r="P82" s="5" t="str">
         <v>pages/news.vue 已實作 hasError + .btn-retry 按鈕模式（搭配 _animation.scss .part-error 樣式）。articles.vue / collaborator.vue / ifare/result.vue 三頁尚未套用同一錯誤狀態元件。</v>
       </c>
     </row>
@@ -8443,1173 +8491,1173 @@
       </c>
     </row>
     <row r="90" ht="100.8" customHeight="1" xml:space="preserve">
-      <c r="A90" s="3">
+      <c r="A90" s="7">
         <v>88</v>
       </c>
-      <c r="B90" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C90" s="3" t="str">
+      <c r="B90" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C90" s="7" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D90" s="3" t="str">
+      <c r="D90" s="7" t="str">
         <v>搜尋介面</v>
       </c>
-      <c r="E90" s="3" t="str">
+      <c r="E90" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F90" s="3" t="str">
+      <c r="F90" s="7" t="str">
         <v>黏著</v>
       </c>
-      <c r="G90" s="3" t="str">
+      <c r="G90" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H90" s="3" t="str">
+      <c r="H90" s="7" t="str">
         <v>新增關鍵字搜尋輸入欄</v>
       </c>
-      <c r="I90" s="3" t="str">
+      <c r="I90" s="7" t="str">
         <v>原本搜尋只能用三個下拉選單（政策類別、受助對象、地區），缺少自由文字搜尋入口</v>
       </c>
-      <c r="J90" s="3" t="str">
+      <c r="J90" s="7" t="str">
         <v>ifare 與結果頁各加 &lt;input.input-keyword&gt;（含 Enter 快捷鍵），搜尋條件擴增 keyword 參數，後端 LIKE 查詢</v>
       </c>
-      <c r="K90" s="3" t="str">
+      <c r="K90" s="7" t="str">
         <v>pages/ifare.vue pages/ifare/result.vue</v>
       </c>
-      <c r="L90" s="3" t="str" xml:space="preserve">
+      <c r="L90" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">pages/ifare.vue_x000d__x000d__x000d_
 pages/ifare/result.vue_x000d__x000d__x000d_
 assets/style/components/_appBody_ifare.scss_x000d__x000d__x000d_
 assets/style/components/_appBodyChild_ifare.scss</v>
       </c>
-      <c r="M90" s="3" t="str">
+      <c r="M90" s="7" t="str">
         <v>改版補登；後端 IFare_API.Application/Fare/Policy/* 已加 Keyword filter</v>
       </c>
-      <c r="N90" s="3" t="str">
+      <c r="N90" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O90" s="3" t="str">
+      <c r="O90" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P90" s="3" t="str">
+      <c r="P90" s="7" t="str">
         <v>改版補登；前端 Search() 已帶 keyword 參數，API 傳 Keyword 欄位</v>
       </c>
     </row>
     <row r="91" ht="57.6" customHeight="1">
-      <c r="A91" s="3">
+      <c r="A91" s="7">
         <v>89</v>
       </c>
-      <c r="B91" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C91" s="3" t="str">
+      <c r="B91" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C91" s="7" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D91" s="3" t="str">
+      <c r="D91" s="7" t="str">
         <v>查詢結果</v>
       </c>
-      <c r="E91" s="3" t="str">
+      <c r="E91" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F91" s="3" t="str">
+      <c r="F91" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G91" s="3" t="str">
+      <c r="G91" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H91" s="3" t="str">
+      <c r="H91" s="7" t="str">
         <v>結果頁未支援 URL query 初始化</v>
       </c>
-      <c r="I91" s="3" t="str">
+      <c r="I91" s="7" t="str">
         <v>結果頁從 ifare 跳轉過來時若重整或從外部進入，搜尋條件無法保留</v>
       </c>
-      <c r="J91" s="3" t="str">
+      <c r="J91" s="7" t="str">
         <v>解析 route.query 初始化各 ref（policy / recipient / area / keyword），支援深度連結與重整保留條件</v>
       </c>
-      <c r="K91" s="3" t="str">
+      <c r="K91" s="7" t="str">
         <v>pages/ifare/result.vue</v>
       </c>
-      <c r="L91" s="3" t="str">
+      <c r="L91" s="7" t="str">
         <v>pages/ifare/result.vue</v>
       </c>
-      <c r="M91" s="3" t="str">
+      <c r="M91" s="7" t="str">
         <v>改版補登；搭配 #88 關鍵字欄位一起實作</v>
       </c>
-      <c r="N91" s="3" t="str">
+      <c r="N91" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O91" s="3" t="str">
+      <c r="O91" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P91" s="3" t="str">
+      <c r="P91" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="92" ht="57.6" customHeight="1">
-      <c r="A92" s="3">
+      <c r="A92" s="7">
         <v>90</v>
       </c>
-      <c r="B92" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C92" s="3" t="str">
+      <c r="B92" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C92" s="7" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D92" s="3" t="str">
+      <c r="D92" s="7" t="str">
         <v>搜尋介面</v>
       </c>
-      <c r="E92" s="3" t="str">
+      <c r="E92" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F92" s="3" t="str">
+      <c r="F92" s="7" t="str">
         <v>RWD</v>
       </c>
-      <c r="G92" s="3" t="str">
+      <c r="G92" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H92" s="3" t="str">
+      <c r="H92" s="7" t="str">
         <v>搜尋按鈕區手機版橫排擠壓</v>
       </c>
-      <c r="I92" s="3" t="str">
+      <c r="I92" s="7" t="str">
         <v>.item-bottom 原為橫排，手機版按鈕和提示文字擠在一起</v>
       </c>
-      <c r="J92" s="3" t="str">
+      <c r="J92" s="7" t="str">
         <v>_appBody_ifare.scss .item-bottom 改 flex-direction: column + gap + 居中，並加 .filter-hint 樣式</v>
       </c>
-      <c r="K92" s="3" t="str">
+      <c r="K92" s="7" t="str">
         <v>pages/ifare.vue</v>
       </c>
-      <c r="L92" s="3" t="str">
+      <c r="L92" s="7" t="str">
         <v>iFare_Frontend/assets/style/components/_appBody_ifare.scss</v>
       </c>
-      <c r="M92" s="3" t="str">
+      <c r="M92" s="7" t="str">
         <v>改版補登；搭配 #1 disabled 移除後新增的提示文字調整版面</v>
       </c>
-      <c r="N92" s="3" t="str">
+      <c r="N92" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O92" s="3" t="str">
+      <c r="O92" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P92" s="3" t="str">
+      <c r="P92" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="93" ht="86.40000000000002" customHeight="1" xml:space="preserve">
-      <c r="A93" s="3">
+      <c r="A93" s="7">
         <v>91</v>
       </c>
-      <c r="B93" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C93" s="3" t="str">
+      <c r="B93" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C93" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D93" s="3" t="str">
+      <c r="D93" s="7" t="str">
         <v>AppFooter</v>
       </c>
-      <c r="E93" s="3" t="str">
+      <c r="E93" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F93" s="3" t="str">
+      <c r="F93" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G93" s="3" t="str">
+      <c r="G93" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H93" s="3" t="str">
+      <c r="H93" s="7" t="str">
         <v>Footer 聯絡資訊缺 icon</v>
       </c>
-      <c r="I93" s="3" t="str">
+      <c r="I93" s="7" t="str">
         <v>footer 4 個 label（聯絡電話 / 聯絡信箱 / 地址 / 服務時間）僅有純文字，缺乏視覺辨識</v>
       </c>
-      <c r="J93" s="3" t="str">
+      <c r="J93" s="7" t="str">
         <v>4 個 label 前各加對應 icon（Tel / Mail / Address / Clock），與站內既有 icon 風格一致</v>
       </c>
-      <c r="K93" s="3" t="str">
+      <c r="K93" s="7" t="str">
         <v>components/AppFooter.vue</v>
       </c>
-      <c r="L93" s="3" t="str" xml:space="preserve">
+      <c r="L93" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/AppFooter.vue_x000d__x000d__x000d_
 assets/style/components/_appFooter.scss_x000d__x000d__x000d_
 assets/style/_font.scss_x000d__x000d__x000d_
 assets/img/Mail.svg (新增)_x000d__x000d__x000d_
 assets/img/Clock.svg (新增)</v>
       </c>
-      <c r="M93" s="3" t="str">
+      <c r="M93" s="7" t="str">
         <v>改版補登；新增 Mail.svg + Clock.svg 用 mask-image 著色為 rgba(white,.7)，沿用既有 Tel.svg / Location.svg。原 ::before content 的 CSS-only label 改為 HTML &lt;span class="footer-info-label"&gt; 結構</v>
       </c>
-      <c r="N93" s="3" t="str">
+      <c r="N93" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O93" s="3" t="str">
+      <c r="O93" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P93" s="3" t="str">
+      <c r="P93" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="94" ht="273.6" customHeight="1" xml:space="preserve">
-      <c r="A94" s="3">
+      <c r="A94" s="7">
         <v>92</v>
       </c>
-      <c r="B94" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C94" s="3" t="str">
+      <c r="B94" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C94" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D94" s="3" t="str">
+      <c r="D94" s="7" t="str">
         <v>AppFooter</v>
       </c>
-      <c r="E94" s="3" t="str">
+      <c r="E94" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F94" s="3" t="str">
+      <c r="F94" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G94" s="3" t="str">
+      <c r="G94" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H94" s="3" t="str">
+      <c r="H94" s="7" t="str">
         <v>社群連結 LINE / Facebook 分散兩處</v>
       </c>
-      <c r="I94" s="3" t="str">
+      <c r="I94" s="7" t="str">
         <v>LINE 在「進一步瞭解更多」CTA 區塊內，Facebook 在獨立 .part-middle 區塊；兩者都是社群媒體應該放一起</v>
       </c>
-      <c r="J94" s="3" t="str">
+      <c r="J94" s="7" t="str">
         <v>把 Facebook 從 .part-middle 移到 .card-more 內 .card-more-socials div 與 LINE 並排，整合為單一社群區塊</v>
       </c>
-      <c r="K94" s="3" t="str">
+      <c r="K94" s="7" t="str">
         <v>components/AppFooter.vue</v>
       </c>
-      <c r="L94" s="3" t="str" xml:space="preserve">
+      <c r="L94" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/AppFooter.vue_x000d__x000d__x000d_
 assets/style/components/_appFooter.scss_x000d__x000d__x000d_
 assets/style/rwd/_rwd_appFooter.scss</v>
       </c>
-      <c r="M94" s="3" t="str">
+      <c r="M94" s="7" t="str">
         <v>改版補登；移除原 .part-middle 與 .link-track 樣式</v>
       </c>
-      <c r="N94" s="3" t="str">
+      <c r="N94" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O94" s="3" t="str">
+      <c r="O94" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P94" s="3" t="str">
+      <c r="P94" s="7" t="str">
         <v>改版補登；同步修桌面 1025-1280px overflow（加 FB 後 .card-more 內容寬度 ~1300px 會爆）：.card-more 加 flex-wrap: wrap + max-width: calc(100% - 64px)；.info-more 加 max-width: 480px 讓長文字桌面換 2 行</v>
       </c>
     </row>
     <row r="95" ht="129.6" customHeight="1" xml:space="preserve">
-      <c r="A95" s="3">
+      <c r="A95" s="7">
         <v>93</v>
       </c>
-      <c r="B95" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C95" s="3" t="str">
+      <c r="B95" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C95" s="7" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D95" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E95" s="3" t="str">
+      <c r="D95" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E95" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F95" s="3" t="str">
+      <c r="F95" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G95" s="3" t="str">
+      <c r="G95" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H95" s="3" t="str">
+      <c r="H95" s="7" t="str">
         <v>About 三大核心介紹缺乏互動性</v>
       </c>
-      <c r="I95" s="3" t="str">
+      <c r="I95" s="7" t="str">
         <v>環境保育/人才培育/社會關懷三張卡片原為靜態圖文，使用者掃過無視覺反應，缺乏吸引點擊探索的動機</v>
       </c>
-      <c r="J95" s="3" t="str">
+      <c r="J95" s="7" t="str">
         <v>改造為 iOS Dynamic Island 風格 morph 卡片：暖象牙白漸層底 + 圓角 28px + 預設只露 icon+標題 → hover/click toggle 平滑展開內文（grid-template-rows trick）+ translateY 浮起 + 邊框露出青綠光暈</v>
       </c>
-      <c r="K95" s="3" t="str">
+      <c r="K95" s="7" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L95" s="3" t="str" xml:space="preserve">
+      <c r="L95" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/about.vue_x000d__x000d__x000d_
 assets/style/components/_appBody_about.scss_x000d__x000d__x000d_
 assets/style/rwd/_rwd_about.scss</v>
       </c>
-      <c r="M95" s="3" t="str">
+      <c r="M95" s="7" t="str">
         <v>改版補登；HTML 重組（icon+title 合進 .how-top、info 包 .how-info-wrap）；script 加 activeHow ref + toggleHow handler；keyboard a11y (Enter/Space) 與 tabindex；GPU 優化（will-change + ::before opacity overlay 取代 gradient transition）；Apple spring easing cubic-bezier(0.32, 0.72, 0, 1)</v>
       </c>
-      <c r="N95" s="3" t="str">
+      <c r="N95" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O95" s="3" t="str">
+      <c r="O95" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P95" s="3" t="str">
+      <c r="P95" s="7" t="str">
         <v>改版補登；對應 #44 三大核心圖示靜態問題已連動修正</v>
       </c>
     </row>
     <row r="96" ht="100.8" customHeight="1">
-      <c r="A96" s="3">
+      <c r="A96" s="7">
         <v>94</v>
       </c>
-      <c r="B96" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C96" s="3" t="str">
+      <c r="B96" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C96" s="7" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D96" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E96" s="3" t="str">
+      <c r="D96" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E96" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F96" s="3" t="str">
+      <c r="F96" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G96" s="3" t="str">
+      <c r="G96" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H96" s="3" t="str">
+      <c r="H96" s="7" t="str">
         <v>About 成員照片缺 hover 互動</v>
       </c>
-      <c r="I96" s="3" t="str">
+      <c r="I96" s="7" t="str">
         <v>陳進財/鄔筠軒/顏杏蓉三位成員區塊原無 hover 反饋，掃過時視覺無變化</v>
       </c>
-      <c r="J96" s="3" t="str">
+      <c r="J96" s="7" t="str">
         <v>陳進財/鄔筠軒整組 hover：照片 scale(1.06) + 白框 scale(1.03) + box-shadow 加深 + 橘色標牌 translateY(-4px)；顏杏蓉（無照片）標牌 hover translateY(-4px) + scale(1.04)</v>
       </c>
-      <c r="K96" s="3" t="str">
+      <c r="K96" s="7" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L96" s="3" t="str">
+      <c r="L96" s="7" t="str">
         <v>iFare_Frontend/assets/style/components/_appBody_about.scss</v>
       </c>
-      <c r="M96" s="3" t="str">
+      <c r="M96" s="7" t="str">
         <v>改版補登；同套 cubic-bezier(0.32, 0.72, 0, 1) easing；will-change: transform 給 .member-photo 預先建 GPU layer</v>
       </c>
-      <c r="N96" s="3" t="str">
+      <c r="N96" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O96" s="3" t="str">
+      <c r="O96" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P96" s="3" t="str">
+      <c r="P96" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="97" ht="57.6" customHeight="1">
-      <c r="A97" s="3">
+      <c r="A97" s="7">
         <v>95</v>
       </c>
-      <c r="B97" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C97" s="3" t="str">
+      <c r="B97" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C97" s="7" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D97" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E97" s="3" t="str">
+      <c r="D97" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E97" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F97" s="3" t="str">
+      <c r="F97" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G97" s="3" t="str">
+      <c r="G97" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H97" s="3" t="str">
+      <c r="H97" s="7" t="str">
         <v>About 底部 CTA 連結缺 hover micro-animation</v>
       </c>
-      <c r="I97" s="3" t="str">
+      <c r="I97" s="7" t="str">
         <v>「前往 i-Fare」與「查看最新消息」兩個 advance-link 原為靜態，hover 無互動反饋，無法強化「點我前進」訊號</v>
       </c>
-      <c r="J97" s="3" t="str">
+      <c r="J97" s="7" t="str">
         <v>連結 hover 時 translateY(-2px) 上浮，箭頭 icon translateX(6px) 向右滑出，引導視線前進</v>
       </c>
-      <c r="K97" s="3" t="str">
+      <c r="K97" s="7" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L97" s="3" t="str">
+      <c r="L97" s="7" t="str">
         <v>iFare_Frontend/assets/style/components/_appBody_about.scss</v>
       </c>
-      <c r="M97" s="3" t="str">
+      <c r="M97" s="7" t="str">
         <v>改版補登；統一 cubic-bezier(0.32, 0.72, 0, 1) easing 0.22s</v>
       </c>
-      <c r="N97" s="3" t="str">
+      <c r="N97" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O97" s="3" t="str">
+      <c r="O97" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P97" s="3" t="str">
+      <c r="P97" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="98" ht="129.6" customHeight="1" xml:space="preserve">
-      <c r="A98" s="3">
+      <c r="A98" s="7">
         <v>96</v>
       </c>
-      <c r="B98" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C98" s="3" t="str">
+      <c r="B98" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C98" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D98" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E98" s="3" t="str">
+      <c r="D98" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E98" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F98" s="3" t="str">
+      <c r="F98" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G98" s="3" t="str">
+      <c r="G98" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H98" s="3" t="str">
+      <c r="H98" s="7" t="str">
         <v>News 列表呈現升級為浮起卡片 + 入場動畫 + 日期 pill</v>
       </c>
-      <c r="I98" s="3" t="str">
+      <c r="I98" s="7" t="str">
         <v>原本最新消息為「底線分隔的清單列」，hover 只是淡白底 + 箭頭轉橘，視覺扁平、缺乏互動感、日期不醒目、長內文無截斷</v>
       </c>
-      <c r="J98" s="3" t="str">
+      <c r="J98" s="7" t="str">
         <v>列表整體升級：圓角 16px 浮起卡片（white .7 + shadow）+ stagger fade-up 入場動畫（@for 1~12 each +50ms）+ 日期變橘色 pill 標籤（border + 半透明橘底）+ hover translateY(-3px) + 背景變實白 + 箭頭橘色滑右 6px</v>
       </c>
-      <c r="K98" s="3" t="str">
+      <c r="K98" s="7" t="str">
         <v>pages/news.vue</v>
       </c>
-      <c r="L98" s="3" t="str" xml:space="preserve">
+      <c r="L98" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/news.vue_x000d__x000d__x000d_
 assets/style/components/_appBody.scss_x000d__x000d__x000d_
 assets/style/_animation.scss_x000d__x000d__x000d_
 assets/style/rwd/_rwd.scss</v>
       </c>
-      <c r="M98" s="3" t="str">
+      <c r="M98" s="7" t="str">
         <v>改版補登；@keyframes newsItemEnter 放 _animation.scss；統一 cubic-bezier(0.32, 0.72, 0, 1) easing；配色全用既有 token 沒引入新色</v>
       </c>
-      <c r="N98" s="3" t="str">
+      <c r="N98" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O98" s="3" t="str">
+      <c r="O98" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P98" s="3" t="str">
+      <c r="P98" s="7" t="str">
         <v>改版補登；同次改動連帶解決 #23 (line-clamp 2)、#24 (aria-label)、#26 (NEW badge)</v>
       </c>
     </row>
     <row r="99" ht="72" customHeight="1" xml:space="preserve">
-      <c r="A99" s="3">
+      <c r="A99" s="7">
         <v>97</v>
       </c>
-      <c r="B99" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C99" s="3" t="str">
+      <c r="B99" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C99" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D99" s="3" t="str">
+      <c r="D99" s="7" t="str">
         <v>AppFooter / AppHeader</v>
       </c>
-      <c r="E99" s="3" t="str">
+      <c r="E99" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F99" s="3" t="str">
+      <c r="F99" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G99" s="3" t="str">
+      <c r="G99" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H99" s="3" t="str">
+      <c r="H99" s="7" t="str">
         <v>社群外連結未開新分頁，可能丟失當前頁狀態</v>
       </c>
-      <c r="I99" s="3" t="str">
+      <c r="I99" s="7" t="str">
         <v>AppFooter LINE/Facebook 與 AppHeader 手機版社群 icon 連結原為一般 &lt;a href&gt;，點擊會在當前分頁導向，使用者離開站內後返回成本高</v>
       </c>
-      <c r="J99" s="3" t="str">
+      <c r="J99" s="7" t="str">
         <v>4 個社群連結都加 target="_blank" + rel="noopener noreferrer"：開新分頁、避免反向 tabnabbing、不洩漏 referrer</v>
       </c>
-      <c r="K99" s="3" t="str">
+      <c r="K99" s="7" t="str">
         <v>components/AppFooter.vue components/AppHeader.vue</v>
       </c>
-      <c r="L99" s="3" t="str" xml:space="preserve">
+      <c r="L99" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/AppFooter.vue_x000d__x000d__x000d_
 iFare_Frontend/components/AppHeader.vue</v>
       </c>
-      <c r="M99" s="3" t="str">
+      <c r="M99" s="7" t="str">
         <v>改版補登；rel="noopener" 是 W3C 安全建議</v>
       </c>
-      <c r="N99" s="3" t="str">
+      <c r="N99" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O99" s="3" t="str">
+      <c r="O99" s="7" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="P99" s="3" t="str">
+      <c r="P99" s="7" t="str">
         <v>改版補登</v>
       </c>
     </row>
     <row r="100" ht="100.8" customHeight="1">
-      <c r="A100" s="3">
+      <c r="A100" s="7">
         <v>98</v>
       </c>
-      <c r="B100" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C100" s="3" t="str">
+      <c r="B100" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C100" s="7" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="D100" s="3" t="str">
+      <c r="D100" s="7" t="str">
         <v>三大核心介紹</v>
       </c>
-      <c r="E100" s="3" t="str">
+      <c r="E100" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F100" s="3" t="str">
+      <c r="F100" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G100" s="3" t="str">
+      <c r="G100" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H100" s="3" t="str">
+      <c r="H100" s="7" t="str">
         <v>About 第一張卡 hover 完全無反應 (Round 3 副作用)</v>
       </c>
-      <c r="I100" s="3" t="str">
+      <c r="I100" s="7" t="str">
         <v>cf47cfa Round 3 加的 .section-about-member::before 視覺裝飾 (z-index:48 + 1497x1497px 圓形 + top:-300px/left:-750px) 蓋住上方 about-how 區左半邊，攔截「環境保育」第一張 morph 卡的所有 hover/click events。第二、三張位置在中右側未被覆蓋，因此正常運作。</v>
       </c>
-      <c r="J100" s="3" t="str">
+      <c r="J100" s="7" t="str">
         <v>裝飾性 ::before 加 pointer-events: none 讓 mouse events 穿透到下層的 .how-content</v>
       </c>
-      <c r="K100" s="3" t="str">
+      <c r="K100" s="7" t="str">
         <v>pages/about.vue</v>
       </c>
-      <c r="L100" s="3" t="str">
+      <c r="L100" s="7" t="str">
         <v>iFare_Frontend/assets/style/components/_appBody_about.scss</v>
       </c>
-      <c r="M100" s="3" t="str">
+      <c r="M100" s="7" t="str">
         <v>修復 cf47cfa 副作用；不影響原視覺 (radial-gradient 橘色光暈仍可見)</v>
       </c>
-      <c r="N100" s="3" t="str">
+      <c r="N100" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O100" s="3" t="str">
+      <c r="O100" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P100" s="3" t="str">
+      <c r="P100" s="7" t="str">
         <v>純 1 行 CSS 修法 (.section-about-member::before pointer-events: none)</v>
       </c>
     </row>
     <row r="101" ht="100.8" customHeight="1">
-      <c r="A101" s="3">
+      <c r="A101" s="7">
         <v>99</v>
       </c>
-      <c r="B101" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C101" s="3" t="str">
+      <c r="B101" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C101" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D101" s="3" t="str">
+      <c r="D101" s="7" t="str">
         <v>AppFooter</v>
       </c>
-      <c r="E101" s="3" t="str">
+      <c r="E101" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F101" s="3" t="str">
+      <c r="F101" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G101" s="3" t="str">
+      <c r="G101" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H101" s="3" t="str">
+      <c r="H101" s="7" t="str">
         <v>Footer 聯絡資訊 label 文字重複 (新舊 CSS 共存 bug)</v>
       </c>
-      <c r="I101" s="3" t="str">
+      <c r="I101" s="7" t="str">
         <v>5dfbf91/cf47cfa 把 AppFooter.vue 改用顯式 &lt;span class="footer-info-label"&gt; 顯示 label，但舊的 _font.scss `.footer-info-items [name="tel"]::before { content: "聯絡電話" }` 等 4 條規則沒清掉，造成「聯絡電話 📞 聯絡電話 (02)2797-8383」這種重複顯示</v>
       </c>
-      <c r="J101" s="3" t="str">
+      <c r="J101" s="7" t="str">
         <v>移除 _font.scss 4 個 ::before content 規則 (tel/mail/address/datetime) 與通用 [name]::before 樣式</v>
       </c>
-      <c r="K101" s="3" t="str">
+      <c r="K101" s="7" t="str">
         <v>assets/style/_font.scss</v>
       </c>
-      <c r="L101" s="3" t="str">
+      <c r="L101" s="7" t="str">
         <v>iFare_Frontend/assets/style/_font.scss</v>
       </c>
-      <c r="M101" s="3" t="str">
+      <c r="M101" s="7" t="str">
         <v>回歸測試 OK；保留 [name="tel"] font-family/color 與 [name="datetime"] span:nth-child Roboto 樣式</v>
       </c>
-      <c r="N101" s="3" t="str">
+      <c r="N101" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O101" s="3" t="str">
+      <c r="O101" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P101" s="3" t="str">
+      <c r="P101" s="7" t="str">
         <v>5dfbf91 整理時的 leftover</v>
       </c>
     </row>
     <row r="102" ht="144" customHeight="1">
-      <c r="A102" s="3">
+      <c r="A102" s="7">
         <v>100</v>
       </c>
-      <c r="B102" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C102" s="3" t="str">
+      <c r="B102" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C102" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D102" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E102" s="3" t="str">
+      <c r="D102" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E102" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F102" s="3" t="str">
+      <c r="F102" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G102" s="3" t="str">
+      <c r="G102" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H102" s="3" t="str">
+      <c r="H102" s="7" t="str">
         <v>缺乏全站一致的 hover 靈動回饋</v>
       </c>
-      <c r="I102" s="3" t="str">
+      <c r="I102" s="7" t="str">
         <v>既有 hover 散落在 .relation-item / .article-item / .card-* 等個別元件，nav 連結、Footer 按鈕、btn-icon 等沒有統一浮起回饋；使用者「鼠標移到哪都該有靈動」需求未滿足</v>
       </c>
-      <c r="J102" s="3" t="str">
+      <c r="J102" s="7" t="str">
         <v>_main.scss 加 .hover-lift utility class (Apple spring 0.22s + translateY -2px) + 自動套用到 .app-header nav / .app-footer .btn / .app-footer a / .btn-social / .btn-icon。既有自訂 hover (about morph 卡、news 浮起卡) 不受影響</v>
       </c>
-      <c r="K102" s="3" t="str">
+      <c r="K102" s="7" t="str">
         <v>assets/style/_main.scss</v>
       </c>
-      <c r="L102" s="3" t="str">
+      <c r="L102" s="7" t="str">
         <v>iFare_Frontend/assets/style/_main.scss</v>
       </c>
-      <c r="M102" s="3" t="str">
+      <c r="M102" s="7" t="str">
         <v>cubic-bezier(0.32, 0.72, 0, 1) 與 about morph 卡同套 easing</v>
       </c>
-      <c r="N102" s="3" t="str">
+      <c r="N102" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O102" s="3" t="str">
+      <c r="O102" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P102" s="3" t="str">
+      <c r="P102" s="7" t="str">
         <v>對應 #62 (.btn-filter/.btn-tag hover) 不重疊 — Round 4 涵蓋的是 nav/footer 類；ifare 搜尋按鈕的 ripple 仍待補</v>
       </c>
     </row>
     <row r="103" ht="115.2" customHeight="1" xml:space="preserve">
-      <c r="A103" s="3">
+      <c r="A103" s="7">
         <v>101</v>
       </c>
-      <c r="B103" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C103" s="3" t="str">
+      <c r="B103" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C103" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D103" s="3" t="str">
+      <c r="D103" s="7" t="str">
         <v>AppHeader</v>
       </c>
-      <c r="E103" s="3" t="str">
+      <c r="E103" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F103" s="3" t="str">
+      <c r="F103" s="7" t="str">
         <v>內容</v>
       </c>
-      <c r="G103" s="3" t="str">
+      <c r="G103" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H103" s="3" t="str">
+      <c r="H103" s="7" t="str">
         <v>缺少「未來規劃」頁面入口</v>
       </c>
-      <c r="I103" s="3" t="str">
+      <c r="I103" s="7" t="str">
         <v>主管要求增加「未來規劃」展示基金會願景，nav 應有對應入口</v>
       </c>
-      <c r="J103" s="3" t="str">
+      <c r="J103" s="7" t="str">
         <v>AppHeader 桌面 nav 在 公益夥伴 與 i-Fare 之間插入「未來規劃」連結；行動 nav 加在最後 (與既有 i-Fare/公益夥伴 mobile 順序一致)；新增 pages/future.vue 標題 + FUTURE shadow + 「內容建置中，敬請期待」佔位</v>
       </c>
-      <c r="K103" s="3" t="str">
+      <c r="K103" s="7" t="str">
         <v>components/AppHeader.vue + pages/future.vue (新)</v>
       </c>
-      <c r="L103" s="3" t="str" xml:space="preserve">
+      <c r="L103" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/AppHeader.vue_x000d__x000d__x000d_
 iFare_Frontend/pages/future.vue (新)</v>
       </c>
-      <c r="M103" s="3" t="str">
+      <c r="M103" s="7" t="str">
         <v>route /future 已 wire；之後接 CMS 內容由 admin 管理</v>
       </c>
-      <c r="N103" s="3" t="str">
+      <c r="N103" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O103" s="3" t="str">
+      <c r="O103" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P103" s="3" t="str">
+      <c r="P103" s="7" t="str">
         <v>頁面為佔位，等內容/設計稿確認後再填內</v>
       </c>
     </row>
     <row r="104" ht="144" customHeight="1" xml:space="preserve">
-      <c r="A104" s="3">
+      <c r="A104" s="5">
         <v>102</v>
       </c>
-      <c r="B104" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C104" s="3" t="str">
+      <c r="B104" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C104" s="5" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D104" s="3" t="str">
+      <c r="D104" s="5" t="str">
         <v>文章詳情</v>
       </c>
-      <c r="E104" s="3" t="str">
+      <c r="E104" s="5" t="str">
         <v>提升</v>
       </c>
-      <c r="F104" s="3" t="str">
+      <c r="F104" s="5" t="str">
         <v>內容</v>
       </c>
-      <c r="G104" s="3" t="str">
+      <c r="G104" s="5" t="str">
         <v>中</v>
       </c>
-      <c r="H104" s="3" t="str">
+      <c r="H104" s="5" t="str">
         <v>News 詳情頁缺乏多媒體展示能力</v>
       </c>
-      <c r="I104" s="3" t="str">
+      <c r="I104" s="5" t="str">
         <v>主管希望最新消息可內嵌 YouTube 影片，目前只有 HTML 編輯器內可手動貼連結，無內嵌影片渲染</v>
       </c>
-      <c r="J104" s="3" t="str">
+      <c r="J104" s="5" t="str">
         <v>後台 admin 加「影片網址」el-input + WebAPI.ts InsertNews/UpdateNews 加 videoUrl 參數；前台 news/info.vue 加 iframe section + YouTube URL → embed URL parser (regex 抓 11 字元 video ID) + 16:9 響應式容器 (padding-top: 56.25%)</v>
       </c>
-      <c r="K104" s="3" t="str">
+      <c r="K104" s="5" t="str">
         <v>pages/news/info.vue + News_AddEditView.vue (admin) + WebAPI.ts (admin)</v>
       </c>
-      <c r="L104" s="3" t="str" xml:space="preserve">
+      <c r="L104" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/news/info.vue_x000d__x000d__x000d_
 iFare_Backend/src/views/News/News_AddEditView.vue_x000d__x000d__x000d_
 iFare_Backend/src/plugins/WebAPI.ts</v>
       </c>
-      <c r="M104" s="3" t="str">
+      <c r="M104" s="5" t="str">
         <v>UI 端 wiring 完成；對應後臺優化 #13 (.NET News VideoUrl 欄位)</v>
       </c>
-      <c r="N104" s="3" t="str">
+      <c r="N104" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O104" s="3" t="str">
+      <c r="O104" s="5" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P104" s="3" t="str">
+      <c r="P104" s="5" t="str">
         <v>等 .NET 後端 News.cs entity + DTO + EF migration 加 VideoUrl 才能真實運作</v>
       </c>
     </row>
     <row r="105" ht="115.2" customHeight="1" xml:space="preserve">
-      <c r="A105" s="3">
+      <c r="A105" s="7">
         <v>103</v>
       </c>
-      <c r="B105" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C105" s="3" t="str">
+      <c r="B105" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C105" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D105" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E105" s="3" t="str">
+      <c r="D105" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E105" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F105" s="3" t="str">
+      <c r="F105" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G105" s="3" t="str">
+      <c r="G105" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H105" s="3" t="str">
+      <c r="H105" s="7" t="str">
         <v>本機開發 API 連線失敗 (環境設定指本機 .NET，但機器沒 .NET SDK)</v>
       </c>
-      <c r="I105" s="3" t="str">
+      <c r="I105" s="7" t="str">
         <v>前台 nuxt.config.ts devProxy target 寫死 https://localhost:44312 / 後台 AjaxRef.ts baseURL prod 寫死 http://10.200.0.39 (公司內網 IP)，導致：(1) 本機 dev 抓 dropdown 全 404 (2) 後台 admin Login 失敗 (家用網路 reach 不到 10.200.0.39 內網 IP)</v>
       </c>
-      <c r="J105" s="3" t="str">
+      <c r="J105" s="7" t="str">
         <v>前台 nuxt.config.ts devProxy target 改 https://www.i-fare.org.tw/ifare_api/api/services/app；後台 AjaxRef.getBaseUrl() 改 https://www.i-fare.org.tw/ifare_bdapi (固定走正式)</v>
       </c>
-      <c r="K105" s="3" t="str">
+      <c r="K105" s="7" t="str">
         <v>nuxt.config.ts (前台) + AjaxRef.ts (後台)</v>
       </c>
-      <c r="L105" s="3" t="str" xml:space="preserve">
+      <c r="L105" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/nuxt.config.ts_x000d__x000d__x000d_
 iFare_Backend/src/plugins/AjaxRef.ts</v>
       </c>
-      <c r="M105" s="3" t="str">
+      <c r="M105" s="7" t="str">
         <v>Login 已驗證可通；前台 dropdown 已能抓資料</v>
       </c>
-      <c r="N105" s="3" t="str">
+      <c r="N105" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O105" s="3" t="str">
+      <c r="O105" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P105" s="3" t="str">
+      <c r="P105" s="7" t="str">
         <v>對應後臺優化 #8 / #14 (baseURL 環境變數化) — 目前是治標處理，等之後完整改成 .env</v>
       </c>
     </row>
     <row r="106" ht="172.80000000000004" customHeight="1" xml:space="preserve">
-      <c r="A106" s="3">
+      <c r="A106" s="7">
         <v>104</v>
       </c>
-      <c r="B106" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C106" s="3" t="str">
+      <c r="B106" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C106" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D106" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E106" s="3" t="str">
+      <c r="D106" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E106" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F106" s="3" t="str">
+      <c r="F106" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G106" s="3" t="str">
+      <c r="G106" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H106" s="3" t="str">
+      <c r="H106" s="7" t="str">
         <v>VS Code 顯示 3 個 TypeScript deprecation warning</v>
       </c>
-      <c r="I106" s="3" t="str">
+      <c r="I106" s="7" t="str">
         <v>iFare_Backend/tsconfig.app.json 用 baseUrl + moduleResolution=node10 / iFare_Frontend/tsconfig.json 透過 .nuxt/tsconfig.json extend 也帶 node10，被 TypeScript 5.x 標 deprecated (TS 7.0 才停用)</v>
       </c>
-      <c r="J106" s="3" t="str">
+      <c r="J106" s="7" t="str">
         <v>加 "ignoreDeprecations": "6.0" — 後台直接放 tsconfig.app.json compilerOptions；前台改透過 nuxt.config.ts typescript.tsConfig.compilerOptions 注入 .nuxt/tsconfig.json (因為 user-facing tsconfig.json 加 ignoreDeprecations 抑制不到 extend 的 .nuxt/tsconfig.json)</v>
       </c>
-      <c r="K106" s="3" t="str">
+      <c r="K106" s="7" t="str">
         <v>tsconfig.app.json + tsconfig.json + nuxt.config.ts</v>
       </c>
-      <c r="L106" s="3" t="str" xml:space="preserve">
+      <c r="L106" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Backend/tsconfig.app.json_x000d__x000d__x000d_
 iFare_Frontend/tsconfig.json_x000d__x000d__x000d_
 iFare_Frontend/nuxt.config.ts</v>
       </c>
-      <c r="M106" s="3" t="str">
+      <c r="M106" s="7" t="str">
         <v>TS 5.x 不影響執行 / build</v>
       </c>
-      <c r="N106" s="3" t="str">
+      <c r="N106" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O106" s="3" t="str">
+      <c r="O106" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P106" s="3" t="str">
+      <c r="P106" s="7" t="str">
         <v>純 IDE 觀感修補；VS Code 需 Ctrl+Shift+P → Restart TS Server 才會 reload</v>
       </c>
     </row>
     <row r="107" ht="115.2" customHeight="1" xml:space="preserve">
-      <c r="A107" s="3">
+      <c r="A107" s="7">
         <v>105</v>
       </c>
-      <c r="B107" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C107" s="3" t="str">
+      <c r="B107" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C107" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D107" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E107" s="3" t="str">
+      <c r="D107" s="7" t="str">
+        <v/>
+      </c>
+      <c r="E107" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F107" s="3" t="str">
+      <c r="F107" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G107" s="3" t="str">
+      <c r="G107" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H107" s="3" t="str">
+      <c r="H107" s="7" t="str">
         <v>主管手動合併 master 時漏合 5dfbf91/cf47cfa 部分改動</v>
       </c>
-      <c r="I107" s="3" t="str">
+      <c r="I107" s="7" t="str">
         <v>切到 master 開 feat/uiux-round4 新分支後抽樣驗證發現：5dfbf91 漏合的 footer 樣式 (LINE 綠/FB 藍 SVG icon、_appFooter.scss 重新設計、_animation.scss page transition、_rwd_appFooter.scss、Mail/Clock SVG)；cf47cfa 整個沒合 (About 靈動島 + News 卡片升級 + 社群外連結) — 9 個檔</v>
       </c>
-      <c r="J107" s="3" t="str">
+      <c r="J107" s="7" t="str">
         <v>從 frontend 分支 git show 補回 16 個檔到新分支對應路徑 (Dev/Dev Code/iFare_Frontend/...)；cf47cfa 9 檔以 d5a7674 commit；footer 7 檔以 e2b1cae commit</v>
       </c>
-      <c r="K107" s="3" t="str">
+      <c r="K107" s="7" t="str">
         <v>16 個 SCSS / Vue / SVG</v>
       </c>
-      <c r="L107" s="3" t="str" xml:space="preserve">
+      <c r="L107" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">Dev/Dev Code/iFare_Frontend/assets/style/components/_appFooter.scss_x000d__x000d__x000d_
 iFare_Frontend/assets/style/_animation.scss_x000d__x000d__x000d_
 iFare_Frontend/components/AppFooter.vue 等 16 檔</v>
       </c>
-      <c r="M107" s="3" t="str">
+      <c r="M107" s="7" t="str">
         <v>修補 release 環境必要</v>
       </c>
-      <c r="N107" s="3" t="str">
+      <c r="N107" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O107" s="3" t="str">
+      <c r="O107" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P107" s="3" t="str">
+      <c r="P107" s="7" t="str">
         <v>不是純 UI/UX 議題，但屬於 Round 1-3 work 真正落地的前提</v>
       </c>
     </row>
     <row r="108" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A108" s="3">
+      <c r="A108" s="7">
         <v>106</v>
       </c>
-      <c r="B108" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C108" s="3" t="str">
+      <c r="B108" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C108" s="7" t="str">
         <v>安全性</v>
       </c>
-      <c r="D108" s="3" t="str">
+      <c r="D108" s="7" t="str">
         <v>v-html XSS</v>
       </c>
-      <c r="E108" s="3" t="str">
+      <c r="E108" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F108" s="3" t="str">
+      <c r="F108" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G108" s="3" t="str">
+      <c r="G108" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H108" s="3" t="str">
+      <c r="H108" s="7" t="str">
         <v>v-html 渲染未清理的服務器內容，存在 XSS 風險</v>
       </c>
-      <c r="I108" s="3" t="str">
+      <c r="I108" s="7" t="str">
         <v>news/info, articles/lazy, articles/welfare, ifare/info 多頁用 v-html 渲染 API content；若後端未正確清理 HTML/JavaScript，可遭 XSS</v>
       </c>
-      <c r="J108" s="3" t="str">
+      <c r="J108" s="7" t="str">
         <v>用 DOMPurify 或 sanitize-html 清理 HTML；至少在伺服器端驗證內容不含危險標籤</v>
       </c>
-      <c r="K108" s="3" t="str">
+      <c r="K108" s="7" t="str">
         <v>pages/news/info.vue + articles/lazy/welfare + ifare/info</v>
       </c>
-      <c r="L108" s="3" t="str" xml:space="preserve">
+      <c r="L108" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/news/info.vue (L25)_x000d__x000d_
 iFare_Frontend/pages/articles/lazy.vue (L16)_x000d__x000d_
 iFare_Frontend/pages/articles/welfare.vue (L19)_x000d__x000d_
 iFare_Frontend/pages/ifare/info.vue (L23, 31, 40, 47)</v>
       </c>
-      <c r="M108" s="3" t="str">
+      <c r="M108" s="7" t="str">
         <v>高優先級安全缺陷</v>
       </c>
-      <c r="N108" s="3" t="str">
+      <c r="N108" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O108" s="3" t="str">
+      <c r="O108" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P108" s="3" t="str">
+      <c r="P108" s="7" t="str">
         <v>Round 9 (批次 B): 安裝 isomorphic-dompurify (SSR + client safe)；新增 composables/useSanitize.ts 統一清理規範 (white-list ALLOWED_TAGS / ALLOWED_ATTR、阻 javascript:/data: URI、FORBID script/style/iframe/onerror)；7 處 v-html 用 useSanitize 包起來: news/info、articles/lazy、articles/welfare、ifare/info × 4 (qualification/welfareInfo/evidence/remark)。</v>
       </c>
     </row>
     <row r="109" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A109" s="3">
+      <c r="A109" s="5">
         <v>107</v>
       </c>
-      <c r="B109" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C109" s="3" t="str">
+      <c r="B109" s="5" t="str">
+        <v>V</v>
+      </c>
+      <c r="C109" s="5" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D109" s="3" t="str">
+      <c r="D109" s="5" t="str">
         <v>WebAPI 錯誤處理</v>
       </c>
-      <c r="E109" s="3" t="str">
+      <c r="E109" s="5" t="str">
         <v>修復</v>
       </c>
-      <c r="F109" s="3" t="str">
+      <c r="F109" s="5" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G109" s="3" t="str">
+      <c r="G109" s="5" t="str">
         <v>高</v>
       </c>
-      <c r="H109" s="3" t="str">
+      <c r="H109" s="5" t="str">
         <v>WebAPI.ts 未區分錯誤類型，一律 return null，頁面無法判斷失敗原因</v>
       </c>
-      <c r="I109" s="3" t="str">
+      <c r="I109" s="5" t="str">
         <v>plugins/WebAPI.ts (L9-15) 捕獲所有錯誤返回 null，無法區分網路超時/伺服器 500/驗證失敗；news.vue 等雖有 hasError 但無法提示具體原因</v>
       </c>
-      <c r="J109" s="3" t="str">
+      <c r="J109" s="5" t="str">
         <v>返回結構化錯誤物件 {code, message, status}，頁面根據錯誤類型顯示不同提示 (網路錯誤、伺服器維護中等)</v>
       </c>
-      <c r="K109" s="3" t="str">
+      <c r="K109" s="5" t="str">
         <v>plugins/WebAPI.ts</v>
       </c>
-      <c r="L109" s="3" t="str" xml:space="preserve">
+      <c r="L109" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/plugins/WebAPI.ts_x000d__x000d_
 iFare_Frontend/pages/news.vue_x000d__x000d_
 iFare_Frontend/pages/articles.vue_x000d__x000d_
 iFare_Frontend/pages/ifare.vue</v>
       </c>
-      <c r="M109" s="3" t="str">
+      <c r="M109" s="5" t="str">
         <v>影響全站用戶體驗</v>
       </c>
-      <c r="N109" s="3" t="str">
+      <c r="N109" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="O109" s="3" t="str">
+      <c r="O109" s="5" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P109" s="3" t="str">
+      <c r="P109" s="5" t="str">
         <v>Round 9 (批次 B): plugins/WebAPI.ts 加 categorizeError (timeout/network/client/server/unknown)、結構化 logError 取代 console.error、try-catch wrapper。Return signature 不變 (data/null) 維持向下相容，所有 caller 不用改。**UI 端錯誤呈現** (顯示 toast / 重試提示) 尚未做，需與整體錯誤元件設計一起。</v>
       </c>
     </row>
     <row r="110" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A110" s="3">
+      <c r="A110" s="7">
         <v>108</v>
       </c>
-      <c r="B110" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C110" s="3" t="str">
+      <c r="B110" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C110" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D110" s="3" t="str">
+      <c r="D110" s="7" t="str">
         <v>API 超時</v>
       </c>
-      <c r="E110" s="3" t="str">
+      <c r="E110" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F110" s="3" t="str">
+      <c r="F110" s="7" t="str">
         <v>效能</v>
       </c>
-      <c r="G110" s="3" t="str">
+      <c r="G110" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H110" s="3" t="str">
+      <c r="H110" s="7" t="str">
         <v>$fetch 無超時設定，API 無回應頁面會無限期卡 loading</v>
       </c>
-      <c r="I110" s="3" t="str">
+      <c r="I110" s="7" t="str">
         <v>所有頁面的 API 呼叫未設 timeout，若 API 無回應，UI 會永遠停在 loading 無退出機制</v>
       </c>
-      <c r="J110" s="3" t="str">
+      <c r="J110" s="7" t="str">
         <v>WebAPI.ts 設預設 timeout 10-15 秒，超時返回特定錯誤碼讓頁面顯示「連線逾時，請重試」</v>
       </c>
-      <c r="K110" s="3" t="str">
+      <c r="K110" s="7" t="str">
         <v>plugins/WebAPI.ts</v>
       </c>
-      <c r="L110" s="3" t="str" xml:space="preserve">
+      <c r="L110" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/plugins/WebAPI.ts_x000d__x000d_
 iFare_Frontend/pages/news/info.vue_x000d__x000d_
 iFare_Frontend/pages/articles/lazy.vue_x000d__x000d_
 iFare_Frontend/pages/articles/welfare.vue_x000d__x000d_
 iFare_Frontend/pages/ifare/contact.vue</v>
       </c>
-      <c r="M110" s="3" t="str">
+      <c r="M110" s="7" t="str">
         <v>可能導致用戶感知應用無反應</v>
       </c>
-      <c r="N110" s="3" t="str">
+      <c r="N110" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O110" s="3" t="str">
+      <c r="O110" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P110" s="3" t="str">
+      <c r="P110" s="7" t="str">
         <v>Round 9 (批次 B): plugins/WebAPI.ts WebApiGet/WebApiPost $fetch 加 timeout: API_TIMEOUT_MS (15000ms)。逾時會被 categorizeError 標記為 timeout 類別。</v>
       </c>
     </row>
     <row r="111" ht="14.4" customHeight="1">
-      <c r="A111" s="3">
+      <c r="A111" s="7">
         <v>109</v>
       </c>
-      <c r="B111" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C111" s="3" t="str">
+      <c r="B111" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C111" s="7" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D111" s="3" t="str">
+      <c r="D111" s="7" t="str">
         <v>ifare/contact</v>
       </c>
-      <c r="E111" s="3" t="str">
+      <c r="E111" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F111" s="3" t="str">
+      <c r="F111" s="7" t="str">
         <v>互動</v>
       </c>
-      <c r="G111" s="3" t="str">
+      <c r="G111" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H111" s="3" t="str">
+      <c r="H111" s="7" t="str">
         <v>contact.vue 缺 API 失敗處理，API 失敗用戶看不到內容</v>
       </c>
-      <c r="I111" s="3" t="str">
+      <c r="I111" s="7" t="str">
         <v>ifare/contact.vue (L153) 呼叫 GetIFareOfficeUnitList 但無檢查 res.result、無 catch 區塊、無 loading/error 狀態。若 API 失敗頁面呈現空白</v>
       </c>
-      <c r="J111" s="3" t="str">
+      <c r="J111" s="7" t="str">
         <v>加 try-catch、loading ref、error 狀態，仿 news.vue 的錯誤處理模式</v>
       </c>
-      <c r="K111" s="3" t="str">
+      <c r="K111" s="7" t="str">
         <v>pages/ifare/contact.vue</v>
       </c>
-      <c r="L111" s="3" t="str">
+      <c r="L111" s="7" t="str">
         <v>iFare_Frontend/pages/ifare/contact.vue</v>
       </c>
-      <c r="M111" s="3" t="str">
+      <c r="M111" s="7" t="str">
         <v>用戶無法看到聯絡資訊時毫無提示</v>
       </c>
-      <c r="N111" s="3" t="str">
+      <c r="N111" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O111" s="3" t="str">
+      <c r="O111" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P111" s="3" t="str">
+      <c r="P111" s="7" t="str">
         <v>Round 9 (批次 B): pages/ifare/contact.vue 重構為 loadOfficeUnit() async + isLoading/hasError ref。template 加 v-if 三分支: loading (skeleton-line role=status)、error (重試按鈕 role=alert)、success (原內容)。重試會清空既有資料再呼叫。</v>
       </c>
     </row>
     <row r="112" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A112" s="3">
+      <c r="A112" s="7">
         <v>110</v>
       </c>
-      <c r="B112" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C112" s="3" t="str">
+      <c r="B112" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C112" s="7" t="str">
         <v>全站通用</v>
       </c>
-      <c r="D112" s="3" t="str">
+      <c r="D112" s="7" t="str">
         <v>console.log</v>
       </c>
-      <c r="E112" s="3" t="str">
+      <c r="E112" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F112" s="3" t="str">
+      <c r="F112" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G112" s="3" t="str">
+      <c r="G112" s="7" t="str">
         <v>高</v>
       </c>
-      <c r="H112" s="3" t="str">
+      <c r="H112" s="7" t="str">
         <v>生產環境仍有 20+ 個 console.log，洩露內部邏輯</v>
       </c>
-      <c r="I112" s="3" t="str">
+      <c r="I112" s="7" t="str">
         <v>news.vue (L198), ifare.vue (L305), ifare/result.vue (L236-265, 385, 541), ifare/contact.vue (L163, 193) 等多處 console.log，可被用戶開發工具看到</v>
       </c>
-      <c r="J112" s="3" t="str">
+      <c r="J112" s="7" t="str">
         <v>移除所有生產 console.log，改用生產環境禁用的日誌系統，或開發時用環境變數判斷</v>
       </c>
-      <c r="K112" s="3" t="str">
+      <c r="K112" s="7" t="str">
         <v>多 pages</v>
       </c>
-      <c r="L112" s="3" t="str" xml:space="preserve">
+      <c r="L112" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/news.vue_x000d__x000d_
 iFare_Frontend/pages/ifare.vue_x000d__x000d_
 iFare_Frontend/pages/ifare/result.vue_x000d__x000d_
@@ -9617,16 +9665,16 @@
 iFare_Frontend/components/CompPage.vue_x000d__x000d_
 iFare_Frontend/components/CompPageNum.vue</v>
       </c>
-      <c r="M112" s="3" t="str">
+      <c r="M112" s="7" t="str">
         <v>安全與代碼質量問題</v>
       </c>
-      <c r="N112" s="3" t="str">
+      <c r="N112" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O112" s="3" t="str">
+      <c r="O112" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P112" s="3" t="str">
+      <c r="P112" s="7" t="str">
         <v>Round 7 (批次 A): 移除 13 處 console.log — pages/news.vue (1)、pages/ifare.vue (1)、pages/ifare/result.vue (5)、pages/ifare/contact.vue (2)、components/CompPage.vue (4)。保留 pages/ifare/info.vue:203 的 console.error (catch 內合理錯誤處理)。</v>
       </c>
     </row>
@@ -9682,54 +9730,54 @@
       </c>
     </row>
     <row r="114" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A114" s="3">
+      <c r="A114" s="7">
         <v>112</v>
       </c>
-      <c r="B114" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C114" s="3" t="str">
+      <c r="B114" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C114" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="D114" s="3" t="str">
+      <c r="D114" s="7" t="str">
         <v>圖片 alt</v>
       </c>
-      <c r="E114" s="3" t="str">
+      <c r="E114" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F114" s="3" t="str">
+      <c r="F114" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G114" s="3" t="str">
+      <c r="G114" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H114" s="3" t="str">
+      <c r="H114" s="7" t="str">
         <v>多頁圖片 alt 屬性缺失 (collaborator, articles/lazy, index 背景)</v>
       </c>
-      <c r="I114" s="3" t="str">
+      <c r="I114" s="7" t="str">
         <v>collaborator.vue (L22) &lt;img&gt; 無 alt；articles/lazy.vue (L77) 自動生成 &lt;img&gt; 無 alt；index 背景 CSS 無 alt</v>
       </c>
-      <c r="J114" s="3" t="str">
+      <c r="J114" s="7" t="str">
         <v>所有 img 加 alt (collaborator 用機構名稱，articles/lazy 用文章標題)；背景圖改 img 或加 aria-label</v>
       </c>
-      <c r="K114" s="3" t="str">
+      <c r="K114" s="7" t="str">
         <v>collaborator / articles/lazy / index</v>
       </c>
-      <c r="L114" s="3" t="str" xml:space="preserve">
+      <c r="L114" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/collaborator.vue_x000d__x000d_
 iFare_Frontend/pages/articles/lazy.vue_x000d__x000d_
 iFare_Frontend/pages/index.vue</v>
       </c>
-      <c r="M114" s="3" t="str">
+      <c r="M114" s="7" t="str">
         <v>WCAG 2.1 AA 必要，影響視障用戶</v>
       </c>
-      <c r="N114" s="3" t="str">
+      <c r="N114" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O114" s="3" t="str">
+      <c r="O114" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P114" s="3" t="str">
+      <c r="P114" s="7" t="str">
         <v>Round 8 (批次 C): pages/index.vue 的 .part-bg-top 加 aria-hidden="true" — 5 張裝飾性 .bg-img 不需被屏幕閱讀器讀。collaborator.vue + articles/lazy.vue 的 &lt;img&gt; alt 已在 Round 7 (#127) 順手做。</v>
       </c>
     </row>
@@ -9785,108 +9833,108 @@
       </c>
     </row>
     <row r="116" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A116" s="3">
+      <c r="A116" s="7">
         <v>114</v>
       </c>
-      <c r="B116" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C116" s="3" t="str">
+      <c r="B116" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C116" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D116" s="3" t="str">
+      <c r="D116" s="7" t="str">
         <v>CompSelect 鍵盤</v>
       </c>
-      <c r="E116" s="3" t="str">
+      <c r="E116" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F116" s="3" t="str">
+      <c r="F116" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G116" s="3" t="str">
+      <c r="G116" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H116" s="3" t="str">
+      <c r="H116" s="7" t="str">
         <v>CompSelect 系列元件無鍵盤操作 (Tab/Enter/Esc/Arrow)，僅滑鼠</v>
       </c>
-      <c r="I116" s="3" t="str">
+      <c r="I116" s="7" t="str">
         <v>CompSelect / CompSelectRecipient / CompSelectElse 的開關、選項點擊均未綁定鍵盤事件，無法用鍵盤導航選擇</v>
       </c>
-      <c r="J116" s="3" t="str">
+      <c r="J116" s="7" t="str">
         <v>加 @keydown.tab/enter/esc/arrow-down/up 事件，實現 ARIA authoring practices 完整鍵盤導航</v>
       </c>
-      <c r="K116" s="3" t="str">
+      <c r="K116" s="7" t="str">
         <v>components/CompSelect*</v>
       </c>
-      <c r="L116" s="3" t="str" xml:space="preserve">
+      <c r="L116" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/CompSelect.vue_x000d__x000d_
 iFare_Frontend/components/CompSelectRecipient.vue_x000d__x000d_
 iFare_Frontend/components/CompSelectElse.vue</v>
       </c>
-      <c r="M116" s="3" t="str">
+      <c r="M116" s="7" t="str">
         <v>WCAG 2.1 AA 必要</v>
       </c>
-      <c r="N116" s="3" t="str">
+      <c r="N116" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O116" s="3" t="str">
+      <c r="O116" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P116" s="3" t="str">
+      <c r="P116" s="7" t="str">
         <v>Round 8 (批次 C): 3 個 component (CompSelect / CompSelectRecipient / CompSelectElse) 加 tabindex="0" + role="combobox" + aria-expanded + aria-haspopup + aria-label。CompSelect / CompSelectRecipient 加完整鍵盤導航 (Enter/Space toggle 或選擇 focused 項目；Esc 關閉；Arrow Up/Down 切換 focused 項目)；CompSelectElse 因含兩組選項 (Income + Identity) 結構複雜，僅加 Enter/Space toggle + Esc 關閉，方向鍵需後續再處理。選項加 role="option" + aria-selected。</v>
       </c>
     </row>
     <row r="117" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A117" s="3">
+      <c r="A117" s="7">
         <v>115</v>
       </c>
-      <c r="B117" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C117" s="3" t="str">
+      <c r="B117" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C117" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="D117" s="3" t="str">
+      <c r="D117" s="7" t="str">
         <v>Heading 層級</v>
       </c>
-      <c r="E117" s="3" t="str">
+      <c r="E117" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F117" s="3" t="str">
+      <c r="F117" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G117" s="3" t="str">
+      <c r="G117" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H117" s="3" t="str">
+      <c r="H117" s="7" t="str">
         <v>Heading 層級結構不規範，多頁 h3 直接跟 h1 後，h6 用於非末級</v>
       </c>
-      <c r="I117" s="3" t="str">
+      <c r="I117" s="7" t="str">
         <v>about.vue (L11 h3 缺 h2)、index.vue (L21 h1 + L38 h3)、news/info.vue (L4 h2 後直接 h6)、ifare/info.vue (L5 h1 + L21 h3) 不遵循層級規則</v>
       </c>
-      <c r="J117" s="3" t="str">
+      <c r="J117" s="7" t="str">
         <v>調整 heading 層級遞增 (h1 &gt; h2 &gt; h3...)；不跳級；副標題用適當 h2-h3 而非 h6</v>
       </c>
-      <c r="K117" s="3" t="str">
+      <c r="K117" s="7" t="str">
         <v>about / index / news/info / ifare/info / collaborator</v>
       </c>
-      <c r="L117" s="3" t="str" xml:space="preserve">
+      <c r="L117" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/about.vue_x000d__x000d_
 iFare_Frontend/pages/index.vue_x000d__x000d_
 iFare_Frontend/pages/news/info.vue_x000d__x000d_
 iFare_Frontend/pages/ifare/info.vue_x000d__x000d_
 iFare_Frontend/pages/collaborator.vue</v>
       </c>
-      <c r="M117" s="3" t="str">
+      <c r="M117" s="7" t="str">
         <v>影響屏幕閱讀器用戶導航</v>
       </c>
-      <c r="N117" s="3" t="str">
+      <c r="N117" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O117" s="3" t="str">
+      <c r="O117" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P117" s="3" t="str">
+      <c r="P117" s="7" t="str">
         <v>Round 8 (批次 C): 已 grep 確認 SCSS 全用 class selector (.comp-title / .member-name / .news-title 等)，改 tag 不破壞視覺。修正：about.vue (h3 → h1 主標 / h6 → h4 member-name × 3)；index.vue (h3 → p sub-title / h2 → h4 news-title / h2 → h4 card-title)；news/info.vue (h6 → p article-date)；ifare/info.vue (h3 → h2 × 5 區塊標 / h5 → h2 relation-title / h6 → h3 link-title)。</v>
       </c>
     </row>
@@ -9995,52 +10043,52 @@
       </c>
     </row>
     <row r="120" ht="14.4" customHeight="1">
-      <c r="A120" s="3">
+      <c r="A120" s="7">
         <v>118</v>
       </c>
-      <c r="B120" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C120" s="3" t="str">
+      <c r="B120" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C120" s="7" t="str">
         <v>最新消息</v>
       </c>
-      <c r="D120" s="3" t="str">
+      <c r="D120" s="7" t="str">
         <v>iframe 安全</v>
       </c>
-      <c r="E120" s="3" t="str">
+      <c r="E120" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F120" s="3" t="str">
+      <c r="F120" s="7" t="str">
         <v>程式碼</v>
       </c>
-      <c r="G120" s="3" t="str">
+      <c r="G120" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H120" s="3" t="str">
+      <c r="H120" s="7" t="str">
         <v>YouTube iframe 缺 sandbox 屬性，allow 過寬鬆</v>
       </c>
-      <c r="I120" s="3" t="str">
+      <c r="I120" s="7" t="str">
         <v>news/info.vue (L12-19) iframe allow 含 accelerometer/autoplay/clipboard-write 等未設 sandbox，可能被跨域腳本利用</v>
       </c>
-      <c r="J120" s="3" t="str">
+      <c r="J120" s="7" t="str">
         <v>加 sandbox="allow-same-origin allow-scripts allow-presentation"；移除非必要 allow (例如 clipboard-write)</v>
       </c>
-      <c r="K120" s="3" t="str">
+      <c r="K120" s="7" t="str">
         <v>pages/news/info.vue</v>
       </c>
-      <c r="L120" s="3" t="str">
+      <c r="L120" s="7" t="str">
         <v>iFare_Frontend/pages/news/info.vue</v>
       </c>
-      <c r="M120" s="3" t="str">
+      <c r="M120" s="7" t="str">
         <v>防止潛在跨域攻擊</v>
       </c>
-      <c r="N120" s="3" t="str">
+      <c r="N120" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O120" s="3" t="str">
+      <c r="O120" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P120" s="3" t="str">
+      <c r="P120" s="7" t="str">
         <v>Round 9 (批次 B): pages/news/info.vue 的 YouTube iframe 加 sandbox="allow-same-origin allow-scripts allow-presentation allow-popups"；移除非必要 allow="clipboard-write" (剪貼簿權限不應自動給)。</v>
       </c>
     </row>
@@ -10097,52 +10145,52 @@
       </c>
     </row>
     <row r="122" ht="14.4" customHeight="1">
-      <c r="A122" s="3">
+      <c r="A122" s="7">
         <v>120</v>
       </c>
-      <c r="B122" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C122" s="3" t="str">
+      <c r="B122" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C122" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D122" s="3" t="str">
+      <c r="D122" s="7" t="str">
         <v>AppFooter 版權</v>
       </c>
-      <c r="E122" s="3" t="str">
+      <c r="E122" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F122" s="3" t="str">
+      <c r="F122" s="7" t="str">
         <v>內容</v>
       </c>
-      <c r="G122" s="3" t="str">
+      <c r="G122" s="7" t="str">
         <v>中</v>
       </c>
-      <c r="H122" s="3" t="str">
+      <c r="H122" s="7" t="str">
         <v>Footer 版權年份過舊 (1995-2020)，已過期 6 年</v>
       </c>
-      <c r="I122" s="3" t="str">
+      <c r="I122" s="7" t="str">
         <v>AppFooter.vue (L42) 顯示「© 1995-2020」，現在是 2026</v>
       </c>
-      <c r="J122" s="3" t="str">
+      <c r="J122" s="7" t="str">
         <v>改 `© 1995-${new Date().getFullYear()}`，或在 footer data 中維護</v>
       </c>
-      <c r="K122" s="3" t="str">
+      <c r="K122" s="7" t="str">
         <v>components/AppFooter.vue</v>
       </c>
-      <c r="L122" s="3" t="str">
+      <c r="L122" s="7" t="str">
         <v>iFare_Frontend/components/AppFooter.vue (L42)</v>
       </c>
-      <c r="M122" s="3" t="str">
+      <c r="M122" s="7" t="str">
         <v>簡易修復</v>
       </c>
-      <c r="N122" s="3" t="str">
+      <c r="N122" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O122" s="3" t="str">
+      <c r="O122" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P122" s="3" t="str">
+      <c r="P122" s="7" t="str">
         <v>Round 7 (批次 A): components/AppFooter.vue L42 「© 1995-2020」改成 「© 1995-{{ new Date().getFullYear() }}」 — 模板內 inline 執行，自動跟系統年份。</v>
       </c>
     </row>
@@ -10352,154 +10400,154 @@
       </c>
     </row>
     <row r="127" ht="14.4" customHeight="1">
-      <c r="A127" s="3">
+      <c r="A127" s="7">
         <v>125</v>
       </c>
-      <c r="B127" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C127" s="3" t="str">
+      <c r="B127" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C127" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D127" s="3" t="str">
+      <c r="D127" s="7" t="str">
         <v>AppHeader 行動 focus</v>
       </c>
-      <c r="E127" s="3" t="str">
+      <c r="E127" s="7" t="str">
         <v>修復</v>
       </c>
-      <c r="F127" s="3" t="str">
+      <c r="F127" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G127" s="3" t="str">
+      <c r="G127" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H127" s="3" t="str">
+      <c r="H127" s="7" t="str">
         <v>AppHeader 行動菜單開啟時焦點未自動移至菜單，關閉時未返回觸發按鈕</v>
       </c>
-      <c r="I127" s="3" t="str">
+      <c r="I127" s="7" t="str">
         <v>AppHeader.vue (L136) 菜單關閉按鈕有 focus，但開啟時焦點未管理，屏幕閱讀器用戶會迷失</v>
       </c>
-      <c r="J127" s="3" t="str">
+      <c r="J127" s="7" t="str">
         <v>用 ref 在菜單開啟時 focus 至菜單標題或第一個項目；關閉時 focus 返回菜單按鈕</v>
       </c>
-      <c r="K127" s="3" t="str">
+      <c r="K127" s="7" t="str">
         <v>components/AppHeader.vue</v>
       </c>
-      <c r="L127" s="3" t="str">
+      <c r="L127" s="7" t="str">
         <v>iFare_Frontend/components/AppHeader.vue (L136)</v>
       </c>
-      <c r="M127" s="3" t="str">
+      <c r="M127" s="7" t="str">
         <v>增進屏幕閱讀器友善性</v>
       </c>
-      <c r="N127" s="3" t="str">
+      <c r="N127" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O127" s="3" t="str">
+      <c r="O127" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P127" s="3" t="str">
+      <c r="P127" s="7" t="str">
         <v>Round 8 (批次 C): components/AppHeader.vue 加 menuButtonRef 綁 .btn-menu，watch(isShowMenu) → 開啟時 querySelector focus 至首個 mobile menu link，關閉時 focus 回菜單按鈕。.btn-menu 加 :aria-expanded="isShowMenu" + aria-controls="mobile-menu" + aria-label="開啟菜單"；.mobile-menu 加 id="mobile-menu" + role="dialog" + aria-modal="true" + aria-label="行動選單"。全域加 ESC 鍵監聽關閉 menu (onMounted/onBeforeUnmount window.addEventListener)。</v>
       </c>
     </row>
     <row r="128" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A128" s="3">
+      <c r="A128" s="7">
         <v>126</v>
       </c>
-      <c r="B128" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C128" s="3" t="str">
+      <c r="B128" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C128" s="7" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="D128" s="3" t="str">
+      <c r="D128" s="7" t="str">
         <v>disabled 視覺</v>
       </c>
-      <c r="E128" s="3" t="str">
+      <c r="E128" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F128" s="3" t="str">
+      <c r="F128" s="7" t="str">
         <v>視覺</v>
       </c>
-      <c r="G128" s="3" t="str">
+      <c r="G128" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H128" s="3" t="str">
+      <c r="H128" s="7" t="str">
         <v>ifare.vue 搜尋按鈕 disabled 狀態無灰化視覺反饋</v>
       </c>
-      <c r="I128" s="3" t="str">
+      <c r="I128" s="7" t="str">
         <v>ifare.vue (L79) :disabled="!canSearch" 但 SCSS 無 button:disabled 樣式，用戶可能誤以為按鈕可點</v>
       </c>
-      <c r="J128" s="3" t="str">
+      <c r="J128" s="7" t="str">
         <v>_button.scss 加 button:disabled { opacity: 0.5; cursor: not-allowed; }</v>
       </c>
-      <c r="K128" s="3" t="str">
+      <c r="K128" s="7" t="str">
         <v>pages/ifare.vue + _button.scss</v>
       </c>
-      <c r="L128" s="3" t="str" xml:space="preserve">
+      <c r="L128" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/ifare.vue (L79)_x000d__x000d_
 iFare_Frontend/assets/style/components/_button.scss</v>
       </c>
-      <c r="M128" s="3" t="str">
+      <c r="M128" s="7" t="str">
         <v>簡易視覺修復</v>
       </c>
-      <c r="N128" s="3" t="str">
+      <c r="N128" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O128" s="3" t="str">
+      <c r="O128" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P128" s="3" t="str">
+      <c r="P128" s="7" t="str">
         <v>Round 7 (批次 A): assets/style/components/_button.scss 開頭加 generic 規則 — button:disabled / .btn:disabled / .btn.disabled 都套 opacity 0.5 + cursor not-allowed + pointer-events none。.btn-filter 既有 disabled 樣式 (L186) 不衝突。</v>
       </c>
     </row>
     <row r="129" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A129" s="3">
+      <c r="A129" s="7">
         <v>127</v>
       </c>
-      <c r="B129" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C129" s="3" t="str">
+      <c r="B129" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C129" s="7" t="str">
         <v>效能</v>
       </c>
-      <c r="D129" s="3" t="str">
+      <c r="D129" s="7" t="str">
         <v>圖片 lazy load</v>
       </c>
-      <c r="E129" s="3" t="str">
+      <c r="E129" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F129" s="3" t="str">
+      <c r="F129" s="7" t="str">
         <v>效能</v>
       </c>
-      <c r="G129" s="3" t="str">
+      <c r="G129" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H129" s="3" t="str">
+      <c r="H129" s="7" t="str">
         <v>collaborator 機構圖片、articles/lazy 自動生成圖片未設 loading="lazy"</v>
       </c>
-      <c r="I129" s="3" t="str">
+      <c r="I129" s="7" t="str">
         <v>collaborator.vue (L22) 和 articles/lazy.vue (L77 動態) 的 &lt;img&gt; 無 loading 屬性，所有圖片串行加載</v>
       </c>
-      <c r="J129" s="3" t="str">
+      <c r="J129" s="7" t="str">
         <v>所有 &lt;img&gt; 加 loading="lazy" (首屏 eager)；大圖考慮 WebP 或壓縮</v>
       </c>
-      <c r="K129" s="3" t="str">
+      <c r="K129" s="7" t="str">
         <v>pages/collaborator + articles/lazy</v>
       </c>
-      <c r="L129" s="3" t="str" xml:space="preserve">
+      <c r="L129" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/pages/collaborator.vue_x000d__x000d_
 iFare_Frontend/pages/articles/lazy.vue</v>
       </c>
-      <c r="M129" s="3" t="str">
+      <c r="M129" s="7" t="str">
         <v>首屏效能優化</v>
       </c>
-      <c r="N129" s="3" t="str">
+      <c r="N129" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O129" s="3" t="str">
+      <c r="O129" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P129" s="3" t="str">
+      <c r="P129" s="7" t="str">
         <v>Round 7 (批次 A): pages/collaborator.vue L22 &lt;img&gt; 加 loading="lazy" + :alt="`${_coll.title} logo`"；pages/articles/lazy.vue L77 動態 &lt;img&gt; 加 loading="lazy" + alt="${title} - ${j+1}"。</v>
       </c>
     </row>
@@ -10606,103 +10654,103 @@
       </c>
     </row>
     <row r="132" ht="14.4" customHeight="1">
-      <c r="A132" s="3">
+      <c r="A132" s="7">
         <v>130</v>
       </c>
-      <c r="B132" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C132" s="3" t="str">
+      <c r="B132" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C132" s="7" t="str">
         <v>共用元件</v>
       </c>
-      <c r="D132" s="3" t="str">
+      <c r="D132" s="7" t="str">
         <v>AppHeader aria</v>
       </c>
-      <c r="E132" s="3" t="str">
+      <c r="E132" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F132" s="3" t="str">
+      <c r="F132" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G132" s="3" t="str">
+      <c r="G132" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H132" s="3" t="str">
+      <c r="H132" s="7" t="str">
         <v>AppHeader 行動菜單關閉按鈕無 aria-label</v>
       </c>
-      <c r="I132" s="3" t="str">
+      <c r="I132" s="7" t="str">
         <v>AppHeader.vue (L136) &lt;button class="btn btn-icon btn-close"&gt; 無 aria-label，屏幕閱讀器只念「按鈕」</v>
       </c>
-      <c r="J132" s="3" t="str">
+      <c r="J132" s="7" t="str">
         <v>加 aria-label="關閉菜單"</v>
       </c>
-      <c r="K132" s="3" t="str">
+      <c r="K132" s="7" t="str">
         <v>components/AppHeader.vue</v>
       </c>
-      <c r="L132" s="3" t="str">
+      <c r="L132" s="7" t="str">
         <v>iFare_Frontend/components/AppHeader.vue (L136)</v>
       </c>
-      <c r="M132" s="3" t="str">
+      <c r="M132" s="7" t="str">
         <v>簡易無障礙修復</v>
       </c>
-      <c r="N132" s="3" t="str">
+      <c r="N132" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O132" s="3" t="str">
+      <c r="O132" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P132" s="3" t="str">
+      <c r="P132" s="7" t="str">
         <v>Round 7 (批次 A): components/AppHeader.vue L136 行動選單 .btn-close 加 aria-label="關閉菜單"。</v>
       </c>
     </row>
     <row r="133" ht="14.4" customHeight="1" xml:space="preserve">
-      <c r="A133" s="3">
+      <c r="A133" s="7">
         <v>131</v>
       </c>
-      <c r="B133" s="3" t="str">
-        <v>V</v>
-      </c>
-      <c r="C133" s="3" t="str">
+      <c r="B133" s="7" t="str">
+        <v>V</v>
+      </c>
+      <c r="C133" s="7" t="str">
         <v>導航</v>
       </c>
-      <c r="D133" s="3" t="str">
+      <c r="D133" s="7" t="str">
         <v>aria-current</v>
       </c>
-      <c r="E133" s="3" t="str">
+      <c r="E133" s="7" t="str">
         <v>提升</v>
       </c>
-      <c r="F133" s="3" t="str">
+      <c r="F133" s="7" t="str">
         <v>無障礙</v>
       </c>
-      <c r="G133" s="3" t="str">
+      <c r="G133" s="7" t="str">
         <v>低</v>
       </c>
-      <c r="H133" s="3" t="str">
+      <c r="H133" s="7" t="str">
         <v>AppHeader 與其他導航元件當前頁面連結無 aria-current="page"</v>
       </c>
-      <c r="I133" s="3" t="str">
+      <c r="I133" s="7" t="str">
         <v>AppHeader (L48-69) 用 :class="{ active: $route.name }" 但無 aria-current；屏幕閱讀器無法知道哪個是當前頁</v>
       </c>
-      <c r="J133" s="3" t="str">
+      <c r="J133" s="7" t="str">
         <v>:aria-current="$route.name === 'about' ? 'page' : undefined"</v>
       </c>
-      <c r="K133" s="3" t="str">
+      <c r="K133" s="7" t="str">
         <v>components/AppHeader + CompBreadCrumb</v>
       </c>
-      <c r="L133" s="3" t="str" xml:space="preserve">
+      <c r="L133" s="7" t="str" xml:space="preserve">
         <v xml:space="preserve">iFare_Frontend/components/AppHeader.vue_x000d__x000d_
 iFare_Frontend/components/CompBreadCrumb.vue</v>
       </c>
-      <c r="M133" s="3" t="str">
+      <c r="M133" s="7" t="str">
         <v>WCAG 2.1 最佳實踐 + 外部連結指示符可選加 ic-external-link icon</v>
       </c>
-      <c r="N133" s="3" t="str">
+      <c r="N133" s="7" t="str">
         <v>已修正</v>
       </c>
-      <c r="O133" s="3" t="str">
+      <c r="O133" s="7" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="P133" s="3" t="str">
+      <c r="P133" s="7" t="str">
         <v>Round 7 (批次 A): components/AppHeader.vue 桌面 5 + 行動 6 + i-Fare 桌面 1 共 12 個 NuxtLink 加 :aria-current="$route.name === 'xxx' ? 'page' : undefined"。i-Fare 用 includes('ifare') 涵蓋子路由。</v>
       </c>
     </row>
@@ -10731,54 +10779,54 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="3" t="str">
         <v>【1】整體進度</v>
       </c>
-      <c r="B1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H1" s="4" t="str">
+      <c r="B1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H1" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="3" t="str">
         <v>Sheet 名稱</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="3" t="str">
         <v>總計</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="3" t="str">
         <v>已修正</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="3" t="str">
         <v>部分修正</v>
       </c>
-      <c r="E2" s="5" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="F2" s="5" t="str">
+      <c r="E2" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="F2" s="3" t="str">
         <v>完成率</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="3" t="str">
         <v>備註</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -10789,13 +10837,13 @@
       <c r="B3" s="3">
         <v>131</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>39</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="3">
         <v>7</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="3">
         <v>85</v>
       </c>
       <c r="F3" s="3" t="str">
@@ -10815,13 +10863,13 @@
       <c r="B4" s="3">
         <v>54</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>0</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="3">
         <v>0</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="3">
         <v>54</v>
       </c>
       <c r="F4" s="3" t="str">
@@ -10841,13 +10889,13 @@
       <c r="B5" s="3">
         <v>12</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="3">
         <v>0</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="3">
         <v>12</v>
       </c>
       <c r="F5" s="3" t="str">
@@ -10861,54 +10909,54 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="3" t="str">
         <v>【2】Round 時間軸 — 每輪做了什麼</v>
       </c>
-      <c r="B7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="4" t="str">
+      <c r="B7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
+      <c r="A8" s="3" t="str">
         <v>Round</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B8" s="3" t="str">
         <v>日期</v>
       </c>
-      <c r="C8" s="5" t="str">
+      <c r="C8" s="3" t="str">
         <v>主題</v>
       </c>
-      <c r="D8" s="5" t="str">
+      <c r="D8" s="3" t="str">
         <v>UIUX 標完成</v>
       </c>
-      <c r="E8" s="5" t="str">
+      <c r="E8" s="3" t="str">
         <v>UIUX 新增</v>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="3" t="str">
         <v>後臺新增</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="3" t="str">
         <v>Schema</v>
       </c>
-      <c r="H8" s="5" t="str">
+      <c r="H8" s="3" t="str">
         <v>主要產出</v>
       </c>
     </row>
@@ -11069,54 +11117,54 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="str">
+      <c r="A16" s="3" t="str">
         <v>【3】後臺優化 — 5 主軸分布 (拿這個去提案!)</v>
       </c>
-      <c r="B16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G16" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H16" s="4" t="str">
+      <c r="B16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G16" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H16" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="str">
+      <c r="A17" s="3" t="str">
         <v>主軸</v>
       </c>
-      <c r="B17" s="5" t="str">
+      <c r="B17" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C17" s="5" t="str">
+      <c r="C17" s="3" t="str">
         <v>比例</v>
       </c>
-      <c r="D17" s="5" t="str">
+      <c r="D17" s="3" t="str">
         <v>主要訴求</v>
       </c>
-      <c r="E17" s="5" t="str">
+      <c r="E17" s="3" t="str">
         <v>對應 #</v>
       </c>
-      <c r="F17" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G17" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H17" s="5" t="str">
+      <c r="F17" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G17" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H17" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -11277,54 +11325,54 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="str">
+      <c r="A25" s="3" t="str">
         <v>【4】UIUX — 優先級 × 狀態分布</v>
       </c>
-      <c r="B25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G25" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H25" s="4" t="str">
+      <c r="B25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H25" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="str">
+      <c r="A26" s="3" t="str">
         <v>優先級</v>
       </c>
-      <c r="B26" s="5" t="str">
+      <c r="B26" s="3" t="str">
         <v>已修正</v>
       </c>
-      <c r="C26" s="5" t="str">
+      <c r="C26" s="3" t="str">
         <v>部分修正</v>
       </c>
-      <c r="D26" s="5" t="str">
-        <v>待處理</v>
-      </c>
-      <c r="E26" s="5" t="str">
+      <c r="D26" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="E26" s="3" t="str">
         <v>小計</v>
       </c>
-      <c r="F26" s="5" t="str">
+      <c r="F26" s="3" t="str">
         <v>完成率</v>
       </c>
-      <c r="G26" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H26" s="5" t="str">
+      <c r="G26" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H26" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -11332,13 +11380,13 @@
       <c r="A27" s="3" t="str">
         <v>高</v>
       </c>
-      <c r="B27" s="6">
+      <c r="B27" s="3">
         <v>7</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="3">
         <v>4</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="3">
         <v>6</v>
       </c>
       <c r="E27" s="3">
@@ -11358,13 +11406,13 @@
       <c r="A28" s="3" t="str">
         <v>中</v>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="3">
         <v>14</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="3">
         <v>1</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="3">
         <v>44</v>
       </c>
       <c r="E28" s="3">
@@ -11384,13 +11432,13 @@
       <c r="A29" s="3" t="str">
         <v>低</v>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="3">
         <v>18</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="3">
         <v>2</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="3">
         <v>35</v>
       </c>
       <c r="E29" s="3">
@@ -11407,54 +11455,54 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="str">
+      <c r="A31" s="3" t="str">
         <v>【5】UIUX — 各區塊問題分布</v>
       </c>
-      <c r="B31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G31" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H31" s="4" t="str">
+      <c r="B31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H31" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="str">
+      <c r="A32" s="3" t="str">
         <v>區塊</v>
       </c>
-      <c r="B32" s="5" t="str">
+      <c r="B32" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C32" s="5" t="str">
+      <c r="C32" s="3" t="str">
         <v>佔比</v>
       </c>
-      <c r="D32" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E32" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F32" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G32" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H32" s="5" t="str">
+      <c r="D32" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E32" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F32" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G32" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H32" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -11927,54 +11975,54 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="str">
+      <c r="A52" s="3" t="str">
         <v>【6】後臺優化 — 各區塊問題分布</v>
       </c>
-      <c r="B52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G52" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H52" s="4" t="str">
+      <c r="B52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H52" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="str">
+      <c r="A53" s="3" t="str">
         <v>區塊</v>
       </c>
-      <c r="B53" s="5" t="str">
+      <c r="B53" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C53" s="5" t="str">
+      <c r="C53" s="3" t="str">
         <v>佔比</v>
       </c>
-      <c r="D53" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E53" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F53" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G53" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H53" s="5" t="str">
+      <c r="D53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H53" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -12577,54 +12625,54 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="str">
+      <c r="A78" s="3" t="str">
         <v>【7】你做了什麼 — 已完成項目摘要 (依 Round 分組)</v>
       </c>
-      <c r="B78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G78" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H78" s="4" t="str">
+      <c r="B78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H78" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="str">
+      <c r="A79" s="3" t="str">
         <v>Round</v>
       </c>
-      <c r="B79" s="5" t="str">
+      <c r="B79" s="3" t="str">
         <v>日期</v>
       </c>
-      <c r="C79" s="5" t="str">
+      <c r="C79" s="3" t="str">
         <v>已修正 (綠)</v>
       </c>
-      <c r="D79" s="5" t="str">
+      <c r="D79" s="3" t="str">
         <v>部分修正 (黃)</v>
       </c>
-      <c r="E79" s="5" t="str">
+      <c r="E79" s="3" t="str">
         <v>已修正 # 清單</v>
       </c>
-      <c r="F79" s="5" t="str">
+      <c r="F79" s="3" t="str">
         <v>部分修正 # 清單</v>
       </c>
-      <c r="G79" s="5" t="str">
+      <c r="G79" s="3" t="str">
         <v>主要重點</v>
       </c>
-      <c r="H79" s="5" t="str">
+      <c r="H79" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -12635,10 +12683,10 @@
       <c r="B80" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C80" s="6">
+      <c r="C80" s="3">
         <v>24</v>
       </c>
-      <c r="D80" s="7">
+      <c r="D80" s="3">
         <v>6</v>
       </c>
       <c r="E80" s="3" t="str">
@@ -12661,10 +12709,10 @@
       <c r="B81" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C81" s="6">
+      <c r="C81" s="3">
         <v>2</v>
       </c>
-      <c r="D81" s="7">
+      <c r="D81" s="3">
         <v>0</v>
       </c>
       <c r="E81" s="3" t="str">
@@ -12687,10 +12735,10 @@
       <c r="B82" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C82" s="6">
+      <c r="C82" s="3">
         <v>6</v>
       </c>
-      <c r="D82" s="7">
+      <c r="D82" s="3">
         <v>0</v>
       </c>
       <c r="E82" s="3" t="str">
@@ -12713,10 +12761,10 @@
       <c r="B83" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C83" s="6">
+      <c r="C83" s="3">
         <v>7</v>
       </c>
-      <c r="D83" s="7">
+      <c r="D83" s="3">
         <v>1</v>
       </c>
       <c r="E83" s="3" t="str">

</xml_diff>

<commit_message>
revert(frontend): UIUX #163 移除動態島手機選單入口 — 依 Emma 反饋
Codex 在 e0c0050 加的 .menu-island（黑橢圓 + 「長穩選單」/ 橘色「導覽」標籤）
視覺上不需要，刪除後手機選單回到單純 close 按鈕 + 選單列表。

- AppHeader.vue: 刪 menu-island HTML（line 53-57）+ mobileMenuIslandLabel const + mobileMenuPageLabel computed
- _rwd_appHeader.scss: 刪 .menu-island 整段（含 __camera / __label / __page 子規則，共 52 行）
- xlsx: #163 補驗證備註標註已撤銷實作（狀態保留「已修正」避免重做）

驗證：http://localhost:3000/ 切手機 viewport 開漢堡選單，最上面只剩 close 按鈕；
桌面選單行為不變；focus 管理 / MenuToggle / NuxtLink 都不受影響。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -12540,16 +12540,16 @@
 Dev/Dev Code/iFare_Frontend/assets/style/rwd/_rwd_appHeader.scss</v>
       </c>
       <c r="M165" s="4" t="str">
-        <v>已於 mobile-menu 新增置中靈動島，顯示「長穩選單」與目前頁面名稱，並調整 safe-area、close 按鈕與 menu list 垂直間距。</v>
+        <v>2026-05-12 撤銷實作：AppHeader.vue 與 _rwd_appHeader.scss 已將 .menu-island 入口（含 __camera / __label / __page 與相關 JS computed mobileMenuPageLabel）整段移除。</v>
       </c>
       <c r="N165" s="5" t="str">
         <v>已修正</v>
       </c>
       <c r="O165" s="4" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-12</v>
       </c>
       <c r="P165" s="4" t="str">
-        <v>AppHeader.vue 新增 mobileMenuIslandLabel / mobileMenuPageLabel；_rwd_appHeader.scss 新增 menu-island 膠囊樣式、暗色毛玻璃與手機版 overlay 專用 top padding。</v>
+        <v>依使用者反饋，這個 dynamic island 視覺非必要；漢堡 toggle / close / focus 管理 / 選單列表均不受影響。</v>
       </c>
     </row>
   </sheetData>
@@ -12649,7 +12649,7 @@
         <v>65.0%</v>
       </c>
       <c r="G3" s="3" t="str">
-        <v>更新 #2/#11/#12/#13/#86/#87：第四批 i-Fare 收尾（受助篩選動畫、洽辦互動拆分、多通道分享、contact RWD 統一、result 空狀態 CTA、FAQ focus-visible 強化）</v>
+        <v>#163 動態島手機選單已依使用者反饋撤銷實作；狀態保留「已修正」並補驗證備註說明。</v>
       </c>
       <c r="H3" s="3" t="str">
         <v/>

</xml_diff>

<commit_message>
chore(tracking): 修正 sheet2 #53 重複編號誤標
sheet2 有兩條 row 編號都是 #53：
- Row 49 = 效能 / 大列表 lazy load
- Row 57 = 後台首頁 / Dashboard 重構

前一個 12b2271 commit 的 update-uiux-2026-05-12-batch.mjs 用 findRowById
找第一個 match 就 return，所以 HomeView Dashboard 重構的 note 被誤標到 Row 49
（lazy load）上，Row 57 反而沒動。

本 commit:
- Row 49 (#53 lazy load) revert 回「待處理」並清掉錯的 M/O/P
- Row 57 (#53 後台首頁 Dashboard) 補標「部分修正」+ 正確 verify note

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -3668,16 +3668,16 @@
 後端 confirm pagination</v>
       </c>
       <c r="M49" s="3" t="str">
-        <v>HomeView.vue +365 行（commit 93d1186）後台首頁整體重構。</v>
+        <v/>
       </c>
       <c r="N49" s="3" t="str">
-        <v>部分修正</v>
+        <v>待處理</v>
       </c>
       <c r="O49" s="3" t="str">
-        <v>2026-05-12</v>
+        <v/>
       </c>
       <c r="P49" s="3" t="str">
-        <v>部分修正 — Codex 大改完整 Dashboard 結構，但整合搜尋 / 總覽 / 待辦 / 快捷的完整性待 review。</v>
+        <v/>
       </c>
       <c r="Q49" s="3" t="str">
         <v>做得快</v>
@@ -4107,16 +4107,16 @@
         <v>後台 Vue 3：重寫 src/views/Index/IndexView.vue 或新增 src/views/Dashboard/DashboardView.vue + 新增 src/composables/useDashboardSearch.ts；後端需新增 API：Dashboard/GetSummary（系統概況 + 待辦摘要）+ Dashboard/Search（全站搜尋）+ Dashboard/RecentActivity（最近更新）</v>
       </c>
       <c r="M57" s="3" t="str">
-        <v>使用者明確要求「不再只是歡迎頁，是工作入口頁」。第一版可暫緩 ⑦ 數據摘要區。</v>
+        <v>HomeView.vue +365 行（commit 93d1186）後台首頁整體重構。</v>
       </c>
       <c r="N57" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O57" s="3" t="str">
-        <v/>
+        <v>2026-05-12</v>
       </c>
       <c r="P57" s="3" t="str">
-        <v>來源：2026-05-05 使用者草圖。設計重點：「整合搜尋、總覽、待辦與快捷操作的工作入口頁，讓使用者快速找到要做的事與對應功能位置」。搜尋示例：輸入「步道」應回「功能入口（頁管 &gt; 新增頁面 / 福利專欄 &gt; 新增文章）/ 相關內容（頁管 步道專區、福利專欄 親子步道介紹、最新消息 步道公告）/ 建議操作（新增步道頁面 / 查看步道文章 / 前往圖片管理）」。</v>
+        <v>部分修正 — Codex 大改完整 Dashboard 結構，但整合搜尋 / 總覽 / 待辦 / 快捷的完整性待 review。</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(page-management): PoC v2 Day2-fix — 預設 status=published + draft toast warning
Emma 完整 v2 驗證後遇到「toast 連結點過去看 Nuxt 404」狀況。
排查 server/data/dynamic-pages.json 確認自動同步已 work（4 筆 page 都寫進去了），
root cause：createDefaultPage() 預設 status='draft'，被前端 isPublishable() 擋掉。
這跟 Emma「按下新增就到前端」直覺期望衝突。

修法：
- useDynamicPages.ts:271 createDefaultPage() 預設 status: 'draft' → 'published'
  影響：新增頁面直接「已發布」，符合 PoC v2 體驗；想當草稿仍可主動切回
- AddEditView 儲存後 toast 分支：
  · status=published → successWithLink「前往前端預覽」（既有行為）
  · 其他（draft / unpublished）→ warning「頁面已暫存為草稿，前端不會顯示」

PoC md（docs/iFare_PageBuilder_前端顯示PoC_2026-05-18.md）：
- 「v2 改了什麼」段加入 createDefaultPage 預設改變說明
- demo 流程步驟 3 拿掉「狀態切已發布」（現在預設就是）
- 「PoC 範圍與限制」加一行：預設 status PoC published / 工程化 draft + 審核

既有 4 筆 draft 資料：Emma 進後台手動切「已發布」存檔即可（會自動 sync）。

xlsx：day2c script 更新 #66 驗證備註 + 備註，加註 Day2-fix。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -4632,44 +4632,44 @@
       </c>
     </row>
     <row r="69" ht="14.4" customHeight="1">
-      <c r="A69" s="2">
+      <c r="A69" s="3">
         <v>66</v>
       </c>
-      <c r="B69" s="2" t="str">
-        <v>V</v>
-      </c>
-      <c r="C69" s="2" t="str">
+      <c r="B69" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C69" s="3" t="str">
         <v>頁面管理</v>
       </c>
-      <c r="D69" s="2" t="str">
+      <c r="D69" s="3" t="str">
         <v>PageBuilder 前端顯示</v>
       </c>
-      <c r="E69" s="2" t="str">
+      <c r="E69" s="3" t="str">
         <v>新增</v>
       </c>
-      <c r="F69" s="2" t="str">
+      <c r="F69" s="3" t="str">
         <v>架構</v>
       </c>
-      <c r="G69" s="2" t="str">
+      <c r="G69" s="3" t="str">
         <v>中</v>
       </c>
-      <c r="H69" s="2" t="str">
+      <c r="H69" s="3" t="str">
         <v>PageBuilder 新增 page 完無法在前端顯示 — 前端動態路由 + 自動同步 (v2 完成)</v>
       </c>
-      <c r="I69" s="2" t="str">
+      <c r="I69" s="3" t="str">
         <v>v1 跨應用 localStorage 不共享，PoC 用手動貼 JSON 走通渲染鏈路；v2 用 Nuxt server route 當中介層自動同步，後台儲存→fire-and-forget PUT→前端 useAsyncData 讀，達成「後台按下儲存→前端重整看得到」端到端體驗</v>
       </c>
-      <c r="J69" s="2" t="str">
+      <c r="J69" s="3" t="str">
         <v>後台新建 utils/frontendSync.ts (fetch PUT 整批) + writeAll() dual write；後台 useFeedback 新增 successWithLink + AddEditView toast 加「前往前端預覽」連結；前端新建 server/utils/cors.ts + 3 個 server/api/dynamic-pages.{get,put,options}.ts 寫進 server/data/dynamic-pages.json；前端 composables/useDynamicPages.ts 改 async ($fetch) + pages/[slug].vue 改 useAsyncData + throw createError(404) 升級 SSR</v>
       </c>
-      <c r="K69" s="2" t="str">
+      <c r="K69" s="3" t="str">
         <v>iFare_Backend/src/utils/frontendSync.ts (新建); iFare_Backend/src/composables/useDynamicPages.ts (writeAll 改); iFare_Backend/src/composables/useFeedback.ts (加 successWithLink); iFare_Backend/src/views/PageManagement/PageManagement_AddEditView.vue (toast 升級); iFare_Frontend/server/utils/cors.ts (新建); iFare_Frontend/server/api/dynamic-pages.{get,put,options}.ts (新建); iFare_Frontend/server/data/.gitignore (新建); iFare_Frontend/composables/useDynamicPages.ts (改寫); iFare_Frontend/pages/[slug].vue (改 SSR)</v>
       </c>
-      <c r="L69" s="2" t="str">
+      <c r="L69" s="3" t="str">
         <v>Dev/Dev Code/iFare_Backend/src/utils/frontendSync.ts; Dev/Dev Code/iFare_Backend/src/composables/useDynamicPages.ts:180-186; Dev/Dev Code/iFare_Backend/src/composables/useFeedback.ts; Dev/Dev Code/iFare_Backend/src/views/PageManagement/PageManagement_AddEditView.vue; Dev/Dev Code/iFare_Frontend/server/utils/cors.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.get.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.put.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.options.ts; Dev/Dev Code/iFare_Frontend/composables/useDynamicPages.ts; Dev/Dev Code/iFare_Frontend/pages/[slug].vue; docs/iFare_PageBuilder_前端顯示PoC_2026-05-18.md</v>
       </c>
       <c r="M69" s="2" t="str">
-        <v>v2 完整端到端：跨應用同步 ⚠️→✅、SSR/SEO ❌→✅、404 真正回傳 ❌→✅；後台 writeAll 是所有 mutation 唯一 persist 入口，改一處 cover insert/update/remove/importJson</v>
+        <v>v2 完整端到端：跨應用同步 ⚠️→✅、SSR/SEO ❌→✅、404 真正回傳 ❌→✅；Day2-fix 把 createDefaultPage 預設 status 從 draft 改成 published，符合「按下新增就到前端」體驗；後台 writeAll 是所有 mutation 唯一 persist 入口，改一處 cover insert/update/remove/importJson</v>
       </c>
       <c r="N69" s="2" t="str">
         <v>已修正</v>
@@ -4678,7 +4678,7 @@
         <v>2026-05-18</v>
       </c>
       <c r="P69" s="2" t="str">
-        <v>dev only — prod 上線要把 Nuxt server JSON 中介層換成 .NET API（已在 frontendSync 預留 VITE_FRONTEND_SYNC_URL env var）；發布排程 worker、slug 衝突、多人協作互蓋仍未做</v>
+        <v>dev only — prod 上線要把 Nuxt server JSON 中介層換成 .NET API（已在 frontendSync 預留 VITE_FRONTEND_SYNC_URL env var）；Day2-fix toast 偵測 status=draft 改顯示 warning 提示前端不顯示；發布排程 worker、slug 衝突、多人協作互蓋、預設改回 draft + 審核工作流 仍未做</v>
       </c>
     </row>
     <row r="70" ht="14.4" customHeight="1">

</xml_diff>

<commit_message>
feat: finalize uiux and page builder fixes
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -979,8 +979,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q85"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:Q89"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="6"/>
     <col min="2" max="2" customWidth="1" width="6"/>
@@ -2122,16 +2122,16 @@
 src/views/*/DataListView.vue</v>
       </c>
       <c r="M22" s="3" t="str">
-        <v>CardSearchParam.vue +147 行（commit 93d1186）涉及搜尋條件清除等改動。</v>
+        <v>2026-05-19：補齊 CardSearchParam 清除流程；「清除全部 / 清除條件」會一次重置日期、單選、下拉、文字欄位並清空 URL query。另補 upload 與 imgManagerType query 讀寫，圖片管理重整後可保留/清除搜尋條件。backend type-check 通過。</v>
       </c>
       <c r="N22" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O22" s="3" t="str">
-        <v>2026-05-12</v>
+        <v>2026-05-19</v>
       </c>
       <c r="P22" s="3" t="str">
-        <v>部分修正 — Codex 第六輪涉及，完成度待 review。</v>
+        <v>完成本輪 review：移除日期 console.log，補 reset icon / aria-label；ImgManager 初始載入會讀取 upload/imgManagerType/word query。</v>
       </c>
       <c r="Q22" s="3" t="str">
         <v>做得快</v>
@@ -2176,16 +2176,16 @@
 src/components/CardTable.vue (L250-336)</v>
       </c>
       <c r="M23" s="3" t="str">
-        <v>誤刪風險高，尤其列表多項同時編輯時</v>
+        <v>2026-05-19：CardTable 新增 openDeleteConfirm/getDeleteTargetLabel，刪除前會依序顯示 title、question、user_name、name、account、email 或編號；DialogAlert 改為清楚標題與可換行訊息。backend type-check 通過。</v>
       </c>
       <c r="N23" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O23" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P23" s="3" t="str">
-        <v/>
+        <v>覆蓋 News、Articles、IFare Policy/QA、Collaborator、ImgManager 共用刪除流程；彈窗文案改為「確定要刪除『名稱』嗎？刪除後無法復原。」</v>
       </c>
       <c r="Q23" s="3" t="str">
         <v>不容易錯</v>
@@ -2391,16 +2391,16 @@
         <v>src/components/CardTable.vue (L4-9)</v>
       </c>
       <c r="M27" s="3" t="str">
-        <v>改善搜尋體驗，減少困惑</v>
+        <v>2026-05-19：確認 CardTable 已有表格 empty slot，無資料時顯示「目前沒有符合條件的資料」與可調整搜尋/新增內容提示。backend type-check/build 通過。</v>
       </c>
       <c r="N27" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O27" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P27" s="3" t="str">
-        <v/>
+        <v>本項為補登既有完成狀態；空狀態已套用 CardTable 共用列表。</v>
       </c>
       <c r="Q27" s="3" t="str">
         <v>看得懂</v>
@@ -2444,16 +2444,16 @@
         <v>src/components/CompDateRangePicker.vue</v>
       </c>
       <c r="M28" s="3" t="str">
-        <v>CardSearchParam.vue +147 行涉及日期選擇 / 快捷選項。</v>
+        <v>2026-05-19：CompDateRangePicker 加入 Element Plus daterange shortcuts：今天、本週、本月、最近 7 天、最近 30 天；同步設定 format/value-format，讓 URL query 與 API 搜尋維持 MM/DD/YYYY。backend type-check 通過。</v>
       </c>
       <c r="N28" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O28" s="3" t="str">
-        <v>2026-05-12</v>
+        <v>2026-05-19</v>
       </c>
       <c r="P28" s="3" t="str">
-        <v>部分修正 — Codex 第六輪涉及，完成度待 review。</v>
+        <v>日期快捷已套用所有共用搜尋日期欄位。</v>
       </c>
       <c r="Q28" s="3" t="str">
         <v>做得快</v>
@@ -2551,16 +2551,16 @@
         <v>src/components/CardTable.vue (L178-185)</v>
       </c>
       <c r="M30" s="3" t="str">
-        <v>影響大資料量列表操作</v>
+        <v>2026-05-19：CardTable pageSize watcher 改為切換每頁筆數時先回到第 1 頁，再 clamp 頁碼，避免留在不存在頁數造成空列表。backend type-check/build 通過。</v>
       </c>
       <c r="N30" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O30" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P30" s="3" t="str">
-        <v/>
+        <v>低風險共用元件修正，覆蓋所有使用 CardTable 的列表。</v>
       </c>
       <c r="Q30" s="3" t="str">
         <v>做得快</v>
@@ -2978,16 +2978,16 @@
         <v>src/views/LoginView.vue (L26-32)</v>
       </c>
       <c r="M38" s="3" t="str">
-        <v>改善登入體驗，減少忘記密碼查詢</v>
+        <v>2026-05-19：LoginView 密碼欄位監聽 CapsLock 狀態，開啟時於欄位下方顯示提示；blur 後隱藏。backend type-check/build 通過。</v>
       </c>
       <c r="N38" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O38" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P38" s="3" t="str">
-        <v/>
+        <v>不改登入流程，只補輸入輔助提示。</v>
       </c>
       <c r="Q38" s="3" t="str">
         <v>不容易錯</v>
@@ -3085,16 +3085,16 @@
         <v>src/views/NoPermission.vue</v>
       </c>
       <c r="M40" s="3" t="str">
-        <v>提升錯誤頁面的可用性，但使用頻率低</v>
+        <v>2026-05-19：NoPermission 頁改為 403 空狀態，加入說明文案、返回上一頁與回首頁按鈕，並補手機版按鈕堆疊。backend type-check/build 通過。</v>
       </c>
       <c r="N40" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O40" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P40" s="3" t="str">
-        <v/>
+        <v>不改權限邏輯，只改善無權限落地頁。</v>
       </c>
       <c r="Q40" s="3" t="str">
         <v>看得懂</v>
@@ -4919,16 +4919,16 @@
         <v>Dev/Dev Code/iFare_Backend/src/views/Analysis/Analysis_DashboardView.vue (analytics-grid / filter-bar / hero-status-grid 段 + style scoped)</v>
       </c>
       <c r="M74" s="3" t="str">
-        <v>可借用 #63 (PageManagement 編輯頁 RWD) 已驗證的斷點與技巧；本次只動 CSS，不動 chart 設定</v>
+        <v>2026-05-19：Analysis_DashboardView 只調整 CSS/RWD。補 grid 子項 min-width:0、ApexCharts 容器 max-width、filter bar 響應式堆疊、1024px 圖表改單欄、768/640/520px 細化手機斷點。backend type-check / build 通過。</v>
       </c>
       <c r="N74" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O74" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P74" s="3" t="str">
-        <v>apexcharts 對寬度變化是 reactive 的，CSS 改動後 chart 會自動 redraw 不需手動觸發</v>
+        <v>延續 PageManagement RWD 手法；不動 chart 設定與資料邏輯。</v>
       </c>
     </row>
     <row r="75" ht="14.4" customHeight="1">
@@ -5489,6 +5489,223 @@
       </c>
       <c r="P85" s="3" t="str">
         <v>建議與版本 diff / snapshot 一起規劃。</v>
+      </c>
+    </row>
+    <row r="86" ht="14.4" customHeight="1">
+      <c r="A86" s="3">
+        <v>83</v>
+      </c>
+      <c r="B86" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C86" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="D86" s="3" t="str">
+        <v>前台預覽</v>
+      </c>
+      <c r="E86" s="3" t="str">
+        <v>修復</v>
+      </c>
+      <c r="F86" s="3" t="str">
+        <v>RWD</v>
+      </c>
+      <c r="G86" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H86" s="3" t="str">
+        <v>前台預覽裝置切換未依所選版面呈現</v>
+      </c>
+      <c r="I86" s="3" t="str">
+        <v>新增/編輯頁的 PreviewPane template 使用 device-desktop/tablet/mobile class，但 CSS 寫成 .tablet/.mobile，導致選平板或手機時仍以桌機尺寸顯示。</v>
+      </c>
+      <c r="J86" s="3" t="str">
+        <v>統一 device class 命名，補桌機、平板、手機預覽寬度限制，讓預覽跟選取版面同步。</v>
+      </c>
+      <c r="K86" s="3" t="str">
+        <v>src/components/PageBuilder/PreviewPane.vue</v>
+      </c>
+      <c r="L86" s="3" t="str">
+        <v>Dev/Dev Code/iFare_Backend/src/components/PageBuilder/PreviewPane.vue</v>
+      </c>
+      <c r="M86" s="3" t="str">
+        <v>2026-05-19 驗證：backend type-check / build 通過；桌機 max 1280、平板 840、手機 390。</v>
+      </c>
+      <c r="N86" s="3" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O86" s="3" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="P86" s="3" t="str">
+        <v>修正 .device-tablet / .device-mobile CSS selector mismatch。</v>
+      </c>
+      <c r="Q86" s="3" t="str">
+        <v>不容易錯</v>
+      </c>
+    </row>
+    <row r="87" ht="14.4" customHeight="1">
+      <c r="A87" s="3">
+        <v>84</v>
+      </c>
+      <c r="B87" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C87" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="D87" s="3" t="str">
+        <v>圖片欄位 / 本機圖片</v>
+      </c>
+      <c r="E87" s="3" t="str">
+        <v>修復</v>
+      </c>
+      <c r="F87" s="3" t="str">
+        <v>互動</v>
+      </c>
+      <c r="G87" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H87" s="3" t="str">
+        <v>圖文並列圖片路徑貼入後無法顯示</v>
+      </c>
+      <c r="I87" s="3" t="str">
+        <v>使用者貼入 C:\Users\... 本機路徑時，前台瀏覽器無法讀取本機檔案；只會顯示「圖片路徑無法載入」或破圖。</v>
+      </c>
+      <c r="J87" s="3" t="str">
+        <v>新增「選擇本機圖片」上傳流程，透過 Nuxt server API 存到 dynamic-assets，圖片欄位改存 http URL；同時補上本機路徑警示。</v>
+      </c>
+      <c r="K87" s="3" t="str">
+        <v>SectionEditor.vue / dynamic-assets API / DynamicPage image resolver</v>
+      </c>
+      <c r="L87" s="3" t="str">
+        <v>Dev/Dev Code/iFare_Backend/src/components/PageBuilder/SectionEditor.vue
+Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets*.ts
+Dev/Dev Code/iFare_Frontend/utils/dynamicImage.ts
+Dev/Dev Code/iFare_Frontend/components/DynamicPage/SectionImageText.vue</v>
+      </c>
+      <c r="M87" s="3" t="str">
+        <v>支援 gif/png/jpg/jpeg/webp/svg/avif，8MB 限制；上傳成功會自動填圖片 URL 和 alt。</v>
+      </c>
+      <c r="N87" s="3" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O87" s="3" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="P87" s="3" t="str">
+        <v>新增 /api/dynamic-assets POST/GET/OPTIONS，server/data/dynamic-assets 已列入 .gitignore。</v>
+      </c>
+      <c r="Q87" s="3" t="str">
+        <v>不容易錯</v>
+      </c>
+    </row>
+    <row r="88" ht="14.4" customHeight="1">
+      <c r="A88" s="3">
+        <v>85</v>
+      </c>
+      <c r="B88" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C88" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="D88" s="3" t="str">
+        <v>儲存流程</v>
+      </c>
+      <c r="E88" s="3" t="str">
+        <v>修復</v>
+      </c>
+      <c r="F88" s="3" t="str">
+        <v>互動</v>
+      </c>
+      <c r="G88" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H88" s="3" t="str">
+        <v>更新圖片後儲存按鈕一直 loading</v>
+      </c>
+      <c r="I88" s="3" t="str">
+        <v>圖片若被舊流程存成 data:image base64，localStorage 容量可能超過配額；原儲存流程沒有完整 try/catch，saving 狀態無法恢復。</v>
+      </c>
+      <c r="J88" s="3" t="str">
+        <v>儲存前阻擋嵌入式 base64 圖片並提示改用上傳；insert/update 加 try/catch 與 afterSave，錯誤訊息可落地。</v>
+      </c>
+      <c r="K88" s="3" t="str">
+        <v>PageManagement_AddEditView.vue</v>
+      </c>
+      <c r="L88" s="3" t="str">
+        <v>Dev/Dev Code/iFare_Backend/src/views/PageManagement/PageManagement_AddEditView.vue</v>
+      </c>
+      <c r="M88" s="3" t="str">
+        <v>backend type-check 通過；QuotaExceeded / storage / page not found 會顯示對應錯誤，避免無限轉圈。</v>
+      </c>
+      <c r="N88" s="3" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O88" s="3" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="P88" s="3" t="str">
+        <v>舊 data URL 頁面需重新用「選擇本機圖片」上傳一次。</v>
+      </c>
+      <c r="Q88" s="3" t="str">
+        <v>出事能追回來</v>
+      </c>
+    </row>
+    <row r="89" ht="14.4" customHeight="1">
+      <c r="A89" s="3">
+        <v>86</v>
+      </c>
+      <c r="B89" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C89" s="3" t="str">
+        <v>前台動態頁</v>
+      </c>
+      <c r="D89" s="3" t="str">
+        <v>圖片載入</v>
+      </c>
+      <c r="E89" s="3" t="str">
+        <v>修復</v>
+      </c>
+      <c r="F89" s="3" t="str">
+        <v>資料同步</v>
+      </c>
+      <c r="G89" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H89" s="3" t="str">
+        <v>前端動態頁圖片網址被存成 IPv4:// 導致破圖</v>
+      </c>
+      <c r="I89" s="3" t="str">
+        <v>Nuxt server origin 取 x-forwarded-proto 時可能拿到 IPv4，產生 IPv4://localhost:3000/...；瀏覽器不能載入，前台只顯示破圖 alt。</v>
+      </c>
+      <c r="J89" s="3" t="str">
+        <v>server 端限制 proto 只允許 http/https；前端 image resolver 兼容修正既有 IPv4:// / IPv6:// 壞資料為 http://。</v>
+      </c>
+      <c r="K89" s="3" t="str">
+        <v>server/api/dynamic-assets.post.ts / utils/dynamicImage.ts</v>
+      </c>
+      <c r="L89" s="3" t="str">
+        <v>Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets.post.ts
+Dev/Dev Code/iFare_Frontend/utils/dynamicImage.ts
+Dev/Dev Code/iFare_Frontend/server/data/dynamic-pages.json (local)</v>
+      </c>
+      <c r="M89" s="3" t="str">
+        <v>本機資料已改為 http://localhost:3000/api/dynamic-assets/wave_pro_pro-...gif；frontend build 通過。</v>
+      </c>
+      <c r="N89" s="3" t="str">
+        <v>已修正</v>
+      </c>
+      <c r="O89" s="3" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="P89" s="3" t="str">
+        <v>若 dev server 已啟動很久，需重啟 Nuxt 讓新 server route 生效。</v>
+      </c>
+      <c r="Q89" s="3" t="str">
+        <v>不容易錯</v>
       </c>
     </row>
   </sheetData>
@@ -5503,7 +5720,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:P176"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="5.77734375"/>
@@ -13453,16 +13670,16 @@
 Dev/Dev Code/iFare_Frontend/components/**/*.vue</v>
       </c>
       <c r="M156" s="3" t="str">
-        <v>本次程式碼審查僅能確認 RWD 架構存在，仍需固定 viewport 視覺驗證。</v>
+        <v>2026-05-19：新增 docs/iFare_RWD回歸檢查清單.md，整理桌機、小桌機、平板、手機固定 viewport，以及後台/前台/部署前 smoke test 檢查項目。</v>
       </c>
       <c r="N156" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O156" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P156" s="3" t="str">
-        <v/>
+        <v>文件型 UIUX 治理項目，先建立可重複執行的回歸檢查基準。</v>
       </c>
     </row>
     <row r="157" ht="14.4" customHeight="1" xml:space="preserve">
@@ -14499,8 +14716,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H94"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H95"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="14.5546875"/>
     <col min="2" max="2" customWidth="1" width="12.5546875"/>
@@ -14572,19 +14789,19 @@
         <v>174</v>
       </c>
       <c r="C3" s="3">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D3" s="3">
         <v>19</v>
       </c>
       <c r="E3" s="3">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F3" s="3" t="str">
-        <v>70.1%</v>
+        <v>70.7%</v>
       </c>
       <c r="G3" s="3" t="str">
-        <v>2026-05-18：#167-#174 前台福利進階功能皆已完成 MVP，後續可進入後台資料結構與跨裝置同步。</v>
+        <v>2026-05-19：補完成 #154 RWD 固定 viewport 回歸檢查清單，部署前可依清單做 smoke test。</v>
       </c>
       <c r="H3" s="3" t="str">
         <v/>
@@ -14595,22 +14812,22 @@
         <v>後臺優化 (admin)</v>
       </c>
       <c r="B4" s="3">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C4" s="3">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" s="3">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F4" s="3" t="str">
-        <v>4.8%</v>
+        <v>20.7%</v>
       </c>
       <c r="G4" s="3" t="str">
-        <v>2026-05-18：已補入 i-Fare 前台進階功能對應後台支援任務 #73-#82，#80 政策健康檢查完成編輯頁 MVP。</v>
+        <v>2026-05-19：完成 #20/#21/#25/#26/#28/#36/#38/#71，以及 PageManagement / 動態頁圖片修復 #83-#86。</v>
       </c>
       <c r="H4" s="3" t="str">
         <v/>
@@ -16797,6 +17014,32 @@
         <v>future.vue 補強手機版主標換行、空狀態導引卡與上下節奏，讓頁面在未上線時也有清楚下一步</v>
       </c>
       <c r="H94" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="14.4" customHeight="1">
+      <c r="A95" s="3" t="str">
+        <v>Round 15</v>
+      </c>
+      <c r="B95" s="3" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="C95" s="3">
+        <v>13</v>
+      </c>
+      <c r="D95" s="3">
+        <v>0</v>
+      </c>
+      <c r="E95" s="3" t="str">
+        <v>後臺優化 #20, #21, #25, #26, #28, #36, #38, #71, #83, #84, #85, #86；UIUX #154</v>
+      </c>
+      <c r="F95" s="3" t="str">
+        <v>-</v>
+      </c>
+      <c r="G95" s="3" t="str">
+        <v>PageManagement 預覽與圖片修復；搜尋清除、日期快捷、刪除確認、表格空狀態、分頁重設、登入 Caps Lock、無權限頁、Analysis Dashboard RWD、RWD 回歸清單</v>
+      </c>
+      <c r="H95" s="3" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add critical project audit issues
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -77,9 +77,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -979,8 +985,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q89"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q102"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="6"/>
     <col min="2" max="2" customWidth="1" width="6"/>
@@ -2013,16 +2019,18 @@
 src/views/Collaborator/Collaborator_AddEditView.vue (L29-76)</v>
       </c>
       <c r="M20" s="3" t="str">
-        <v>2026-05-12 AddEditView.vue 加 errors ref + onSave 失敗時填 inline 紅字 + has-error class 的 el-input 紅框 + label 變紅。</v>
+        <v>Collaborator_AddEditView 與 ArticlesLazy_AddEditView 已新增 inline 必填檢查、紅框錯誤提示與儲存前阻擋；vue-tsc 已通過。</v>
       </c>
       <c r="N20" s="3" t="str">
         <v>部分修正</v>
       </c>
       <c r="O20" s="3" t="str">
-        <v>2026-05-12</v>
-      </c>
-      <c r="P20" s="3" t="str">
-        <v>只針對 title / slug / status 3 個必填欄位，進階設定（SEO / cover / tags / publishTime）尚未套同 pattern，故為部分修正。</v>
+        <v>2026-05-19</v>
+      </c>
+      <c r="P20" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">只針對 title / slug / status 3 個必填欄位，進階設定（SEO / cover / tags / publishTime）尚未套同 pattern，故為部分修正。
+2026-05-19：再套用至 Collaborator / ArticlesLazy - 再套用至 Collaborator_AddEditView 與 ArticlesLazy_AddEditView，補 inline 必填錯誤、欄位提示與儲存前阻擋；其他 AddEditView 尚未全面改為 el-form rules，維持部分修正。
+2026-05-19：新增功能建議補強 - 表單驗證建議由單頁修補升級為共用 helper / composable，統一必填、URL、圖片、儲存 loading 與錯誤提示。</v>
       </c>
       <c r="Q20" s="3" t="str">
         <v>不容易錯</v>
@@ -2068,16 +2076,16 @@
 src/views/IFare/OfficeUnit/IFareOfficeUnit_AddEditView.vue</v>
       </c>
       <c r="M21" s="3" t="str">
-        <v>使用者無法確認操作是否成功，易誤以為沒儲存</v>
+        <v>Collaborator / ArticlesLazy 儲存按鈕已新增 loading / disabled；API 失敗解除 loading 並停留，成功顯示訊息後返回。</v>
       </c>
       <c r="N21" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O21" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P21" s="3" t="str">
-        <v/>
+        <v>2026-05-19：Collaborator / ArticlesLazy 儲存回饋 - Collaborator / ArticlesLazy 儲存按鈕新增 loading/disabled，API 失敗會停留並解除 loading，成功顯示訊息後返回；全站 SaveAction 尚未統一，標部分修正。</v>
       </c>
       <c r="Q21" s="3" t="str">
         <v>看得懂</v>
@@ -2230,16 +2238,16 @@
 src/views/IFare/Policy/IFarePolicy_AddEditView.vue (L54-86)</v>
       </c>
       <c r="M24" s="3" t="str">
-        <v>減少使用者困惑，提升表單填寫速度</v>
+        <v>ArticlesLazy 新增頁已以 [] 初始化多選，政策類別載入後預設第一筆，並補 placeholder / hint。</v>
       </c>
       <c r="N24" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O24" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P24" s="3" t="str">
-        <v/>
+        <v>2026-05-19：ArticlesLazy 選單預設與 placeholder - ArticlesLazy 新增頁改以 [] 初始化多選、政策類別載入後預設第一筆並補 placeholder/hint；CompItemSelect 與其他頁尚未全域整理。</v>
       </c>
       <c r="Q24" s="3" t="str">
         <v>不容易錯</v>
@@ -2285,16 +2293,16 @@
 src/components/DialogAddEditImg.vue (L27-43)</v>
       </c>
       <c r="M25" s="3" t="str">
-        <v>防止上傳無效檔案導致後端錯誤</v>
+        <v>Collaborator / ArticlesLazy 上傳 on-change 已檢查 JPG/JPEG/PNG 與 500KB，違規檔案會移除並提示。</v>
       </c>
       <c r="N25" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O25" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P25" s="3" t="str">
-        <v/>
+        <v>2026-05-19：Collaborator / ArticlesLazy 上傳預檢 - Collaborator / ArticlesLazy on-change 新增 JPG/JPEG/PNG 與 500KB 預檢，違規檔案會移除並提示；DialogAddEditImg 尚未套用。</v>
       </c>
       <c r="Q25" s="3" t="str">
         <v>不容易錯</v>
@@ -2498,16 +2506,17 @@
 src/views/News/News_AddEditView.vue (L37-44)</v>
       </c>
       <c r="M29" s="3" t="str">
-        <v>減少使用者困惑，降低後續編輯次數</v>
+        <v>Collaborator / ArticlesLazy 已補欄位範例、上傳規格、選單提示與說明文字；vue-tsc 已通過。</v>
       </c>
       <c r="N29" s="3" t="str">
         <v>部分修正</v>
       </c>
       <c r="O29" s="3" t="str">
-        <v>2026-05-12</v>
-      </c>
-      <c r="P29" s="3" t="str">
-        <v>2026-05-12：先在 PageManagement_AddEditView 補強欄位說明與範例，包含頁面名稱用途說明、Slug 操作提示、URL 預覽、SEO 描述搜尋結果預覽。屬於單一頁面快改，整體後台尚未全面套用，故標記為部分修正。</v>
+        <v>2026-05-19</v>
+      </c>
+      <c r="P29" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">2026-05-12：先在 PageManagement_AddEditView 補強欄位說明與範例，包含頁面名稱用途說明、Slug 操作提示、URL 預覽、SEO 描述搜尋結果預覽。屬於單一頁面快改，整體後台尚未全面套用，故標記為部分修正。
+2026-05-19：Collaborator / ArticlesLazy 欄位提示 - Collaborator / ArticlesLazy 補欄位範例、上傳規格與選單操作提示；其餘 News/IFarePolicy 待後續。</v>
       </c>
       <c r="Q29" s="3" t="str">
         <v>看得懂</v>
@@ -4308,7 +4317,7 @@
         <v/>
       </c>
       <c r="P62" s="3" t="str">
-        <v/>
+        <v>2026-05-19：新增功能建議補強 - 內容健康檢查中心已被列為部署前後最值得做的新增功能；MVP 可先掃缺 SEO、缺圖、圖片過大、失效連結、動態頁區塊未填。</v>
       </c>
       <c r="Q62" s="3" t="str">
         <v>不容易錯</v>
@@ -4418,7 +4427,7 @@
         <v/>
       </c>
       <c r="P64" s="3" t="str">
-        <v/>
+        <v>2026-05-19：新增功能建議補強 - 媒體資產治理延伸為圖片庫/媒體管理功能：顯示可複製路徑、檔案大小、是否被引用、超大圖警告與過期素材。</v>
       </c>
       <c r="Q64" s="3" t="str">
         <v>做得快</v>
@@ -4668,16 +4677,16 @@
       <c r="L69" s="3" t="str">
         <v>Dev/Dev Code/iFare_Backend/src/utils/frontendSync.ts; Dev/Dev Code/iFare_Backend/src/composables/useDynamicPages.ts:180-186; Dev/Dev Code/iFare_Backend/src/composables/useFeedback.ts; Dev/Dev Code/iFare_Backend/src/views/PageManagement/PageManagement_AddEditView.vue; Dev/Dev Code/iFare_Frontend/server/utils/cors.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.get.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.put.ts; Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.options.ts; Dev/Dev Code/iFare_Frontend/composables/useDynamicPages.ts; Dev/Dev Code/iFare_Frontend/pages/[slug].vue; docs/iFare_PageBuilder_前端顯示PoC_2026-05-18.md</v>
       </c>
-      <c r="M69" s="2" t="str">
+      <c r="M69" s="3" t="str">
         <v>v2 完整端到端：跨應用同步 ⚠️→✅、SSR/SEO ❌→✅、404 真正回傳 ❌→✅；Day2-fix 把 createDefaultPage 預設 status 從 draft 改成 published，符合「按下新增就到前端」體驗；後台 writeAll 是所有 mutation 唯一 persist 入口，改一處 cover insert/update/remove/importJson</v>
       </c>
-      <c r="N69" s="2" t="str">
+      <c r="N69" s="3" t="str">
         <v>已修正</v>
       </c>
-      <c r="O69" s="2" t="str">
+      <c r="O69" s="3" t="str">
         <v>2026-05-18</v>
       </c>
-      <c r="P69" s="2" t="str">
+      <c r="P69" s="3" t="str">
         <v>dev only — prod 上線要把 Nuxt server JSON 中介層換成 .NET API（已在 frontendSync 預留 VITE_FRONTEND_SYNC_URL env var）；Day2-fix toast 偵測 status=draft 改顯示 warning 提示前端不顯示；發布排程 worker、slug 衝突、多人協作互蓋、預設改回 draft + 審核工作流 仍未做</v>
       </c>
     </row>
@@ -5544,7 +5553,7 @@
         <v>不容易錯</v>
       </c>
     </row>
-    <row r="87" ht="14.4" customHeight="1">
+    <row r="87" ht="14.4" customHeight="1" xml:space="preserve">
       <c r="A87" s="3">
         <v>84</v>
       </c>
@@ -5578,8 +5587,8 @@
       <c r="K87" s="3" t="str">
         <v>SectionEditor.vue / dynamic-assets API / DynamicPage image resolver</v>
       </c>
-      <c r="L87" s="3" t="str">
-        <v>Dev/Dev Code/iFare_Backend/src/components/PageBuilder/SectionEditor.vue
+      <c r="L87" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/components/PageBuilder/SectionEditor.vue
 Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets*.ts
 Dev/Dev Code/iFare_Frontend/utils/dynamicImage.ts
 Dev/Dev Code/iFare_Frontend/components/DynamicPage/SectionImageText.vue</v>
@@ -5653,7 +5662,7 @@
         <v>出事能追回來</v>
       </c>
     </row>
-    <row r="89" ht="14.4" customHeight="1">
+    <row r="89" ht="14.4" customHeight="1" xml:space="preserve">
       <c r="A89" s="3">
         <v>86</v>
       </c>
@@ -5687,8 +5696,8 @@
       <c r="K89" s="3" t="str">
         <v>server/api/dynamic-assets.post.ts / utils/dynamicImage.ts</v>
       </c>
-      <c r="L89" s="3" t="str">
-        <v>Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets.post.ts
+      <c r="L89" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets.post.ts
 Dev/Dev Code/iFare_Frontend/utils/dynamicImage.ts
 Dev/Dev Code/iFare_Frontend/server/data/dynamic-pages.json (local)</v>
       </c>
@@ -5706,6 +5715,712 @@
       </c>
       <c r="Q89" s="3" t="str">
         <v>不容易錯</v>
+      </c>
+    </row>
+    <row r="90" xml:space="preserve">
+      <c r="A90" s="3">
+        <v>87</v>
+      </c>
+      <c r="B90" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C90" s="3" t="str">
+        <v>後台通用</v>
+      </c>
+      <c r="D90" s="3" t="str">
+        <v>部署健康檢查</v>
+      </c>
+      <c r="E90" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F90" s="3" t="str">
+        <v>部署</v>
+      </c>
+      <c r="G90" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H90" s="3" t="str">
+        <v>部署健康檢查頁 — 遠端主機上線後可快速確認環境與服務狀態</v>
+      </c>
+      <c r="I90" s="3" t="str">
+        <v>專案準備上遠端主機，但目前缺少一個集中檢查頁確認 API URL、目前環境、登入狀態、圖片上傳路徑、必要 env 是否缺漏；部署後若設定錯誤，需要靠人工逐頁排查。</v>
+      </c>
+      <c r="J90" s="3" t="str">
+        <v>新增後台 Health Check / Deploy Check 頁：顯示前台 API URL、後台 API URL、目前 mode、必要 env、圖片上傳/讀取路徑、API ping 結果與最後檢查時間；先做 read-only，不牽 DB。</v>
+      </c>
+      <c r="K90" s="3" t="str">
+        <v>Backend admin / env / deploy</v>
+      </c>
+      <c r="L90" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/**
+Dev/Dev Code/iFare_Backend/src/router/**
+.env.example / deployment docs</v>
+      </c>
+      <c r="M90" s="3" t="str">
+        <v>新增功能建議，適合部署前先做 MVP。</v>
+      </c>
+      <c r="N90" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P90" s="3" t="str">
+        <v>2026-05-19：使用流程盤點後新增。此項可降低遠端主機部署後 API/env/圖片路徑設定錯誤的排查成本。</v>
+      </c>
+      <c r="Q90" s="3" t="str">
+        <v>部署與環境治理</v>
+      </c>
+    </row>
+    <row r="91" xml:space="preserve">
+      <c r="A91" s="3">
+        <v>88</v>
+      </c>
+      <c r="B91" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C91" s="3" t="str">
+        <v>後台通用</v>
+      </c>
+      <c r="D91" s="3" t="str">
+        <v>部署驗收</v>
+      </c>
+      <c r="E91" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F91" s="3" t="str">
+        <v>流程</v>
+      </c>
+      <c r="G91" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H91" s="3" t="str">
+        <v>部署後 Smoke Test 清單頁 — 固定驗收登入、上傳、前台顯示與 API 狀態</v>
+      </c>
+      <c r="I91" s="3" t="str">
+        <v>遠端部署後缺少固定驗收流程，容易只確認首頁能開，漏測後台登入、PageManagement、圖片上傳、前台動態頁、i-Fare 查詢與 chatbot fallback。</v>
+      </c>
+      <c r="J91" s="3" t="str">
+        <v>新增 Smoke Test 清單，可先用文件或後台 read-only checklist；列出必測項目、測試結果、測試時間與備註，作為每次部署後的驗收紀錄。</v>
+      </c>
+      <c r="K91" s="3" t="str">
+        <v>Deployment docs / Backend admin</v>
+      </c>
+      <c r="L91" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">docs/iFare_部署維運與異常處理手冊.md
+Dev/Dev Code/iFare_Backend/src/views/**</v>
+      </c>
+      <c r="M91" s="3" t="str">
+        <v>新增功能建議，部署前可先文件化，後續再做成後台頁。</v>
+      </c>
+      <c r="N91" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P91" s="3" t="str">
+        <v>2026-05-19：使用流程盤點後新增。建議先列為部署前必做項，降低遠端主機驗收漏項。</v>
+      </c>
+      <c r="Q91" s="3" t="str">
+        <v>部署與環境治理</v>
+      </c>
+    </row>
+    <row r="92" xml:space="preserve">
+      <c r="A92" s="3">
+        <v>89</v>
+      </c>
+      <c r="B92" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C92" s="3" t="str">
+        <v>共用元件</v>
+      </c>
+      <c r="D92" s="3" t="str">
+        <v>表單驗證 helper</v>
+      </c>
+      <c r="E92" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F92" s="3" t="str">
+        <v>程式碼</v>
+      </c>
+      <c r="G92" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H92" s="3" t="str">
+        <v>後台表單共用驗證規格 — 必填、URL、圖片、儲存 loading 與 API 錯誤提示集中管理</v>
+      </c>
+      <c r="I92" s="3" t="str">
+        <v>目前 Collaborator / ArticlesLazy 已先補 inline 驗證與上傳預檢，但各 AddEditView 若持續手刻，規則會分散，後續維護成本高。</v>
+      </c>
+      <c r="J92" s="3" t="str">
+        <v>建立共用 form helper / composable：required、url、image type/size、saving state、API error message formatter；先套高頻新增/編輯頁，再逐步回收重複邏輯。</v>
+      </c>
+      <c r="K92" s="3" t="str">
+        <v>Backend form components / composables</v>
+      </c>
+      <c r="L92" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/composables/**
+Dev/Dev Code/iFare_Backend/src/views/**/*AddEditView.vue
+Dev/Dev Code/iFare_Backend/src/assets/style/_card.scss</v>
+      </c>
+      <c r="M92" s="3" t="str">
+        <v>新增功能建議，承接 #18/#19/#23/#27 的共用化工作。</v>
+      </c>
+      <c r="N92" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P92" s="3" t="str">
+        <v>2026-05-19：使用流程盤點後新增。今天已在 Collaborator / ArticlesLazy 驗證模式，下一步建議抽共用 helper，避免各頁規則散落。</v>
+      </c>
+      <c r="Q92" s="3" t="str">
+        <v>共用元件與維護性</v>
+      </c>
+    </row>
+    <row r="93" xml:space="preserve">
+      <c r="A93" s="3">
+        <v>90</v>
+      </c>
+      <c r="B93" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C93" s="3" t="str">
+        <v>後台通用</v>
+      </c>
+      <c r="D93" s="3" t="str">
+        <v>維護首頁</v>
+      </c>
+      <c r="E93" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F93" s="3" t="str">
+        <v>流程</v>
+      </c>
+      <c r="G93" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H93" s="3" t="str">
+        <v>非工程維護首頁 — 用「我要做什麼」取代功能選單搜尋</v>
+      </c>
+      <c r="I93" s="3" t="str">
+        <v>後續維護者沒有程式基礎，若只靠側邊欄模組名稱，容易不知道新增頁面、編輯消息、上傳圖片、預覽前台該從哪裡開始。</v>
+      </c>
+      <c r="J93" s="3" t="str">
+        <v>新增維護首頁，使用任務型入口：我要新增頁面、我要編輯最新消息、我要上傳圖片、我要查看待處理、我要預覽前台；每個入口連到正確功能並附一句白話說明。</v>
+      </c>
+      <c r="K93" s="3" t="str">
+        <v>Backend Dashboard / PageManagement / ImgManager</v>
+      </c>
+      <c r="L93" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/HomeView.vue
+Dev/Dev Code/iFare_Backend/src/router/**</v>
+      </c>
+      <c r="M93" s="3" t="str">
+        <v>新增功能規劃，需以非工程使用者操作路徑驗證。</v>
+      </c>
+      <c r="N93" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O93" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P93" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，能降低新接手人員找功能的成本。</v>
+      </c>
+      <c r="Q93" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="94" xml:space="preserve">
+      <c r="A94" s="3">
+        <v>91</v>
+      </c>
+      <c r="B94" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C94" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="D94" s="3" t="str">
+        <v>新增頁面精靈</v>
+      </c>
+      <c r="E94" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F94" s="3" t="str">
+        <v>互動</v>
+      </c>
+      <c r="G94" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H94" s="3" t="str">
+        <v>新增頁面精靈 — 以步驟式流程完成頁面建立、預覽與發布</v>
+      </c>
+      <c r="I94" s="3" t="str">
+        <v>PageBuilder 若直接給空白編輯器，非工程使用者需要理解版面、區塊、圖片路徑與發布狀態，學習成本高。</v>
+      </c>
+      <c r="J94" s="3" t="str">
+        <v>新增 wizard：選頁面用途 → 選版型 → 填文字 → 上傳/選圖片 → 桌機/手機預覽 → 發布前檢查 → 發布。每步只顯示必要欄位。</v>
+      </c>
+      <c r="K94" s="3" t="str">
+        <v>PageManagement / PageBuilder</v>
+      </c>
+      <c r="L94" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/PageManagement/**
+Dev/Dev Code/iFare_Frontend/components/DynamicPage/**</v>
+      </c>
+      <c r="M94" s="3" t="str">
+        <v>新增功能規劃，需驗證使用者不看文件也能建立一頁。</v>
+      </c>
+      <c r="N94" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O94" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P94" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，應先支援活動頁與服務介紹頁兩種用途。</v>
+      </c>
+      <c r="Q94" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="95" xml:space="preserve">
+      <c r="A95" s="3">
+        <v>92</v>
+      </c>
+      <c r="B95" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C95" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="D95" s="3" t="str">
+        <v>頁面範本庫</v>
+      </c>
+      <c r="E95" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F95" s="3" t="str">
+        <v>效率</v>
+      </c>
+      <c r="G95" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H95" s="3" t="str">
+        <v>頁面範本庫 — 活動報名、服務介紹、公告、圖文、CTA 頁可直接套用</v>
+      </c>
+      <c r="I95" s="3" t="str">
+        <v>非工程使用者若每次從空白頁開始，容易排版不一致，也會重複思考同類頁面該放哪些區塊。</v>
+      </c>
+      <c r="J95" s="3" t="str">
+        <v>建立可選範本：活動報名頁、服務介紹頁、最新公告頁、圖文介紹頁、CTA 行動頁；套用後只需換文字、圖片與按鈕連結。</v>
+      </c>
+      <c r="K95" s="3" t="str">
+        <v>PageManagement templates</v>
+      </c>
+      <c r="L95" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/PageManagement/**
+Dev/Dev Code/iFare_Frontend/types/dynamic-page.ts</v>
+      </c>
+      <c r="M95" s="3" t="str">
+        <v>新增功能規劃，需確認範本套用後可正常預覽與儲存。</v>
+      </c>
+      <c r="N95" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O95" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P95" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，可先用前端常數範本，後續再改為後台可管理。</v>
+      </c>
+      <c r="Q95" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="96" xml:space="preserve">
+      <c r="A96" s="3">
+        <v>93</v>
+      </c>
+      <c r="B96" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C96" s="3" t="str">
+        <v>內容管理</v>
+      </c>
+      <c r="D96" s="3" t="str">
+        <v>一鍵複製</v>
+      </c>
+      <c r="E96" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F96" s="3" t="str">
+        <v>效率</v>
+      </c>
+      <c r="G96" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H96" s="3" t="str">
+        <v>一鍵複製頁面 / 文章 — 從既有內容複製後改標題與內文</v>
+      </c>
+      <c r="I96" s="3" t="str">
+        <v>維護者常會建立相似活動頁、公告或圖文頁，若每次重建，效率低且容易漏欄位。</v>
+      </c>
+      <c r="J96" s="3" t="str">
+        <v>在文章與 PageManagement 列表新增「複製」動作，複製後自動標記為草稿/未上架，標題加「複本」，slug/網址需重新確認，避免覆蓋原頁。</v>
+      </c>
+      <c r="K96" s="3" t="str">
+        <v>PageManagement / News / Articles</v>
+      </c>
+      <c r="L96" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/PageManagement/**
+Dev/Dev Code/iFare_Backend/src/views/News/**
+Dev/Dev Code/iFare_Backend/src/views/Articles/**</v>
+      </c>
+      <c r="M96" s="3" t="str">
+        <v>新增功能規劃，需驗證複製內容不會共用原 slug 或發布狀態。</v>
+      </c>
+      <c r="N96" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O96" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P96" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，適合活動頁與公告維護。</v>
+      </c>
+      <c r="Q96" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="97" xml:space="preserve">
+      <c r="A97" s="3">
+        <v>94</v>
+      </c>
+      <c r="B97" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C97" s="3" t="str">
+        <v>內容管理</v>
+      </c>
+      <c r="D97" s="3" t="str">
+        <v>內容完整度</v>
+      </c>
+      <c r="E97" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F97" s="3" t="str">
+        <v>提示</v>
+      </c>
+      <c r="G97" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H97" s="3" t="str">
+        <v>內容完整度提示 — 編輯時即時顯示缺圖片、缺 SEO、缺 CTA 與未預覽</v>
+      </c>
+      <c r="I97" s="3" t="str">
+        <v>非工程使用者不一定知道哪些欄位會影響前台呈現、SEO 或發布品質，容易儲存後才發現缺圖、缺按鈕或手機版跑版。</v>
+      </c>
+      <c r="J97" s="3" t="str">
+        <v>在編輯頁側欄顯示完成度分數與待補項目：標題、描述、圖片、圖片替代文字、按鈕連結、SEO、上架狀態、手機預覽。</v>
+      </c>
+      <c r="K97" s="3" t="str">
+        <v>PageManagement / News / Articles / SEO fields</v>
+      </c>
+      <c r="L97" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/**/*AddEditView.vue
+Dev/Dev Code/iFare_Backend/src/views/PageManagement/**</v>
+      </c>
+      <c r="M97" s="3" t="str">
+        <v>新增功能規劃，需驗證提示項目能在儲存前即時更新。</v>
+      </c>
+      <c r="N97" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O97" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P97" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。能把內容健康檢查從事後掃描提前到編輯當下。</v>
+      </c>
+      <c r="Q97" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="98" xml:space="preserve">
+      <c r="A98" s="3">
+        <v>95</v>
+      </c>
+      <c r="B98" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C98" s="3" t="str">
+        <v>圖片管理</v>
+      </c>
+      <c r="D98" s="3" t="str">
+        <v>圖片庫 / 媒體中心</v>
+      </c>
+      <c r="E98" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F98" s="3" t="str">
+        <v>效率</v>
+      </c>
+      <c r="G98" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H98" s="3" t="str">
+        <v>非工程圖片庫 — 上傳、預覽、複製路徑、套用到頁面一次完成</v>
+      </c>
+      <c r="I98" s="3" t="str">
+        <v>維護者不應手打圖片路徑；目前圖片路徑、預覽與前台載入曾出現問題，若沒有圖片庫，後續仍會反覆踩雷。</v>
+      </c>
+      <c r="J98" s="3" t="str">
+        <v>建立圖片庫：上傳圖片、看預覽、顯示檔案大小/尺寸、複製可用路徑、選取並套用到頁面欄位，超過建議大小時提醒壓縮。</v>
+      </c>
+      <c r="K98" s="3" t="str">
+        <v>ImgManager / PageManagement image fields</v>
+      </c>
+      <c r="L98" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/ImgManager/**
+Dev/Dev Code/iFare_Backend/src/views/PageManagement/**
+Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets.post.ts</v>
+      </c>
+      <c r="M98" s="3" t="str">
+        <v>新增功能規劃，需驗證上傳後可直接被前台載入。</v>
+      </c>
+      <c r="N98" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O98" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P98" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，承接媒體資產治理但更偏日常維護操作。</v>
+      </c>
+      <c r="Q98" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
+      <c r="A99" s="3">
+        <v>96</v>
+      </c>
+      <c r="B99" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C99" s="3" t="str">
+        <v>共用元件</v>
+      </c>
+      <c r="D99" s="3" t="str">
+        <v>站內連結選擇器</v>
+      </c>
+      <c r="E99" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F99" s="3" t="str">
+        <v>防呆</v>
+      </c>
+      <c r="G99" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H99" s="3" t="str">
+        <v>站內連結選擇器 — 按鈕連結改用選頁面，不讓維護者手打網址</v>
+      </c>
+      <c r="I99" s="3" t="str">
+        <v>非工程使用者手打 /xxx 或外部網址時容易打錯，造成前台 CTA 404 或導錯頁。</v>
+      </c>
+      <c r="J99" s="3" t="str">
+        <v>建立 LinkPicker：可選最新消息、動態頁、i-Fare、公益夥伴、外部連結；選站內項目自動帶入 URL，外部連結檢查 https:// 格式。</v>
+      </c>
+      <c r="K99" s="3" t="str">
+        <v>PageManagement CTA / News / Articles links</v>
+      </c>
+      <c r="L99" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/components/**
+Dev/Dev Code/iFare_Backend/src/views/PageManagement/**</v>
+      </c>
+      <c r="M99" s="3" t="str">
+        <v>新增功能規劃，需驗證內部連結能正確導到前台路由。</v>
+      </c>
+      <c r="N99" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O99" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P99" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。能大幅降低壞連結與手動輸入錯誤。</v>
+      </c>
+      <c r="Q99" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="100" xml:space="preserve">
+      <c r="A100" s="3">
+        <v>97</v>
+      </c>
+      <c r="B100" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C100" s="3" t="str">
+        <v>發布流程</v>
+      </c>
+      <c r="D100" s="3" t="str">
+        <v>發布前檢查清單</v>
+      </c>
+      <c r="E100" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F100" s="3" t="str">
+        <v>防呆</v>
+      </c>
+      <c r="G100" s="3" t="str">
+        <v>高</v>
+      </c>
+      <c r="H100" s="3" t="str">
+        <v>發布前檢查清單 — 發布前確認手機預覽、SEO、圖片、連結與上架狀態</v>
+      </c>
+      <c r="I100" s="3" t="str">
+        <v>非工程維護者發布前需要明確 checklist，否則容易忘記手機預覽、SEO、圖片載入、按鈕連結與上架狀態。</v>
+      </c>
+      <c r="J100" s="3" t="str">
+        <v>點擊發布時顯示 checklist modal：已預覽桌機/手機、SEO 已填、圖片正常、CTA 連結可用、上架時間正確；高風險項未通過時提示但可依權限決定是否阻擋。</v>
+      </c>
+      <c r="K100" s="3" t="str">
+        <v>PageManagement / publish flow</v>
+      </c>
+      <c r="L100" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/PageManagement/**
+Dev/Dev Code/iFare_Backend/src/components/**</v>
+      </c>
+      <c r="M100" s="3" t="str">
+        <v>新增功能規劃，需驗證發布前可擋下缺圖片/缺連結等常見問題。</v>
+      </c>
+      <c r="N100" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O100" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P100" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，適合部署前後降低發布錯誤。</v>
+      </c>
+      <c r="Q100" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="101" xml:space="preserve">
+      <c r="A101" s="3">
+        <v>98</v>
+      </c>
+      <c r="B101" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C101" s="3" t="str">
+        <v>後台通用</v>
+      </c>
+      <c r="D101" s="3" t="str">
+        <v>欄位白話化</v>
+      </c>
+      <c r="E101" s="3" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F101" s="3" t="str">
+        <v>文案</v>
+      </c>
+      <c r="G101" s="3" t="str">
+        <v>中</v>
+      </c>
+      <c r="H101" s="3" t="str">
+        <v>欄位白話化與範例 — 將 slug、meta、image path 改成維護者看得懂的用語</v>
+      </c>
+      <c r="I101" s="3" t="str">
+        <v>後台若使用工程術語，沒有程式基礎的維護者會不確定欄位用途，容易亂填或跳過。</v>
+      </c>
+      <c r="J101" s="3" t="str">
+        <v>建立欄位命名規範：slug 改「頁面網址」、meta description 改「搜尋結果描述」、image path 改「圖片網址/圖片路徑」；每個欄位補一句用途和範例。</v>
+      </c>
+      <c r="K101" s="3" t="str">
+        <v>Backend forms / PageManagement / SEO fields</v>
+      </c>
+      <c r="L101" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/**/*AddEditView.vue
+Dev/Dev Code/iFare_Backend/src/views/PageManagement/**</v>
+      </c>
+      <c r="M101" s="3" t="str">
+        <v>新增功能規劃，需以維護者能否理解欄位用途驗證。</v>
+      </c>
+      <c r="N101" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O101" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P101" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。可與表單驗證 helper、欄位提示一起逐頁套用。</v>
+      </c>
+      <c r="Q101" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
+      </c>
+    </row>
+    <row r="102" xml:space="preserve">
+      <c r="A102" s="3">
+        <v>99</v>
+      </c>
+      <c r="B102" s="3" t="str">
+        <v>V</v>
+      </c>
+      <c r="C102" s="3" t="str">
+        <v>後台通用</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <v>操作提示</v>
+      </c>
+      <c r="E102" s="3" t="str">
+        <v>新增</v>
+      </c>
+      <c r="F102" s="3" t="str">
+        <v>教學</v>
+      </c>
+      <c r="G102" s="3" t="str">
+        <v>中</v>
+      </c>
+      <c r="H102" s="3" t="str">
+        <v>簡易說明與操作提示 — 每個主要頁面只放短句提醒下一步</v>
+      </c>
+      <c r="I102" s="3" t="str">
+        <v>非工程維護者不會想看完整技術文件，若頁面沒有短提示，容易不知道修改後是否要預覽、發布或等待同步。</v>
+      </c>
+      <c r="J102" s="3" t="str">
+        <v>在主要後台頁加入 1-2 句短提示：這頁用來做什麼、修改後下一步是預覽或發布、哪些欄位會影響前台；避免長篇技術說明。</v>
+      </c>
+      <c r="K102" s="3" t="str">
+        <v>Backend views / help text</v>
+      </c>
+      <c r="L102" s="3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Backend/src/views/**
+Dev/Dev Code/iFare_Backend/src/components/**</v>
+      </c>
+      <c r="M102" s="3" t="str">
+        <v>新增功能規劃，需確認提示不干擾操作且能降低詢問成本。</v>
+      </c>
+      <c r="N102" s="3" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O102" s="3" t="str">
+        <v/>
+      </c>
+      <c r="P102" s="3" t="str">
+        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。適合搭配維護首頁與新增頁面精靈。</v>
+      </c>
+      <c r="Q102" s="3" t="str">
+        <v>非工程人員網站維護模式</v>
       </c>
     </row>
   </sheetData>
@@ -5714,14 +6429,14 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q102"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P176"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P184"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="5.77734375"/>
     <col min="2" max="2" customWidth="1" width="5.77734375"/>
@@ -13367,16 +14082,16 @@
 Dev/Dev Code/iFare_Frontend/assets/style/**/*.scss</v>
       </c>
       <c r="M150" s="3" t="str">
-        <v>build 輸出與檔案大小排序皆顯示首頁圖片偏大。</v>
+        <v>已產生 Index-Img-0~4.jpg 並切換 _icon.scss 首頁背景引用；dynamicImage eager import 已排除首頁舊 PNG 與 Index-border.png；前台 build 輸出不再列出這批大型 PNG。</v>
       </c>
       <c r="N150" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O150" s="3" t="str">
-        <v/>
+        <v>2026-05-19</v>
       </c>
       <c r="P150" s="3" t="str">
-        <v/>
+        <v>2026-05-19：首頁 Hero 圖片壓縮 - 首頁 Hero 首屏圖片完成 JPG 壓縮與 CSS 切換，並排除 dynamicImage 對首頁舊 PNG / Index-border.png 的 eager 打包；後續可再補 WebP/AVIF 與 preload/lazyload。</v>
       </c>
     </row>
     <row r="151" ht="14.4" customHeight="1">
@@ -14702,6 +15417,430 @@
       </c>
       <c r="P176" s="3" t="str">
         <v>2026-05-18 MVP：新增 useDocumentChecklist，詳情頁把 Evidence 解析成可勾選文件清單。正式版仍需後台結構化文件資料。</v>
+      </c>
+    </row>
+    <row r="177" xml:space="preserve">
+      <c r="A177" s="4">
+        <v>175</v>
+      </c>
+      <c r="B177" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C177" s="4" t="str">
+        <v>前台 Nuxt Server API</v>
+      </c>
+      <c r="D177" s="4" t="str">
+        <v>Dynamic Pages / Assets</v>
+      </c>
+      <c r="E177" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F177" s="4" t="str">
+        <v>資安</v>
+      </c>
+      <c r="G177" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H177" s="4" t="str">
+        <v>公開 API 可無驗證覆寫頁面資料與上傳檔案</v>
+      </c>
+      <c r="I177" s="4" t="str">
+        <v>dynamic-pages.put 與 dynamic-assets.post 可直接寫入檔案，CORS 允許 *，未看到後端驗證、容量限制或檔案型別安全處理；外部請求可能竄改頁面內容或累積惡意檔案。</v>
+      </c>
+      <c r="J177" s="4" t="str">
+        <v>立即補 server-side 權限驗證或部署密鑰；限制 CORS 來源；production 關閉 PoC 寫入端點；限制檔案大小與 MIME；SVG 改轉檔或消毒後再提供。</v>
+      </c>
+      <c r="K177" s="4" t="str">
+        <v>Nuxt API、Dynamic Pages、Dynamic Assets</v>
+      </c>
+      <c r="L177" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Frontend/server/api/dynamic-pages.put.ts
+Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets.post.ts
+Dev/Dev Code/iFare_Frontend/server/utils/cors.ts
+Dev/Dev Code/iFare_Frontend/server/api/dynamic-assets/[name].get.ts</v>
+      </c>
+      <c r="M177" s="4" t="str">
+        <v>已讀程式碼：PUT/POST 端點直接 writeFile；CORS 回應 Access-Control-Allow-Origin: *。</v>
+      </c>
+      <c r="N177" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O177" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P177" s="4" t="str">
+        <v>立即處理；屬內容竄改與檔案上傳風險。</v>
+      </c>
+    </row>
+    <row r="178" xml:space="preserve">
+      <c r="A178" s="4">
+        <v>176</v>
+      </c>
+      <c r="B178" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C178" s="4" t="str">
+        <v>後台 API / 帳號</v>
+      </c>
+      <c r="D178" s="4" t="str">
+        <v>密碼管理</v>
+      </c>
+      <c r="E178" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F178" s="4" t="str">
+        <v>資安</v>
+      </c>
+      <c r="G178" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H178" s="4" t="str">
+        <v>後台密碼以明文儲存、比對並可回傳到前端</v>
+      </c>
+      <c r="I178" s="4" t="str">
+        <v>SysUser.Password 為字串欄位，登入以 p.Password == pwd 比對；帳號清單與明細 DTO 也帶出 pwd，前端帳號管理頁可讀寫密碼。資料庫或 API 一旦外洩會直接暴露所有後台密碼。</v>
+      </c>
+      <c r="J178" s="4" t="str">
+        <v>導入 PasswordHasher/BCrypt/Argon2；新增密碼雜湊 migration 與強制重設流程；停止回傳 pwd；新增密碼變更專用 API；清除前端密碼欄位與相關 log。</v>
+      </c>
+      <c r="K178" s="4" t="str">
+        <v>後台帳號、登入、密碼欄位</v>
+      </c>
+      <c r="L178" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_WebApi/iFare.WebApi/Models/DBModel/SysUser.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/AuthTaskManager.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/MainTaskManager.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/PersonalTaskManager.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/AccountTaskManager.cs
+Dev/Dev Code/iFare_Admin/src/views/Account/Account_ItemDetailView.vue
+Dev/Dev Code/iFare_Admin/src/views/Account/Account_AddEditView.vue</v>
+      </c>
+      <c r="M178" s="4" t="str">
+        <v>已讀程式碼：登入直接比對明文密碼，帳號 DTO/前端欄位使用 pwd。</v>
+      </c>
+      <c r="N178" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O178" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P178" s="4" t="str">
+        <v>立即處理；需搭配資料 migration 與使用者重設密碼。</v>
+      </c>
+    </row>
+    <row r="179" xml:space="preserve">
+      <c r="A179" s="4">
+        <v>177</v>
+      </c>
+      <c r="B179" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C179" s="4" t="str">
+        <v>後台 API</v>
+      </c>
+      <c r="D179" s="4" t="str">
+        <v>權限控管</v>
+      </c>
+      <c r="E179" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F179" s="4" t="str">
+        <v>權限</v>
+      </c>
+      <c r="G179" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H179" s="4" t="str">
+        <v>多數新增/修改/刪除 API 只要求登入，未檢查角色或功能權限</v>
+      </c>
+      <c r="I179" s="4" t="str">
+        <v>JwtAuth policy 僅 RequireAuthenticatedUser，多數 AppService 的 POST/PUT/DELETE 只有 [Authorize]；目前僅 AccountAppService 看到 IsEditorCheckerFilter。任一有效 token 可能呼叫不該使用的管理 API。</v>
+      </c>
+      <c r="J179" s="4" t="str">
+        <v>把 Editor/Admin 權限檢查下沉到 API policy/filter；所有 mutation endpoint 補角色或功能授權；前端選單權限僅作 UI 控制，不可取代 API 授權；補授權測試。</v>
+      </c>
+      <c r="K179" s="4" t="str">
+        <v>後台 API、JWT、角色權限</v>
+      </c>
+      <c r="L179" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_WebApi/iFare.WebApi/Program/AuthConfigurer.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/Controllers/AppService/*.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/Controllers/AppService/AccountAppService.cs</v>
+      </c>
+      <c r="M179" s="4" t="str">
+        <v>已讀程式碼：JwtAuth policy 只檢查登入狀態，多數 AppService mutation 未套角色 filter。</v>
+      </c>
+      <c r="N179" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O179" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P179" s="4" t="str">
+        <v>立即處理；避免低權限帳號操作管理功能。</v>
+      </c>
+    </row>
+    <row r="180" xml:space="preserve">
+      <c r="A180" s="4">
+        <v>178</v>
+      </c>
+      <c r="B180" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C180" s="4" t="str">
+        <v>後台 API</v>
+      </c>
+      <c r="D180" s="4" t="str">
+        <v>登入 / 停用帳號</v>
+      </c>
+      <c r="E180" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F180" s="4" t="str">
+        <v>資安</v>
+      </c>
+      <c r="G180" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H180" s="4" t="str">
+        <v>停用帳號仍可先取得 JWT</v>
+      </c>
+      <c r="I180" s="4" t="str">
+        <v>TokenAuthController.Authenticate 只依帳密取得使用者並簽發 token；State 停用檢查出現在後續 LoginCheck 流程。攻擊者可直接呼叫 Authenticate 取得停用帳號的 JWT。</v>
+      </c>
+      <c r="J180" s="4" t="str">
+        <v>在 Authenticate 階段檢查帳號 State/停用狀態；停用或改密碼時撤銷既有 token；JWT claims 加 security stamp 或版本號並於 API 驗證。</v>
+      </c>
+      <c r="K180" s="4" t="str">
+        <v>登入、JWT、帳號停用</v>
+      </c>
+      <c r="L180" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_WebApi/iFare.WebApi/Controllers/TokenAuthController.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/AuthTaskManager.cs
+Dev/Dev Code/iFare_WebApi/iFare.WebApi/TaskManager/MainTaskManager.cs</v>
+      </c>
+      <c r="M180" s="4" t="str">
+        <v>已讀程式碼：Authenticate 呼叫 GetAuthUser 後即產生 token，GetAuthUser 未過濾停用狀態。</v>
+      </c>
+      <c r="N180" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O180" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P180" s="4" t="str">
+        <v>立即處理；與權限控管問題會互相放大風險。</v>
+      </c>
+    </row>
+    <row r="181" xml:space="preserve">
+      <c r="A181" s="4">
+        <v>179</v>
+      </c>
+      <c r="B181" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C181" s="4" t="str">
+        <v>設定 / 部署</v>
+      </c>
+      <c r="D181" s="4" t="str">
+        <v>JWT Secret</v>
+      </c>
+      <c r="E181" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F181" s="4" t="str">
+        <v>資安</v>
+      </c>
+      <c r="G181" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H181" s="4" t="str">
+        <v>JWT SecurityKey 寫在版控設定檔與發佈產物</v>
+      </c>
+      <c r="I181" s="4" t="str">
+        <v>appsettings.json 內含固定 SecurityKey，且 Dev/Prd 版本皆在專案內可讀。若 repository 或發佈包外洩，攻擊者可偽造 JWT。</v>
+      </c>
+      <c r="J181" s="4" t="str">
+        <v>改用環境變數、Secret Manager 或部署平台 secret；立即旋轉正式 JWT key；清查歷史外洩範圍；避免把含 secret 的 appsettings 或發佈產物提交進版控。</v>
+      </c>
+      <c r="K181" s="4" t="str">
+        <v>JWT、appsettings、部署設定</v>
+      </c>
+      <c r="L181" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_WebApi/iFare.WebApi/appsettings.json
+Prd/Prd Code/iFare_WebApi/appsettings.json</v>
+      </c>
+      <c r="M181" s="4" t="str">
+        <v>已讀設定檔：JwtBearer.SecurityKey 直接出現在 tracked appsettings.json。</v>
+      </c>
+      <c r="N181" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O181" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P181" s="4" t="str">
+        <v>立即處理；需同步更新部署環境與 token 失效策略。</v>
+      </c>
+    </row>
+    <row r="182" xml:space="preserve">
+      <c r="A182" s="4">
+        <v>180</v>
+      </c>
+      <c r="B182" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C182" s="4" t="str">
+        <v>後台前端</v>
+      </c>
+      <c r="D182" s="4" t="str">
+        <v>Token / XSS</v>
+      </c>
+      <c r="E182" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F182" s="4" t="str">
+        <v>資安</v>
+      </c>
+      <c r="G182" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H182" s="4" t="str">
+        <v>後台 token 存 localStorage 且有未消毒 v-html，XSS 後可竊取 token</v>
+      </c>
+      <c r="I182" s="4" t="str">
+        <v>Pinia persist 會把登入資訊保存到瀏覽器儲存區；LoginView 與 WebAPI 有敏感資料/回應 log；多個後台內容頁直接 v-html 顯示 CMS HTML。若內容或第三方腳本被植入 XSS，可讀取 token 並呼叫管理 API。</v>
+      </c>
+      <c r="J182" s="4" t="str">
+        <v>移除 token 與 API response console log；v-html 顯示前使用 DOMPurify 等白名單消毒；限制 TinyMCE 可輸入的危險屬性與 script；評估改短效 token/httpOnly cookie 或至少縮短保存時間。</v>
+      </c>
+      <c r="K182" s="4" t="str">
+        <v>後台登入、localStorage、v-html、TinyMCE</v>
+      </c>
+      <c r="L182" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Admin/src/stores/user.ts
+Dev/Dev Code/iFare_Admin/src/views/LoginView.vue
+Dev/Dev Code/iFare_Admin/src/plugins/WebAPI.ts
+Dev/Dev Code/iFare_Admin/src/views/**/**/*View.vue</v>
+      </c>
+      <c r="M182" s="4" t="str">
+        <v>已讀程式碼：user store 使用 persist，LoginView 印出 token，WebAPI 印出 response，多處 detail view 直接 v-html。</v>
+      </c>
+      <c r="N182" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O182" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P182" s="4" t="str">
+        <v>立即處理；與 API 權限不足會形成高風險攻擊鏈。</v>
+      </c>
+    </row>
+    <row r="183" xml:space="preserve">
+      <c r="A183" s="4">
+        <v>181</v>
+      </c>
+      <c r="B183" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C183" s="4" t="str">
+        <v>環境 / API 串接</v>
+      </c>
+      <c r="D183" s="4" t="str">
+        <v>URL 設定</v>
+      </c>
+      <c r="E183" s="4" t="str">
+        <v>修正</v>
+      </c>
+      <c r="F183" s="4" t="str">
+        <v>部署</v>
+      </c>
+      <c r="G183" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H183" s="4" t="str">
+        <v>API 與同步 URL 硬寫，開發可能打正式站、正式同步可能失效</v>
+      </c>
+      <c r="I183" s="4" t="str">
+        <v>後台 AjaxRef 固定指向正式 API URL；前台 PageBuilder 同步與上傳預設 localhost:3000。不同環境 build 時容易誤打正式資料或讓正式同步流程失效。</v>
+      </c>
+      <c r="J183" s="4" t="str">
+        <v>所有 base URL 改由 .env / runtime config / 部署變數注入；建立 dev/stage/prod 設定；build 或 deploy 時檢查必填環境變數，避免 fallback 到正式站或 localhost。</v>
+      </c>
+      <c r="K183" s="4" t="str">
+        <v>API base URL、PageBuilder、部署環境</v>
+      </c>
+      <c r="L183" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dev/Dev Code/iFare_Admin/src/plugins/AjaxRef.ts
+Dev/Dev Code/iFare_Frontend/components/PageBuilder.vue
+Dev/Dev Code/iFare_Frontend/utils/pageBuilderStorage.ts
+Dev/Dev Code/iFare_Frontend/utils/pageBuilderApi.ts</v>
+      </c>
+      <c r="M183" s="4" t="str">
+        <v>已讀程式碼：後台 API_HOST 指向正式站，前台同步/upload API 預設 localhost:3000。</v>
+      </c>
+      <c r="N183" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O183" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P183" s="4" t="str">
+        <v>立即處理；避免資料誤寫與部署後功能不可用。</v>
+      </c>
+    </row>
+    <row r="184" xml:space="preserve">
+      <c r="A184" s="4">
+        <v>182</v>
+      </c>
+      <c r="B184" s="4" t="str">
+        <v>V</v>
+      </c>
+      <c r="C184" s="4" t="str">
+        <v>工程流程</v>
+      </c>
+      <c r="D184" s="4" t="str">
+        <v>CI / 測試 / Repo</v>
+      </c>
+      <c r="E184" s="4" t="str">
+        <v>提升</v>
+      </c>
+      <c r="F184" s="4" t="str">
+        <v>品質</v>
+      </c>
+      <c r="G184" s="4" t="str">
+        <v>高</v>
+      </c>
+      <c r="H184" s="4" t="str">
+        <v>缺 CI 與測試覆蓋，且 repo 追蹤大量發佈產物</v>
+      </c>
+      <c r="I184" s="4" t="str">
+        <v>專案未看到 CI workflow；Vitest 目前找不到測試；本機也缺 dotnet CLI 導致 C# build 未能驗證；repo 內追蹤大量 Prd/Dev binary、DLL、PDB、EXE 與發佈輸出，會提高審查與部署風險。</v>
+      </c>
+      <c r="J184" s="4" t="str">
+        <v>新增 CI：前後台 npm build/type-check/audit、dotnet build/test；建立最小 API auth/permission/security tests；清理或移出發佈產物，改由 release artifact 或部署流程產生。</v>
+      </c>
+      <c r="K184" s="4" t="str">
+        <v>CI、測試、版控清理</v>
+      </c>
+      <c r="L184" s="4" t="str" xml:space="preserve">
+        <v xml:space="preserve">.github/workflows
+Dev/Dev Code/iFare_Admin
+Dev/Dev Code/iFare_Frontend
+Dev/Dev Code/iFare_WebApi
+Prd/Prd Code</v>
+      </c>
+      <c r="M184" s="4" t="str">
+        <v>已執行盤點：npm build 可過；npm audit 無 high/critical；Vitest 無測試；dotnet 指令不存在，C# build 未驗證。</v>
+      </c>
+      <c r="N184" s="4" t="str">
+        <v>待處理</v>
+      </c>
+      <c r="O184" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P184" s="4" t="str">
+        <v>高優先級流程問題；會降低上述風險修復的可驗證性。</v>
       </c>
     </row>
   </sheetData>
@@ -14710,14 +15849,14 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P176"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P184"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H101"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="14.5546875"/>
     <col min="2" max="2" customWidth="1" width="12.5546875"/>
@@ -14729,124 +15868,124 @@
     <col min="8" max="8" customWidth="1" width="14.5546875"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.4" customHeight="1">
-      <c r="A1" s="3" t="str">
+    <row r="1">
+      <c r="A1" s="5" t="str">
         <v>【1】整體進度</v>
       </c>
-      <c r="B1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G1" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H1" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="2" ht="14.4" customHeight="1">
-      <c r="A2" s="3" t="str">
+      <c r="B1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G1" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H1" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="str">
         <v>Sheet 名稱</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="6" t="str">
         <v>總計</v>
       </c>
-      <c r="C2" s="3" t="str">
+      <c r="C2" s="6" t="str">
         <v>已修正</v>
       </c>
-      <c r="D2" s="3" t="str">
+      <c r="D2" s="6" t="str">
         <v>部分修正</v>
       </c>
-      <c r="E2" s="3" t="str">
+      <c r="E2" s="6" t="str">
         <v>待處理</v>
       </c>
-      <c r="F2" s="3" t="str">
+      <c r="F2" s="6" t="str">
         <v>完成率</v>
       </c>
-      <c r="G2" s="3" t="str">
+      <c r="G2" s="6" t="str">
         <v>備註</v>
       </c>
-      <c r="H2" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3" ht="14.4" customHeight="1">
+      <c r="H2" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="3" t="str">
         <v>UIUX問題追蹤清單 (前台)</v>
       </c>
       <c r="B3" s="3">
         <v>174</v>
       </c>
-      <c r="C3" s="3">
-        <v>123</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="7">
+        <v>124</v>
+      </c>
+      <c r="D3" s="8">
         <v>19</v>
       </c>
-      <c r="E3" s="3">
-        <v>32</v>
+      <c r="E3" s="9">
+        <v>31</v>
       </c>
       <c r="F3" s="3" t="str">
-        <v>70.7%</v>
+        <v>71.3%</v>
       </c>
       <c r="G3" s="3" t="str">
-        <v>2026-05-19：補完成 #154 RWD 固定 viewport 回歸檢查清單，部署前可依清單做 smoke test。</v>
+        <v>已歷經 Round 1-4 改版</v>
       </c>
       <c r="H3" s="3" t="str">
         <v/>
       </c>
     </row>
-    <row r="4" ht="14.4" customHeight="1">
+    <row r="4">
       <c r="A4" s="3" t="str">
         <v>後臺優化 (admin)</v>
       </c>
       <c r="B4" s="3">
-        <v>87</v>
-      </c>
-      <c r="C4" s="3">
+        <v>100</v>
+      </c>
+      <c r="C4" s="7">
         <v>18</v>
       </c>
-      <c r="D4" s="3">
-        <v>13</v>
-      </c>
-      <c r="E4" s="3">
-        <v>56</v>
+      <c r="D4" s="8">
+        <v>16</v>
+      </c>
+      <c r="E4" s="9">
+        <v>66</v>
       </c>
       <c r="F4" s="3" t="str">
-        <v>20.7%</v>
+        <v>18.0%</v>
       </c>
       <c r="G4" s="3" t="str">
-        <v>2026-05-19：完成 #20/#21/#25/#26/#28/#36/#38/#71，以及 PageManagement / 動態頁圖片修復 #83-#86。</v>
+        <v>含後台優化規劃與進階功能建議</v>
       </c>
       <c r="H4" s="3" t="str">
         <v/>
       </c>
     </row>
-    <row r="5" ht="14.4" customHeight="1">
+    <row r="5">
       <c r="A5" s="3" t="str">
         <v>PoC研究</v>
       </c>
       <c r="B5" s="3">
         <v>13</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="8">
         <v>0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="9">
         <v>13</v>
       </c>
       <c r="F5" s="3" t="str">
@@ -14859,59 +15998,59 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="14.4" customHeight="1">
-      <c r="A7" s="3" t="str">
+    <row r="7">
+      <c r="A7" s="5" t="str">
         <v>【2】Round 時間軸 — 每輪做了什麼</v>
       </c>
-      <c r="B7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="14.4" customHeight="1">
-      <c r="A8" s="3" t="str">
+      <c r="B7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="str">
         <v>Round</v>
       </c>
-      <c r="B8" s="3" t="str">
+      <c r="B8" s="6" t="str">
         <v>日期</v>
       </c>
-      <c r="C8" s="3" t="str">
+      <c r="C8" s="6" t="str">
         <v>主題</v>
       </c>
-      <c r="D8" s="3" t="str">
+      <c r="D8" s="6" t="str">
         <v>UIUX 標完成</v>
       </c>
-      <c r="E8" s="3" t="str">
+      <c r="E8" s="6" t="str">
         <v>UIUX 新增</v>
       </c>
-      <c r="F8" s="3" t="str">
+      <c r="F8" s="6" t="str">
         <v>後臺新增</v>
       </c>
-      <c r="G8" s="3" t="str">
+      <c r="G8" s="6" t="str">
         <v>Schema</v>
       </c>
-      <c r="H8" s="3" t="str">
+      <c r="H8" s="6" t="str">
         <v>主要產出</v>
       </c>
     </row>
-    <row r="9" ht="14.4" customHeight="1">
+    <row r="9">
       <c r="A9" s="3" t="str">
         <v>Round 1</v>
       </c>
@@ -14937,7 +16076,7 @@
         <v>pages/ifare 加關鍵字搜尋 + URL query 初始化；全站 NuxtPage transition；卡片/按鈕 hover translateY</v>
       </c>
     </row>
-    <row r="10" ht="14.4" customHeight="1">
+    <row r="10">
       <c r="A10" s="3" t="str">
         <v>Round 2</v>
       </c>
@@ -14963,7 +16102,7 @@
         <v>LINE/FB 統一 .btn-social 並排；4 個聯絡資訊加 icon (Tel/Mail/Address/Clock)；footer 觸控 44px</v>
       </c>
     </row>
-    <row r="11" ht="14.4" customHeight="1">
+    <row r="11">
       <c r="A11" s="3" t="str">
         <v>Round 3</v>
       </c>
@@ -14989,7 +16128,7 @@
         <v>About 三大核心 morph 卡 (cf47cfa)；News 浮起卡 + stagger fade-up + NEW pill；外連結 target="_blank" rel="noopener"</v>
       </c>
     </row>
-    <row r="12" ht="14.4" customHeight="1">
+    <row r="12">
       <c r="A12" s="3" t="str">
         <v>Round 4</v>
       </c>
@@ -15015,7 +16154,7 @@
         <v>cf47cfa+5dfbf91 補回 16 檔；devProxy/baseURL → 正式 API；nav 加未來規劃 + future.vue；News videoUrl wiring；tsconfig deprecation 清理；about hover bug 修；footer label 重複修</v>
       </c>
     </row>
-    <row r="13" ht="14.4" customHeight="1">
+    <row r="13">
       <c r="A13" s="3" t="str">
         <v>Round 5</v>
       </c>
@@ -15041,7 +16180,7 @@
         <v>後台 22 個工程角度問題 (CRUD/驗證/錯誤處理)；前台 26 個新發現 (XSS/超時/console.log/無障礙/分頁元件重複)</v>
       </c>
     </row>
-    <row r="14" ht="14.4" customHeight="1">
+    <row r="14">
       <c r="A14" s="3" t="str">
         <v>Round 6</v>
       </c>
@@ -15067,7 +16206,7 @@
         <v>Dashboard 角色化 / 今日待辦 / KPI 分區；批次操作；軟刪除復原；audit log；危險操作預覽；錯誤訊息引導</v>
       </c>
     </row>
-    <row r="15" ht="14.4" customHeight="1">
+    <row r="15">
       <c r="A15" s="3" t="str">
         <v>Round 7</v>
       </c>
@@ -15093,7 +16232,7 @@
         <v>補充 GA4 同步快取、任務中心、自動儲存與編輯鎖定、發布排程、審稿指派、內容健康檢查、通知中心、資產治理</v>
       </c>
     </row>
-    <row r="16" ht="14.4" customHeight="1">
+    <row r="16">
       <c r="A16" s="3" t="str">
         <v>Round 8</v>
       </c>
@@ -15119,7 +16258,7 @@
         <v>HomeView 新增搜尋 / 分組 / 最近使用；PageManagement 補上 URL 預覽、狀態說明、SEO 預覽、常用標籤建議、排程快捷鍵</v>
       </c>
     </row>
-    <row r="17" ht="14.4" customHeight="1">
+    <row r="17">
       <c r="A17" s="3" t="str">
         <v>Round 9</v>
       </c>
@@ -15145,59 +16284,59 @@
         <v>future.vue 補強手機版主標換行、空狀態導引卡、上下留白與 footer CTA 銜接</v>
       </c>
     </row>
-    <row r="19" ht="14.4" customHeight="1">
-      <c r="A19" s="3" t="str">
+    <row r="19">
+      <c r="A19" s="5" t="str">
         <v>【3】後臺優化 — 5 主軸分布 (拿這個去提案!)</v>
       </c>
-      <c r="B19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G19" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H19" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="14.4" customHeight="1">
-      <c r="A20" s="3" t="str">
+      <c r="B19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G19" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H19" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="str">
         <v>主軸</v>
       </c>
-      <c r="B20" s="3" t="str">
+      <c r="B20" s="6" t="str">
         <v>項目數</v>
       </c>
-      <c r="C20" s="3" t="str">
+      <c r="C20" s="6" t="str">
         <v>比例</v>
       </c>
-      <c r="D20" s="3" t="str">
+      <c r="D20" s="6" t="str">
         <v>主要訴求</v>
       </c>
-      <c r="E20" s="3" t="str">
+      <c r="E20" s="6" t="str">
         <v>對應 #</v>
       </c>
-      <c r="F20" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G20" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H20" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="14.4" customHeight="1">
+      <c r="F20" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G20" s="6" t="str">
+        <v/>
+      </c>
+      <c r="H20" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="3" t="str">
         <v>看得懂</v>
       </c>
@@ -15205,7 +16344,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="3" t="str">
-        <v>28.6%</v>
+        <v>18.0%</v>
       </c>
       <c r="D21" s="3" t="str">
         <v>首頁先給重點 / KPI / 異常 / 待辦分區 / 欄位白話 / 狀態流程視覺化</v>
@@ -15223,7 +16362,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="14.4" customHeight="1">
+    <row r="22">
       <c r="A22" s="3" t="str">
         <v>找得到</v>
       </c>
@@ -15231,7 +16370,7 @@
         <v>7</v>
       </c>
       <c r="C22" s="3" t="str">
-        <v>11.1%</v>
+        <v>7.0%</v>
       </c>
       <c r="D22" s="3" t="str">
         <v>全域搜尋 / 麵包屑 / 側邊欄高亮 / 變更密碼入口</v>
@@ -15249,7 +16388,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="14.4" customHeight="1">
+    <row r="23">
       <c r="A23" s="3" t="str">
         <v>做得快</v>
       </c>
@@ -15257,7 +16396,7 @@
         <v>11</v>
       </c>
       <c r="C23" s="3" t="str">
-        <v>17.5%</v>
+        <v>11.0%</v>
       </c>
       <c r="D23" s="3" t="str">
         <v>批次操作 / 儲存搜尋 / 大列表 lazy / 匯出進度 / 日期快捷</v>
@@ -15275,15 +16414,15 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="14.4" customHeight="1">
+    <row r="24">
       <c r="A24" s="3" t="str">
         <v>不容易錯</v>
       </c>
       <c r="B24" s="3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C24" s="3" t="str">
-        <v>23.8%</v>
+        <v>18.0%</v>
       </c>
       <c r="D24" s="3" t="str">
         <v>表單驗證 / 刪除確認 / 影響預覽 / 預設值 / 錯誤引導</v>
@@ -15301,15 +16440,15 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="14.4" customHeight="1">
+    <row r="25">
       <c r="A25" s="3" t="str">
         <v>出事能追回來</v>
       </c>
       <c r="B25" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C25" s="3" t="str">
-        <v>11.1%</v>
+        <v>8.0%</v>
       </c>
       <c r="D25" s="3" t="str">
         <v>audit log / 變更歷史 / 軟刪除復原 / token 管理 / 文件交接</v>
@@ -15327,15 +16466,15 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="14.4" customHeight="1">
+    <row r="26">
       <c r="A26" s="3" t="str">
         <v>—</v>
       </c>
       <c r="B26" s="3">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C26" s="3" t="str">
-        <v>7.9%</v>
+        <v>25.0%</v>
       </c>
       <c r="D26" s="3" t="str">
         <v>純技術 / 環境設定 (不在 5 主軸範圍)</v>
@@ -15353,76 +16492,76 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="14.4" customHeight="1">
-      <c r="A28" s="3" t="str">
+    <row r="28">
+      <c r="A28" s="5" t="str">
         <v>【4】UIUX — 優先級 × 狀態分布</v>
       </c>
-      <c r="B28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G28" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H28" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="14.4" customHeight="1">
-      <c r="A29" s="3" t="str">
+      <c r="B28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G28" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H28" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="str">
         <v>優先級</v>
       </c>
-      <c r="B29" s="3" t="str">
+      <c r="B29" s="6" t="str">
         <v>已修正</v>
       </c>
-      <c r="C29" s="3" t="str">
+      <c r="C29" s="6" t="str">
         <v>部分修正</v>
       </c>
-      <c r="D29" s="3" t="str">
+      <c r="D29" s="6" t="str">
         <v>待處理</v>
       </c>
-      <c r="E29" s="3" t="str">
+      <c r="E29" s="6" t="str">
         <v>小計</v>
       </c>
-      <c r="F29" s="3" t="str">
+      <c r="F29" s="6" t="str">
         <v>完成率</v>
       </c>
-      <c r="G29" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H29" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="14.4" customHeight="1">
+      <c r="G29" s="6" t="str">
+        <v/>
+      </c>
+      <c r="H29" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" s="3" t="str">
         <v>高</v>
       </c>
-      <c r="B30" s="3">
-        <v>22</v>
-      </c>
-      <c r="C30" s="3">
-        <v>6</v>
-      </c>
-      <c r="D30" s="3">
-        <v>4</v>
+      <c r="B30" s="7">
+        <v>23</v>
+      </c>
+      <c r="C30" s="8">
+        <v>10</v>
+      </c>
+      <c r="D30" s="9">
+        <v>3</v>
       </c>
       <c r="E30" s="3">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F30" s="3" t="str">
-        <v>78.1%</v>
+        <v>77.8%</v>
       </c>
       <c r="G30" s="3" t="str">
         <v/>
@@ -15431,24 +16570,24 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="14.4" customHeight="1">
+    <row r="31">
       <c r="A31" s="3" t="str">
         <v>中</v>
       </c>
-      <c r="B31" s="3">
-        <v>59</v>
-      </c>
-      <c r="C31" s="3">
-        <v>1</v>
-      </c>
-      <c r="D31" s="3">
-        <v>18</v>
+      <c r="B31" s="7">
+        <v>61</v>
+      </c>
+      <c r="C31" s="8">
+        <v>5</v>
+      </c>
+      <c r="D31" s="9">
+        <v>17</v>
       </c>
       <c r="E31" s="3">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F31" s="3" t="str">
-        <v>76.3%</v>
+        <v>76.5%</v>
       </c>
       <c r="G31" s="3" t="str">
         <v/>
@@ -15457,17 +16596,17 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="14.4" customHeight="1">
+    <row r="32">
       <c r="A32" s="3" t="str">
         <v>低</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32" s="7">
         <v>40</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="8">
         <v>4</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="9">
         <v>11</v>
       </c>
       <c r="E32" s="3">
@@ -15483,67 +16622,67 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="14.4" customHeight="1">
-      <c r="A34" s="3" t="str">
+    <row r="34">
+      <c r="A34" s="5" t="str">
         <v>【5】UIUX — 各區塊問題分布</v>
       </c>
-      <c r="B34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G34" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H34" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="14.4" customHeight="1">
-      <c r="A35" s="3" t="str">
+      <c r="B34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H34" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="str">
         <v>區塊</v>
       </c>
-      <c r="B35" s="3" t="str">
+      <c r="B35" s="6" t="str">
         <v>項目數</v>
       </c>
-      <c r="C35" s="3" t="str">
+      <c r="C35" s="6" t="str">
         <v>佔比</v>
       </c>
-      <c r="D35" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E35" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F35" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G35" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H35" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="14.4" customHeight="1">
+      <c r="D35" s="6" t="str">
+        <v/>
+      </c>
+      <c r="E35" s="6" t="str">
+        <v/>
+      </c>
+      <c r="F35" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G35" s="6" t="str">
+        <v/>
+      </c>
+      <c r="H35" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36" s="3" t="str">
         <v>全站通用</v>
       </c>
       <c r="B36" s="3">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C36" s="3" t="str">
-        <v>25.5%</v>
+        <v>24.7%</v>
       </c>
       <c r="D36" s="3" t="str">
         <v/>
@@ -15561,15 +16700,15 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="14.4" customHeight="1">
+    <row r="37">
       <c r="A37" s="3" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
       <c r="B37" s="3">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C37" s="3" t="str">
-        <v>15.8%</v>
+        <v>17.2%</v>
       </c>
       <c r="D37" s="3" t="str">
         <v/>
@@ -15587,7 +16726,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="14.4" customHeight="1">
+    <row r="38">
       <c r="A38" s="3" t="str">
         <v>共用元件</v>
       </c>
@@ -15595,7 +16734,7 @@
         <v>25</v>
       </c>
       <c r="C38" s="3" t="str">
-        <v>15.2%</v>
+        <v>14.4%</v>
       </c>
       <c r="D38" s="3" t="str">
         <v/>
@@ -15613,7 +16752,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="14.4" customHeight="1">
+    <row r="39">
       <c r="A39" s="3" t="str">
         <v>福利專欄</v>
       </c>
@@ -15621,7 +16760,7 @@
         <v>11</v>
       </c>
       <c r="C39" s="3" t="str">
-        <v>6.7%</v>
+        <v>6.3%</v>
       </c>
       <c r="D39" s="3" t="str">
         <v/>
@@ -15639,7 +16778,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="14.4" customHeight="1">
+    <row r="40">
       <c r="A40" s="3" t="str">
         <v>首頁</v>
       </c>
@@ -15647,7 +16786,7 @@
         <v>10</v>
       </c>
       <c r="C40" s="3" t="str">
-        <v>6.1%</v>
+        <v>5.7%</v>
       </c>
       <c r="D40" s="3" t="str">
         <v/>
@@ -15665,7 +16804,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="14.4" customHeight="1">
+    <row r="41">
       <c r="A41" s="3" t="str">
         <v>關於長穩</v>
       </c>
@@ -15673,7 +16812,7 @@
         <v>9</v>
       </c>
       <c r="C41" s="3" t="str">
-        <v>5.5%</v>
+        <v>5.2%</v>
       </c>
       <c r="D41" s="3" t="str">
         <v/>
@@ -15691,7 +16830,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="14.4" customHeight="1">
+    <row r="42">
       <c r="A42" s="3" t="str">
         <v>最新消息</v>
       </c>
@@ -15699,7 +16838,7 @@
         <v>8</v>
       </c>
       <c r="C42" s="3" t="str">
-        <v>4.8%</v>
+        <v>4.6%</v>
       </c>
       <c r="D42" s="3" t="str">
         <v/>
@@ -15717,7 +16856,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="14.4" customHeight="1">
+    <row r="43">
       <c r="A43" s="3" t="str">
         <v>公益夥伴</v>
       </c>
@@ -15725,7 +16864,7 @@
         <v>8</v>
       </c>
       <c r="C43" s="3" t="str">
-        <v>4.8%</v>
+        <v>4.6%</v>
       </c>
       <c r="D43" s="3" t="str">
         <v/>
@@ -15743,7 +16882,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="14.4" customHeight="1">
+    <row r="44">
       <c r="A44" s="3" t="str">
         <v>全站微互動</v>
       </c>
@@ -15751,7 +16890,7 @@
         <v>5</v>
       </c>
       <c r="C44" s="3" t="str">
-        <v>3.0%</v>
+        <v>2.9%</v>
       </c>
       <c r="D44" s="3" t="str">
         <v/>
@@ -15769,7 +16908,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="14.4" customHeight="1">
+    <row r="45">
       <c r="A45" s="3" t="str">
         <v>設計系統</v>
       </c>
@@ -15777,7 +16916,7 @@
         <v>5</v>
       </c>
       <c r="C45" s="3" t="str">
-        <v>3.0%</v>
+        <v>2.9%</v>
       </c>
       <c r="D45" s="3" t="str">
         <v/>
@@ -15795,7 +16934,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="14.4" customHeight="1">
+    <row r="46">
       <c r="A46" s="3" t="str">
         <v>未來規劃</v>
       </c>
@@ -15803,7 +16942,7 @@
         <v>3</v>
       </c>
       <c r="C46" s="3" t="str">
-        <v>1.8%</v>
+        <v>1.7%</v>
       </c>
       <c r="D46" s="3" t="str">
         <v/>
@@ -15821,41 +16960,41 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="14.4" customHeight="1">
+    <row r="47">
       <c r="A47" s="3" t="str">
+        <v>i-Fare 福利詳情</v>
+      </c>
+      <c r="B47" s="3">
+        <v>3</v>
+      </c>
+      <c r="C47" s="3" t="str">
+        <v>1.7%</v>
+      </c>
+      <c r="D47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H47" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="str">
         <v>安全性</v>
-      </c>
-      <c r="B47" s="3">
-        <v>2</v>
-      </c>
-      <c r="C47" s="3" t="str">
-        <v>1.2%</v>
-      </c>
-      <c r="D47" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E47" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F47" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G47" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H47" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="14.4" customHeight="1">
-      <c r="A48" s="3" t="str">
-        <v>無障礙</v>
       </c>
       <c r="B48" s="3">
         <v>2</v>
       </c>
       <c r="C48" s="3" t="str">
-        <v>1.2%</v>
+        <v>1.1%</v>
       </c>
       <c r="D48" s="3" t="str">
         <v/>
@@ -15873,35 +17012,35 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="14.4" customHeight="1">
+    <row r="49">
       <c r="A49" s="3" t="str">
+        <v>無障礙</v>
+      </c>
+      <c r="B49" s="3">
+        <v>2</v>
+      </c>
+      <c r="C49" s="3" t="str">
+        <v>1.1%</v>
+      </c>
+      <c r="D49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H49" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="str">
         <v>頁面導航</v>
-      </c>
-      <c r="B49" s="3">
-        <v>1</v>
-      </c>
-      <c r="C49" s="3" t="str">
-        <v>0.6%</v>
-      </c>
-      <c r="D49" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E49" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F49" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G49" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H49" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14.4" customHeight="1">
-      <c r="A50" s="3" t="str">
-        <v>i-Fare 搜尋結果</v>
       </c>
       <c r="B50" s="3">
         <v>1</v>
@@ -15925,9 +17064,9 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="14.4" customHeight="1">
+    <row r="51">
       <c r="A51" s="3" t="str">
-        <v>效能</v>
+        <v>i-Fare 搜尋結果</v>
       </c>
       <c r="B51" s="3">
         <v>1</v>
@@ -15951,9 +17090,9 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="14.4" customHeight="1">
+    <row r="52">
       <c r="A52" s="3" t="str">
-        <v>社群分享</v>
+        <v>效能</v>
       </c>
       <c r="B52" s="3">
         <v>1</v>
@@ -15977,9 +17116,9 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="14.4" customHeight="1">
+    <row r="53">
       <c r="A53" s="3" t="str">
-        <v>導航</v>
+        <v>社群分享</v>
       </c>
       <c r="B53" s="3">
         <v>1</v>
@@ -16003,9 +17142,9 @@
         <v/>
       </c>
     </row>
-    <row r="54" ht="14.4" customHeight="1">
+    <row r="54">
       <c r="A54" s="3" t="str">
-        <v>關於我們</v>
+        <v>導航</v>
       </c>
       <c r="B54" s="3">
         <v>1</v>
@@ -16029,9 +17168,9 @@
         <v/>
       </c>
     </row>
-    <row r="55" ht="14.4" customHeight="1">
+    <row r="55">
       <c r="A55" s="3" t="str">
-        <v>後台</v>
+        <v>關於我們</v>
       </c>
       <c r="B55" s="3">
         <v>1</v>
@@ -16055,9 +17194,9 @@
         <v/>
       </c>
     </row>
-    <row r="56" ht="14.4" customHeight="1">
+    <row r="56">
       <c r="A56" s="3" t="str">
-        <v>preview 頁</v>
+        <v>後台</v>
       </c>
       <c r="B56" s="3">
         <v>1</v>
@@ -16081,9 +17220,9 @@
         <v/>
       </c>
     </row>
-    <row r="57" ht="14.4" customHeight="1">
+    <row r="57">
       <c r="A57" s="3" t="str">
-        <v>追蹤文件</v>
+        <v>preview 頁</v>
       </c>
       <c r="B57" s="3">
         <v>1</v>
@@ -16107,327 +17246,327 @@
         <v/>
       </c>
     </row>
-    <row r="59" ht="14.4" customHeight="1">
+    <row r="58">
+      <c r="A58" s="3" t="str">
+        <v>追蹤文件</v>
+      </c>
+      <c r="B58" s="3">
+        <v>1</v>
+      </c>
+      <c r="C58" s="3" t="str">
+        <v>0.6%</v>
+      </c>
+      <c r="D58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H58" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
       <c r="A59" s="3" t="str">
+        <v>i-Fare 福利政策</v>
+      </c>
+      <c r="B59" s="3">
+        <v>1</v>
+      </c>
+      <c r="C59" s="3" t="str">
+        <v>0.6%</v>
+      </c>
+      <c r="D59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H59" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="str">
         <v>【6】後臺優化 — 各區塊問題分布</v>
       </c>
-      <c r="B59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G59" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H59" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="14.4" customHeight="1">
-      <c r="A60" s="3" t="str">
+      <c r="B61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G61" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H61" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="str">
         <v>區塊</v>
       </c>
-      <c r="B60" s="3" t="str">
+      <c r="B62" s="6" t="str">
         <v>項目數</v>
       </c>
-      <c r="C60" s="3" t="str">
+      <c r="C62" s="6" t="str">
         <v>佔比</v>
       </c>
-      <c r="D60" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E60" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F60" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G60" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H60" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="14.4" customHeight="1">
-      <c r="A61" s="3" t="str">
+      <c r="D62" s="6" t="str">
+        <v/>
+      </c>
+      <c r="E62" s="6" t="str">
+        <v/>
+      </c>
+      <c r="F62" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G62" s="6" t="str">
+        <v/>
+      </c>
+      <c r="H62" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="str">
         <v>後台通用</v>
       </c>
-      <c r="B61" s="3">
-        <v>19</v>
-      </c>
-      <c r="C61" s="3" t="str">
-        <v>30.2%</v>
-      </c>
-      <c r="D61" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E61" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F61" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G61" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H61" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="14.4" customHeight="1">
-      <c r="A62" s="3" t="str">
+      <c r="B63" s="3">
+        <v>26</v>
+      </c>
+      <c r="C63" s="3" t="str">
+        <v>26.0%</v>
+      </c>
+      <c r="D63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H63" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="str">
         <v>共用元件</v>
       </c>
-      <c r="B62" s="3">
-        <v>17</v>
-      </c>
-      <c r="C62" s="3" t="str">
-        <v>27.0%</v>
-      </c>
-      <c r="D62" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E62" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F62" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G62" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H62" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="14.4" customHeight="1">
-      <c r="A63" s="3" t="str">
+      <c r="B64" s="3">
+        <v>21</v>
+      </c>
+      <c r="C64" s="3" t="str">
+        <v>21.0%</v>
+      </c>
+      <c r="D64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H64" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="str">
+        <v>i-Fare 維護</v>
+      </c>
+      <c r="B65" s="3">
+        <v>8</v>
+      </c>
+      <c r="C65" s="3" t="str">
+        <v>8.0%</v>
+      </c>
+      <c r="D65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H65" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="str">
+        <v>頁面管理</v>
+      </c>
+      <c r="B66" s="3">
+        <v>8</v>
+      </c>
+      <c r="C66" s="3" t="str">
+        <v>8.0%</v>
+      </c>
+      <c r="D66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H66" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="str">
+        <v>資料分析</v>
+      </c>
+      <c r="B67" s="3">
+        <v>7</v>
+      </c>
+      <c r="C67" s="3" t="str">
+        <v>7.0%</v>
+      </c>
+      <c r="D67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H67" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="str">
         <v>圖片管理</v>
       </c>
-      <c r="B63" s="3">
-        <v>3</v>
-      </c>
-      <c r="C63" s="3" t="str">
-        <v>4.8%</v>
-      </c>
-      <c r="D63" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E63" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F63" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G63" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H63" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="14.4" customHeight="1">
-      <c r="A64" s="3" t="str">
-        <v>i-Fare 維護</v>
-      </c>
-      <c r="B64" s="3">
+      <c r="B68" s="3">
+        <v>4</v>
+      </c>
+      <c r="C68" s="3" t="str">
+        <v>4.0%</v>
+      </c>
+      <c r="D68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H68" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="str">
+        <v>內容品質</v>
+      </c>
+      <c r="B69" s="3">
         <v>2</v>
       </c>
-      <c r="C64" s="3" t="str">
-        <v>3.2%</v>
-      </c>
-      <c r="D64" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E64" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F64" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G64" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H64" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="14.4" customHeight="1">
-      <c r="A65" s="3" t="str">
+      <c r="C69" s="3" t="str">
+        <v>2.0%</v>
+      </c>
+      <c r="D69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H69" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="str">
+        <v>內容管理</v>
+      </c>
+      <c r="B70" s="3">
+        <v>2</v>
+      </c>
+      <c r="C70" s="3" t="str">
+        <v>2.0%</v>
+      </c>
+      <c r="D70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H70" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="str">
         <v>最新消息維護</v>
-      </c>
-      <c r="B65" s="3">
-        <v>1</v>
-      </c>
-      <c r="C65" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D65" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E65" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F65" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G65" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H65" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="14.4" customHeight="1">
-      <c r="A66" s="3" t="str">
-        <v>帳戶維護 / 全站權限</v>
-      </c>
-      <c r="B66" s="3">
-        <v>1</v>
-      </c>
-      <c r="C66" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D66" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E66" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F66" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G66" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H66" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="67" ht="14.4" customHeight="1">
-      <c r="A67" s="3" t="str">
-        <v>前台通用</v>
-      </c>
-      <c r="B67" s="3">
-        <v>1</v>
-      </c>
-      <c r="C67" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D67" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E67" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F67" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G67" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H67" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="68" ht="14.4" customHeight="1">
-      <c r="A68" s="3" t="str">
-        <v>對話框</v>
-      </c>
-      <c r="B68" s="3">
-        <v>1</v>
-      </c>
-      <c r="C68" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D68" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E68" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F68" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G68" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H68" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="69" ht="14.4" customHeight="1">
-      <c r="A69" s="3" t="str">
-        <v>檔案上傳</v>
-      </c>
-      <c r="B69" s="3">
-        <v>1</v>
-      </c>
-      <c r="C69" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D69" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E69" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F69" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G69" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H69" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="70" ht="14.4" customHeight="1">
-      <c r="A70" s="3" t="str">
-        <v>帳號管理</v>
-      </c>
-      <c r="B70" s="3">
-        <v>1</v>
-      </c>
-      <c r="C70" s="3" t="str">
-        <v>1.6%</v>
-      </c>
-      <c r="D70" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E70" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F70" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G70" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H70" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="71" ht="14.4" customHeight="1">
-      <c r="A71" s="3" t="str">
-        <v>搜尋結果</v>
       </c>
       <c r="B71" s="3">
         <v>1</v>
       </c>
       <c r="C71" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D71" s="3" t="str">
         <v/>
@@ -16445,15 +17584,15 @@
         <v/>
       </c>
     </row>
-    <row r="72" ht="14.4" customHeight="1">
+    <row r="72">
       <c r="A72" s="3" t="str">
-        <v>日期選擇</v>
+        <v>帳戶維護 / 全站權限</v>
       </c>
       <c r="B72" s="3">
         <v>1</v>
       </c>
       <c r="C72" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D72" s="3" t="str">
         <v/>
@@ -16471,15 +17610,15 @@
         <v/>
       </c>
     </row>
-    <row r="73" ht="14.4" customHeight="1">
+    <row r="73">
       <c r="A73" s="3" t="str">
-        <v>表單</v>
+        <v>前台通用</v>
       </c>
       <c r="B73" s="3">
         <v>1</v>
       </c>
       <c r="C73" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D73" s="3" t="str">
         <v/>
@@ -16497,15 +17636,15 @@
         <v/>
       </c>
     </row>
-    <row r="74" ht="14.4" customHeight="1">
+    <row r="74">
       <c r="A74" s="3" t="str">
-        <v>側邊欄</v>
+        <v>對話框</v>
       </c>
       <c r="B74" s="3">
         <v>1</v>
       </c>
       <c r="C74" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D74" s="3" t="str">
         <v/>
@@ -16523,15 +17662,15 @@
         <v/>
       </c>
     </row>
-    <row r="75" ht="14.4" customHeight="1">
+    <row r="75">
       <c r="A75" s="3" t="str">
-        <v>麵包屑導覽</v>
+        <v>檔案上傳</v>
       </c>
       <c r="B75" s="3">
         <v>1</v>
       </c>
       <c r="C75" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D75" s="3" t="str">
         <v/>
@@ -16549,15 +17688,15 @@
         <v/>
       </c>
     </row>
-    <row r="76" ht="14.4" customHeight="1">
+    <row r="76">
       <c r="A76" s="3" t="str">
-        <v>WebAPI</v>
+        <v>帳號管理</v>
       </c>
       <c r="B76" s="3">
         <v>1</v>
       </c>
       <c r="C76" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D76" s="3" t="str">
         <v/>
@@ -16575,15 +17714,15 @@
         <v/>
       </c>
     </row>
-    <row r="77" ht="14.4" customHeight="1">
+    <row r="77">
       <c r="A77" s="3" t="str">
-        <v>帳號變更密碼</v>
+        <v>搜尋結果</v>
       </c>
       <c r="B77" s="3">
         <v>1</v>
       </c>
       <c r="C77" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D77" s="3" t="str">
         <v/>
@@ -16601,15 +17740,15 @@
         <v/>
       </c>
     </row>
-    <row r="78" ht="14.4" customHeight="1">
+    <row r="78">
       <c r="A78" s="3" t="str">
-        <v>Code 代碼管理</v>
+        <v>日期選擇</v>
       </c>
       <c r="B78" s="3">
         <v>1</v>
       </c>
       <c r="C78" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D78" s="3" t="str">
         <v/>
@@ -16627,15 +17766,15 @@
         <v/>
       </c>
     </row>
-    <row r="79" ht="14.4" customHeight="1">
+    <row r="79">
       <c r="A79" s="3" t="str">
-        <v>狀態管理</v>
+        <v>表單</v>
       </c>
       <c r="B79" s="3">
         <v>1</v>
       </c>
       <c r="C79" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D79" s="3" t="str">
         <v/>
@@ -16653,15 +17792,15 @@
         <v/>
       </c>
     </row>
-    <row r="80" ht="14.4" customHeight="1">
+    <row r="80">
       <c r="A80" s="3" t="str">
-        <v>登入頁面</v>
+        <v>側邊欄</v>
       </c>
       <c r="B80" s="3">
         <v>1</v>
       </c>
       <c r="C80" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D80" s="3" t="str">
         <v/>
@@ -16679,15 +17818,15 @@
         <v/>
       </c>
     </row>
-    <row r="81" ht="14.4" customHeight="1">
+    <row r="81">
       <c r="A81" s="3" t="str">
-        <v>HTML 編輯器</v>
+        <v>麵包屑導覽</v>
       </c>
       <c r="B81" s="3">
         <v>1</v>
       </c>
       <c r="C81" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D81" s="3" t="str">
         <v/>
@@ -16705,15 +17844,15 @@
         <v/>
       </c>
     </row>
-    <row r="82" ht="14.4" customHeight="1">
+    <row r="82">
       <c r="A82" s="3" t="str">
-        <v>無權限頁</v>
+        <v>WebAPI</v>
       </c>
       <c r="B82" s="3">
         <v>1</v>
       </c>
       <c r="C82" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D82" s="3" t="str">
         <v/>
@@ -16731,15 +17870,15 @@
         <v/>
       </c>
     </row>
-    <row r="83" ht="14.4" customHeight="1">
+    <row r="83">
       <c r="A83" s="3" t="str">
-        <v>效能</v>
+        <v>帳號變更密碼</v>
       </c>
       <c r="B83" s="3">
         <v>1</v>
       </c>
       <c r="C83" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D83" s="3" t="str">
         <v/>
@@ -16757,15 +17896,15 @@
         <v/>
       </c>
     </row>
-    <row r="84" ht="14.4" customHeight="1">
+    <row r="84">
       <c r="A84" s="3" t="str">
-        <v>後台首頁</v>
+        <v>Code 代碼管理</v>
       </c>
       <c r="B84" s="3">
         <v>1</v>
       </c>
       <c r="C84" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D84" s="3" t="str">
         <v/>
@@ -16783,15 +17922,15 @@
         <v/>
       </c>
     </row>
-    <row r="85" ht="14.4" customHeight="1">
+    <row r="85">
       <c r="A85" s="3" t="str">
-        <v>內容品質</v>
+        <v>狀態管理</v>
       </c>
       <c r="B85" s="3">
         <v>1</v>
       </c>
       <c r="C85" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D85" s="3" t="str">
         <v/>
@@ -16809,15 +17948,15 @@
         <v/>
       </c>
     </row>
-    <row r="86" ht="14.4" customHeight="1">
+    <row r="86">
       <c r="A86" s="3" t="str">
-        <v>資料分析</v>
+        <v>登入頁面</v>
       </c>
       <c r="B86" s="3">
         <v>1</v>
       </c>
       <c r="C86" s="3" t="str">
-        <v>1.6%</v>
+        <v>1.0%</v>
       </c>
       <c r="D86" s="3" t="str">
         <v/>
@@ -16835,218 +17974,348 @@
         <v/>
       </c>
     </row>
-    <row r="88" ht="14.4" customHeight="1">
+    <row r="87">
+      <c r="A87" s="3" t="str">
+        <v>HTML 編輯器</v>
+      </c>
+      <c r="B87" s="3">
+        <v>1</v>
+      </c>
+      <c r="C87" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H87" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
       <c r="A88" s="3" t="str">
+        <v>無權限頁</v>
+      </c>
+      <c r="B88" s="3">
+        <v>1</v>
+      </c>
+      <c r="C88" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H88" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="str">
+        <v>效能</v>
+      </c>
+      <c r="B89" s="3">
+        <v>1</v>
+      </c>
+      <c r="C89" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H89" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="str">
+        <v>後台首頁</v>
+      </c>
+      <c r="B90" s="3">
+        <v>1</v>
+      </c>
+      <c r="C90" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H90" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="str">
+        <v>前台動態頁</v>
+      </c>
+      <c r="B91" s="3">
+        <v>1</v>
+      </c>
+      <c r="C91" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H91" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="str">
+        <v>發布流程</v>
+      </c>
+      <c r="B92" s="3">
+        <v>1</v>
+      </c>
+      <c r="C92" s="3" t="str">
+        <v>1.0%</v>
+      </c>
+      <c r="D92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H92" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="str">
         <v>【7】你做了什麼 — 已完成項目摘要 (依 Round 分組)</v>
       </c>
-      <c r="B88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="C88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="D88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="E88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="F88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="G88" s="3" t="str">
-        <v/>
-      </c>
-      <c r="H88" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="89" ht="14.4" customHeight="1">
-      <c r="A89" s="3" t="str">
+      <c r="B94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="C94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="D94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G94" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H94" s="5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="str">
         <v>Round</v>
       </c>
-      <c r="B89" s="3" t="str">
+      <c r="B95" s="6" t="str">
         <v>日期</v>
       </c>
-      <c r="C89" s="3" t="str">
+      <c r="C95" s="6" t="str">
         <v>已修正 (綠)</v>
       </c>
-      <c r="D89" s="3" t="str">
+      <c r="D95" s="6" t="str">
         <v>部分修正 (黃)</v>
       </c>
-      <c r="E89" s="3" t="str">
+      <c r="E95" s="6" t="str">
         <v>已修正 # 清單</v>
       </c>
-      <c r="F89" s="3" t="str">
+      <c r="F95" s="6" t="str">
         <v>部分修正 # 清單</v>
       </c>
-      <c r="G89" s="3" t="str">
+      <c r="G95" s="6" t="str">
         <v>主要重點</v>
       </c>
-      <c r="H89" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="90" ht="14.4" customHeight="1">
-      <c r="A90" s="3" t="str">
+      <c r="H95" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="str">
         <v>Round 1</v>
       </c>
-      <c r="B90" s="3" t="str">
+      <c r="B96" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C90" s="3">
-        <v>103</v>
-      </c>
-      <c r="D90" s="3">
-        <v>11</v>
-      </c>
-      <c r="E90" s="3" t="str">
-        <v>#1, #2, #3, #6, #7, #9, #11, #12, #13, #14, #15, #16, #17, #22, #23, #24, #27, #28, #29, #30, #31, #32, #36, #37, #38, #40, #41, #44, #45, #46, #47, #48, #49, #50, #52, #53, #54, #55, #56, #58, #59, #60, #61, #70, #71, #75, #77, #79, #80, #82, #86, #87, #88, #89, #90, #106, #108, #109, #110, #111, #112, #113, #114, #115, #116, #117, #118, #119, #120, #122, #123, #124, #125, #126, #127, #128, #129, #130, #131, #132, #133, #134, #135, #137, #138, #139, #140, #143, #145, #146, #147, #149, #150, #151, #152, #153, #155, #156, #157, #159, #161, #162, #163</v>
-      </c>
-      <c r="F90" s="3" t="str">
-        <v>#67, #68, #73, #76, #107, #136, #141, #142, #144, #158, #160</v>
-      </c>
-      <c r="G90" s="3" t="str">
+      <c r="C96" s="7">
+        <v>106</v>
+      </c>
+      <c r="D96" s="8">
+        <v>19</v>
+      </c>
+      <c r="E96" s="3" t="str">
+        <v>#1, #2, #3, #6, #7, #9, #11, #12, #13, #14, #15, #16, #17, #22, #23, #24, #27, #28, #29, #30, #31, #32, #36, #37, #38, #40, #41, #44, #45, #46, #47, #48, #49, #50, #52, #53, #54, #55, #56, #58, #59, #60, #61, #70, #71, #75, #77, #79, #80, #82, #86, #87, #88, #89, #90, #106, #108, #109, #110, #111, #112, #113, #114, #115, #116, #117, #118, #119, #120, #122, #123, #124, #125, #126, #127, #128, #129, #130, #131, #132, #133, #134, #135, #137, #138, #139, #140, #143, #145, #146, #147, #148, #149, #150, #151, #152, #153, #154, #155, #156, #157, #159, #161, #162, #163, #166</v>
+      </c>
+      <c r="F96" s="3" t="str">
+        <v>#67, #68, #73, #76, #107, #136, #141, #142, #144, #158, #160, #167, #168, #169, #170, #171, #172, #173, #174</v>
+      </c>
+      <c r="G96" s="3" t="str">
         <v>搜尋優化 (移除 disabled / 結果摘要) + 全站動畫 + skeleton 載入 + 卡片/按鈕 hover translateY</v>
       </c>
-      <c r="H90" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="91" ht="14.4" customHeight="1">
-      <c r="A91" s="3" t="str">
+      <c r="H96" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="str">
         <v>Round 2</v>
       </c>
-      <c r="B91" s="3" t="str">
+      <c r="B97" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C91" s="3">
+      <c r="C97" s="7">
         <v>2</v>
       </c>
-      <c r="D91" s="3">
+      <c r="D97" s="8">
         <v>0</v>
       </c>
-      <c r="E91" s="3" t="str">
+      <c r="E97" s="3" t="str">
         <v>#91, #92</v>
       </c>
-      <c r="F91" s="3" t="str">
+      <c r="F97" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G91" s="3" t="str">
+      <c r="G97" s="3" t="str">
         <v>Footer 整合 (LINE/FB 並列 .btn-social) + 觸控目標 44px</v>
       </c>
-      <c r="H91" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="92" ht="14.4" customHeight="1">
-      <c r="A92" s="3" t="str">
+      <c r="H97" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="str">
         <v>Round 3</v>
       </c>
-      <c r="B92" s="3" t="str">
+      <c r="B98" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C92" s="3">
+      <c r="C98" s="7">
         <v>6</v>
       </c>
-      <c r="D92" s="3">
+      <c r="D98" s="8">
         <v>0</v>
       </c>
-      <c r="E92" s="3" t="str">
+      <c r="E98" s="3" t="str">
         <v>#26, #93, #94, #95, #96, #97</v>
       </c>
-      <c r="F92" s="3" t="str">
+      <c r="F98" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G92" s="3" t="str">
+      <c r="G98" s="3" t="str">
         <v>About 三大核心 morph 卡 + News 浮起卡 + 浮現動畫 + line-clamp + NEW pill + 社群 target="_blank"</v>
       </c>
-      <c r="H92" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="93" ht="14.4" customHeight="1">
-      <c r="A93" s="3" t="str">
+      <c r="H98" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="str">
         <v>Round 4</v>
       </c>
-      <c r="B93" s="3" t="str">
+      <c r="B99" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C93" s="3">
+      <c r="C99" s="7">
         <v>8</v>
       </c>
-      <c r="D93" s="3">
+      <c r="D99" s="8">
         <v>0</v>
       </c>
-      <c r="E93" s="3" t="str">
+      <c r="E99" s="3" t="str">
         <v>#98, #99, #100, #101, #102, #103, #104, #105</v>
       </c>
-      <c r="F93" s="3" t="str">
+      <c r="F99" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G93" s="3" t="str">
+      <c r="G99" s="3" t="str">
         <v>cf47cfa+5dfbf91 補回 16 檔 + 環境設定 (devProxy/baseURL) + 未來規劃 nav + News videoUrl wiring + tsconfig + about hover bug + footer label 重複</v>
       </c>
-      <c r="H93" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="94" ht="14.4" customHeight="1">
-      <c r="A94" s="3" t="str">
+      <c r="H99" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="str">
         <v>Round 9</v>
       </c>
-      <c r="B94" s="3" t="str">
+      <c r="B100" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C94" s="3">
+      <c r="C100" s="7">
         <v>2</v>
       </c>
-      <c r="D94" s="3">
+      <c r="D100" s="8">
         <v>0</v>
       </c>
-      <c r="E94" s="3" t="str">
+      <c r="E100" s="3" t="str">
         <v>#164, #165</v>
       </c>
-      <c r="F94" s="3" t="str">
+      <c r="F100" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G94" s="3" t="str">
+      <c r="G100" s="3" t="str">
         <v>future.vue 補強手機版主標換行、空狀態導引卡與上下節奏，讓頁面在未上線時也有清楚下一步</v>
       </c>
-      <c r="H94" s="3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95" ht="14.4" customHeight="1">
-      <c r="A95" s="3" t="str">
-        <v>Round 15</v>
-      </c>
-      <c r="B95" s="3" t="str">
-        <v>2026-05-19</v>
-      </c>
-      <c r="C95" s="3">
-        <v>13</v>
-      </c>
-      <c r="D95" s="3">
-        <v>0</v>
-      </c>
-      <c r="E95" s="3" t="str">
-        <v>後臺優化 #20, #21, #25, #26, #28, #36, #38, #71, #83, #84, #85, #86；UIUX #154</v>
-      </c>
-      <c r="F95" s="3" t="str">
-        <v>-</v>
-      </c>
-      <c r="G95" s="3" t="str">
-        <v>PageManagement 預覽與圖片修復；搜尋清除、日期快捷、刪除確認、表格空狀態、分頁重設、登入 Caps Lock、無權限頁、Analysis Dashboard RWD、RWD 回歸清單</v>
-      </c>
-      <c r="H95" s="3" t="str">
+      <c r="H100" s="3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: hash sysuser passwords and block disabled tokens
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -45,70 +45,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <b/>
-      <color rgb="FFFFFF"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <b/>
-      <color rgb="FFFFFF"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-      <color rgb="1F3864"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-      <color rgb="1F3864"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="006100"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="9C5700"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="595959"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="006100"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="9C5700"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="595959"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="2">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -116,66 +54,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E2F3"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E2F3"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -199,47 +77,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15671,13 +15518,13 @@
         <v>已讀程式碼：登入直接比對明文密碼，帳號 DTO/前端欄位使用 pwd。</v>
       </c>
       <c r="N178" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O178" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P178" s="3" t="str">
-        <v>立即處理；需搭配資料 migration 與使用者重設密碼。</v>
+        <v>2026-05-25：SysUser 新增 PBKDF2 hash helper；新增帳號與個人改密碼改寫 hash；登入與 LoginCheck 支援舊明文成功後自動 rehash；AccountResult/DTO 不再回傳 Pwd；後台帳號明細/編輯不再顯示或依賴密碼。待 dotnet/CI 環境編譯驗證與既有資料逐步 rehash。</v>
       </c>
     </row>
     <row r="179" xml:space="preserve">
@@ -15775,13 +15622,13 @@
         <v>已讀程式碼：Authenticate 呼叫 GetAuthUser 後即產生 token，GetAuthUser 未過濾停用狀態。</v>
       </c>
       <c r="N180" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O180" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P180" s="3" t="str">
-        <v>立即處理；與權限控管問題會互相放大風險。</v>
+        <v>2026-05-25：TokenAuthController 呼叫的 AuthTaskManager.GetAuthUser 現在只允許 State == Enabled 的帳號通過，停用/非啟用帳號不再簽發 JWT；LoginCheck 同步檢查 State == Enabled。待 dotnet/CI 環境編譯與 API 測試驗證。</v>
       </c>
     </row>
     <row r="181" xml:space="preserve">
@@ -16010,2899 +15857,2899 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H118"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
-    <col min="5" max="5" width="50.5546875" customWidth="1"/>
-    <col min="6" max="6" width="25.5546875" customWidth="1"/>
-    <col min="7" max="7" width="60.5546875" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="14.5546875"/>
+    <col min="2" max="2" customWidth="1" width="12.5546875"/>
+    <col min="3" max="3" customWidth="1" width="14.5546875"/>
+    <col min="4" max="4" customWidth="1" width="14.5546875"/>
+    <col min="5" max="5" customWidth="1" width="50.5546875"/>
+    <col min="6" max="6" customWidth="1" width="25.5546875"/>
+    <col min="7" max="7" customWidth="1" width="60.5546875"/>
+    <col min="8" max="8" customWidth="1" width="14.5546875"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="str">
         <v>【1】整體進度</v>
       </c>
-      <c r="B1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G1" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H1" s="5" t="str">
+      <c r="B1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G1" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H1" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Sheet 名稱</v>
       </c>
-      <c r="B2" s="7" t="str">
+      <c r="B2" s="5" t="str">
         <v>總計</v>
       </c>
-      <c r="C2" s="7" t="str">
+      <c r="C2" s="5" t="str">
         <v>已修正</v>
       </c>
-      <c r="D2" s="7" t="str">
+      <c r="D2" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="E2" s="7" t="str">
+      <c r="E2" s="5" t="str">
         <v>待處理</v>
       </c>
-      <c r="F2" s="7" t="str">
+      <c r="F2" s="5" t="str">
         <v>完成率</v>
       </c>
-      <c r="G2" s="7" t="str">
+      <c r="G2" s="5" t="str">
         <v>備註</v>
       </c>
-      <c r="H2" s="7" t="str">
+      <c r="H2" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="str">
+      <c r="A3" s="3" t="str">
         <v>UIUX問題追蹤清單 (前台)</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="3">
         <v>182</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="6">
         <v>124</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="7">
         <v>24</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="8">
         <v>34</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="3" t="str">
         <v>68.1%</v>
       </c>
-      <c r="G3" s="8" t="str">
+      <c r="G3" s="3" t="str">
         <v>已歷經 Round 1-4 改版</v>
       </c>
-      <c r="H3" s="8" t="str">
+      <c r="H3" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="str">
+      <c r="A4" s="3" t="str">
         <v>後臺優化 (admin)</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="3">
         <v>100</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="6">
         <v>18</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="7">
         <v>16</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="8">
         <v>66</v>
       </c>
-      <c r="F4" s="9" t="str">
+      <c r="F4" s="3" t="str">
         <v>18.0%</v>
       </c>
-      <c r="G4" s="8" t="str">
+      <c r="G4" s="3" t="str">
         <v>含後台優化規劃與進階功能建議</v>
       </c>
-      <c r="H4" s="8" t="str">
+      <c r="H4" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="str">
+      <c r="A5" s="3" t="str">
         <v>PoC研究</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="3">
         <v>13</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="6">
         <v>0</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="7">
         <v>0</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="8">
         <v>13</v>
       </c>
-      <c r="F5" s="9" t="str">
+      <c r="F5" s="3" t="str">
         <v>0.0%</v>
       </c>
-      <c r="G5" s="8" t="str">
+      <c r="G5" s="3" t="str">
         <v>研究方向，未啟動</v>
       </c>
-      <c r="H5" s="8" t="str">
+      <c r="H5" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="str">
+      <c r="A7" s="4" t="str">
         <v>【2】Round 時間軸 — 每輪做了什麼</v>
       </c>
-      <c r="B7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="5" t="str">
+      <c r="B7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="str">
+      <c r="A8" s="5" t="str">
         <v>Round</v>
       </c>
-      <c r="B8" s="7" t="str">
+      <c r="B8" s="5" t="str">
         <v>日期</v>
       </c>
-      <c r="C8" s="7" t="str">
+      <c r="C8" s="5" t="str">
         <v>主題</v>
       </c>
-      <c r="D8" s="7" t="str">
+      <c r="D8" s="5" t="str">
         <v>UIUX 標完成</v>
       </c>
-      <c r="E8" s="7" t="str">
+      <c r="E8" s="5" t="str">
         <v>UIUX 新增</v>
       </c>
-      <c r="F8" s="7" t="str">
+      <c r="F8" s="5" t="str">
         <v>後臺新增</v>
       </c>
-      <c r="G8" s="7" t="str">
+      <c r="G8" s="5" t="str">
         <v>Schema</v>
       </c>
-      <c r="H8" s="7" t="str">
+      <c r="H8" s="5" t="str">
         <v>主要產出</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="str">
+      <c r="A9" s="3" t="str">
         <v>Round 1</v>
       </c>
-      <c r="B9" s="8" t="str">
+      <c r="B9" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C9" s="8" t="str">
+      <c r="C9" s="3" t="str">
         <v>UI/UX 改版 (搜尋 / Footer / 全站動畫 / RWD)</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="3">
         <v>7</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="3">
         <v>3</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="3">
         <v>0</v>
       </c>
-      <c r="G9" s="8" t="str">
+      <c r="G9" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H9" s="8" t="str">
+      <c r="H9" s="3" t="str">
         <v>pages/ifare 加關鍵字搜尋 + URL query 初始化；全站 NuxtPage transition；卡片/按鈕 hover translateY</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="str">
+      <c r="A10" s="3" t="str">
         <v>Round 2</v>
       </c>
-      <c r="B10" s="8" t="str">
+      <c r="B10" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="3" t="str">
         <v>Footer 整理 + RWD 修正</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="3">
         <v>2</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="3">
         <v>2</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="3">
         <v>0</v>
       </c>
-      <c r="G10" s="8" t="str">
+      <c r="G10" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H10" s="8" t="str">
+      <c r="H10" s="3" t="str">
         <v>LINE/FB 統一 .btn-social 並排；4 個聯絡資訊加 icon (Tel/Mail/Address/Clock)；footer 觸控 44px</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="str">
+      <c r="A11" s="3" t="str">
         <v>Round 3</v>
       </c>
-      <c r="B11" s="8" t="str">
+      <c r="B11" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="3" t="str">
         <v>About 靈動島 + News 卡片升級 + 社群外連結</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="3">
         <v>4</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="3">
         <v>5</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="3">
         <v>0</v>
       </c>
-      <c r="G11" s="8" t="str">
+      <c r="G11" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H11" s="8" t="str">
+      <c r="H11" s="3" t="str">
         <v>About 三大核心 morph 卡 (cf47cfa)；News 浮起卡 + stagger fade-up + NEW pill；外連結 target="_blank" rel="noopener"</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="str">
+      <c r="A12" s="3" t="str">
         <v>Round 4</v>
       </c>
-      <c r="B12" s="8" t="str">
+      <c r="B12" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C12" s="8" t="str">
+      <c r="C12" s="3" t="str">
         <v>切回 master + 開新分支 feat/uiux-round4 + 補做 (環境/補回/新功能)</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="3">
         <v>0</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="3">
         <v>8</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="3">
         <v>4</v>
       </c>
-      <c r="G12" s="8" t="str">
+      <c r="G12" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H12" s="8" t="str">
+      <c r="H12" s="3" t="str">
         <v>cf47cfa+5dfbf91 補回 16 檔；devProxy/baseURL → 正式 API；nav 加未來規劃 + future.vue；News videoUrl wiring；tsconfig deprecation 清理；about hover bug 修；footer label 重複修</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="str">
+      <c r="A13" s="3" t="str">
         <v>Round 5</v>
       </c>
-      <c r="B13" s="8" t="str">
+      <c r="B13" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C13" s="8" t="str">
+      <c r="C13" s="3" t="str">
         <v>前後台全面審查 — 後台 UX audit + 前台新 issue 掃描</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="3">
         <v>0</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="3">
         <v>26</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="3">
         <v>22</v>
       </c>
-      <c r="G13" s="8" t="str">
+      <c r="G13" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H13" s="8" t="str">
+      <c r="H13" s="3" t="str">
         <v>後台 22 個工程角度問題 (CRUD/驗證/錯誤處理)；前台 26 個新發現 (XSS/超時/console.log/無障礙/分頁元件重複)</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="str">
+      <c r="A14" s="3" t="str">
         <v>Round 6</v>
       </c>
-      <c r="B14" s="8" t="str">
+      <c r="B14" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C14" s="8" t="str">
+      <c r="C14" s="3" t="str">
         <v>人性化主軸提案 — 5 主軸 + 16 後台項</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="3">
         <v>0</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="3">
         <v>0</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="3">
         <v>16</v>
       </c>
-      <c r="G14" s="8" t="str">
+      <c r="G14" s="3" t="str">
         <v>+ Q 欄主軸</v>
       </c>
-      <c r="H14" s="8" t="str">
+      <c r="H14" s="3" t="str">
         <v>Dashboard 角色化 / 今日待辦 / KPI 分區；批次操作；軟刪除復原；audit log；危險操作預覽；錯誤訊息引導</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="str">
+      <c r="A15" s="3" t="str">
         <v>Round 7</v>
       </c>
-      <c r="B15" s="8" t="str">
+      <c r="B15" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C15" s="8" t="str">
+      <c r="C15" s="3" t="str">
         <v>後台進階功能建議補充</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="3">
         <v>0</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="3">
         <v>0</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="3">
         <v>8</v>
       </c>
-      <c r="G15" s="8" t="str">
+      <c r="G15" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H15" s="8" t="str">
+      <c r="H15" s="3" t="str">
         <v>補充 GA4 同步快取、任務中心、自動儲存與編輯鎖定、發布排程、審稿指派、內容健康檢查、通知中心、資產治理</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="str">
+      <c r="A16" s="3" t="str">
         <v>Round 8</v>
       </c>
-      <c r="B16" s="8" t="str">
+      <c r="B16" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C16" s="8" t="str">
+      <c r="C16" s="3" t="str">
         <v>後台首頁搜尋 + 表單欄位人性化快改</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="3">
         <v>0</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="3">
         <v>0</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="3">
         <v>0</v>
       </c>
-      <c r="G16" s="8" t="str">
+      <c r="G16" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H16" s="8" t="str">
+      <c r="H16" s="3" t="str">
         <v>HomeView 新增搜尋 / 分組 / 最近使用；PageManagement 補上 URL 預覽、狀態說明、SEO 預覽、常用標籤建議、排程快捷鍵</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="str">
+      <c r="A17" s="3" t="str">
         <v>Round 9</v>
       </c>
-      <c r="B17" s="8" t="str">
+      <c r="B17" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C17" s="8" t="str">
+      <c r="C17" s="3" t="str">
         <v>前台 future 頁空狀態版面優化</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="3">
         <v>0</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="3">
         <v>2</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="3">
         <v>0</v>
       </c>
-      <c r="G17" s="8" t="str">
+      <c r="G17" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H17" s="8" t="str">
+      <c r="H17" s="3" t="str">
         <v>future.vue 補強手機版主標換行、空狀態導引卡、上下留白與 footer CTA 銜接</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="str">
+      <c r="A18" s="3" t="str">
         <v>Round 10</v>
       </c>
-      <c r="B18" s="8" t="str">
+      <c r="B18" s="3" t="str">
         <v>2026-05-11</v>
       </c>
-      <c r="C18" s="8" t="str">
+      <c r="C18" s="3" t="str">
         <v>Round 14 第一+二批 — UIUX 細節打磨</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="3">
         <v>16</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="3">
         <v>0</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="3">
         <v>0</v>
       </c>
-      <c r="G18" s="8" t="str">
+      <c r="G18" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H18" s="8" t="str">
+      <c r="H18" s="3" t="str">
         <v>378c508 第一批 #15/36/41/48/50/58/61/71 (a11y/視覺/RWD)；a7fbf5d 第二批 #1/7/9/28/30/38/60/113 (視覺/互動補強)</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="str">
+      <c r="A19" s="3" t="str">
         <v>Round 11</v>
       </c>
-      <c r="B19" s="8" t="str">
+      <c r="B19" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C19" s="8" t="str">
+      <c r="C19" s="3" t="str">
         <v>Round 14 第三~五批 — Codex 多主題 + i-Fare 收尾 + 共用元件</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="3">
         <v>6</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="3">
         <v>0</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="3">
         <v>0</v>
       </c>
-      <c r="G19" s="8" t="str">
+      <c r="G19" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H19" s="8" t="str">
+      <c r="H19" s="3" t="str">
         <v>e0c0050 Codex 第三輪多主題；ab54066 第四批 i-Fare 收尾 6 條；0edc1c2 第五批 #67/68/70/73/82/116（完成率 65.8%→66.9%）</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="str">
+      <c r="A20" s="3" t="str">
         <v>Round 12</v>
       </c>
-      <c r="B20" s="8" t="str">
+      <c r="B20" s="3" t="str">
         <v>2026-05-18</v>
       </c>
-      <c r="C20" s="8" t="str">
+      <c r="C20" s="3" t="str">
         <v>Round 14 第六輪 — Codex 後端/SEO/Chatbot/後台大批推進</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="3">
         <v>0</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="3">
         <v>0</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="3">
         <v>0</v>
       </c>
-      <c r="G20" s="8" t="str">
+      <c r="G20" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H20" s="8" t="str">
+      <c r="H20" s="3" t="str">
         <v>93d1186 後端/SEO/Chatbot 整批；321aa91 後台優化規劃依 sheet2 54 條 backlog 分三階段；12b2271 backend page-management inline 紅框錯誤</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="str">
+      <c r="A21" s="3" t="str">
         <v>Round 13</v>
       </c>
-      <c r="B21" s="8" t="str">
+      <c r="B21" s="3" t="str">
         <v>2026-05-19</v>
       </c>
-      <c r="C21" s="8" t="str">
+      <c r="C21" s="3" t="str">
         <v>Round 14 第七~九輪 — Dashboard/PageBuilder/Loading/PoC v2</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="3">
         <v>0</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="3">
         <v>0</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="3">
         <v>0</v>
       </c>
-      <c r="G21" s="8" t="str">
+      <c r="G21" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="H21" s="8" t="str">
+      <c r="H21" s="3" t="str">
         <v>cea8433 第七輪 Codex 後台 Dashboard/PageBuilder/future 大改；20dcad6 第八輪 Loading 主題 (#3 useFeedback)；9a5cbca 第九輪 PageBuilder PoC v2 升級（自動同步 + SSR）</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="str">
+      <c r="A22" s="3" t="str">
         <v>Round 14</v>
       </c>
-      <c r="B22" s="8" t="str">
+      <c r="B22" s="3" t="str">
         <v>2026-05-25</v>
       </c>
-      <c r="C22" s="8" t="str">
+      <c r="C22" s="3" t="str">
         <v>page-management UX 收尾 + dynamic page 資安加固 + critical audit</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="3">
         <v>2</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="3">
         <v>8</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="3">
         <v>0</v>
       </c>
-      <c r="G22" s="8" t="str">
+      <c r="G22" s="3" t="str">
         <v>+ #175-182</v>
       </c>
-      <c r="H22" s="8" t="str">
+      <c r="H22" s="3" t="str">
         <v>4a953bd/c93db5f/507b9ca/d7246a6 page-management 操作列升級；ae1c85a #175 部分修正 (dynamic API token + CORS 白名單)、#181 部分修正 (.env runtime config)；770e517 新增 audit issues #175-182</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="str">
+      <c r="A24" s="4" t="str">
         <v>【3】後臺優化 — 5 主軸分布 (拿這個去提案!)</v>
       </c>
-      <c r="B24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G24" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H24" s="5" t="str">
+      <c r="B24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G24" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H24" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="str">
+      <c r="A25" s="5" t="str">
         <v>主軸</v>
       </c>
-      <c r="B25" s="7" t="str">
+      <c r="B25" s="5" t="str">
         <v>項目數</v>
       </c>
-      <c r="C25" s="7" t="str">
+      <c r="C25" s="5" t="str">
         <v>比例</v>
       </c>
-      <c r="D25" s="7" t="str">
+      <c r="D25" s="5" t="str">
         <v>主要訴求</v>
       </c>
-      <c r="E25" s="7" t="str">
+      <c r="E25" s="5" t="str">
         <v>對應 #</v>
       </c>
-      <c r="F25" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G25" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H25" s="7" t="str">
+      <c r="F25" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G25" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H25" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="str">
+      <c r="A26" s="3" t="str">
         <v>看得懂</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="3">
         <v>18</v>
       </c>
-      <c r="C26" s="9" t="str">
+      <c r="C26" s="3" t="str">
         <v>18.0%</v>
       </c>
-      <c r="D26" s="8" t="str">
+      <c r="D26" s="3" t="str">
         <v>首頁先給重點 / KPI / 異常 / 待辦分區 / 欄位白話 / 狀態流程視覺化</v>
       </c>
-      <c r="E26" s="8" t="str">
+      <c r="E26" s="3" t="str">
         <v>#1, #7, #10, #17, #19, #24, #25, #27, #32, #35, #37, #38, #39, #40, #41, #45, #49</v>
       </c>
-      <c r="F26" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G26" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H26" s="8" t="str">
+      <c r="F26" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G26" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H26" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="str">
+      <c r="A27" s="3" t="str">
         <v>找得到</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="3">
         <v>7</v>
       </c>
-      <c r="C27" s="9" t="str">
+      <c r="C27" s="3" t="str">
         <v>7.0%</v>
       </c>
-      <c r="D27" s="8" t="str">
+      <c r="D27" s="3" t="str">
         <v>全域搜尋 / 麵包屑 / 側邊欄高亮 / 變更密碼入口</v>
       </c>
-      <c r="E27" s="8" t="str">
+      <c r="E27" s="3" t="str">
         <v>#6, #29, #30, #33, #44</v>
       </c>
-      <c r="F27" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G27" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H27" s="8" t="str">
+      <c r="F27" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G27" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H27" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="str">
+      <c r="A28" s="3" t="str">
         <v>做得快</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="3">
         <v>11</v>
       </c>
-      <c r="C28" s="9" t="str">
+      <c r="C28" s="3" t="str">
         <v>11.0%</v>
       </c>
-      <c r="D28" s="8" t="str">
+      <c r="D28" s="3" t="str">
         <v>批次操作 / 儲存搜尋 / 大列表 lazy / 匯出進度 / 日期快捷</v>
       </c>
-      <c r="E28" s="8" t="str">
+      <c r="E28" s="3" t="str">
         <v>#3, #11, #20, #26, #28, #42, #43, #53, #54</v>
       </c>
-      <c r="F28" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G28" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H28" s="8" t="str">
+      <c r="F28" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G28" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H28" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="str">
+      <c r="A29" s="3" t="str">
         <v>不容易錯</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="3">
         <v>18</v>
       </c>
-      <c r="C29" s="9" t="str">
+      <c r="C29" s="3" t="str">
         <v>18.0%</v>
       </c>
-      <c r="D29" s="8" t="str">
+      <c r="D29" s="3" t="str">
         <v>表單驗證 / 刪除確認 / 影響預覽 / 預設值 / 錯誤引導</v>
       </c>
-      <c r="E29" s="8" t="str">
+      <c r="E29" s="3" t="str">
         <v>#2, #4, #5, #15, #18, #21, #22, #23, #31, #34, #36, #46, #47, #48</v>
       </c>
-      <c r="F29" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G29" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H29" s="8" t="str">
+      <c r="F29" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G29" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H29" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="str">
+      <c r="A30" s="3" t="str">
         <v>出事能追回來</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="3">
         <v>8</v>
       </c>
-      <c r="C30" s="9" t="str">
+      <c r="C30" s="3" t="str">
         <v>8.0%</v>
       </c>
-      <c r="D30" s="8" t="str">
+      <c r="D30" s="3" t="str">
         <v>audit log / 變更歷史 / 軟刪除復原 / token 管理 / 文件交接</v>
       </c>
-      <c r="E30" s="8" t="str">
+      <c r="E30" s="3" t="str">
         <v>#9, #12, #50, #51, #52</v>
       </c>
-      <c r="F30" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G30" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H30" s="8" t="str">
+      <c r="F30" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G30" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H30" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="str">
+      <c r="A31" s="3" t="str">
         <v>—</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="3">
         <v>25</v>
       </c>
-      <c r="C31" s="9" t="str">
+      <c r="C31" s="3" t="str">
         <v>25.0%</v>
       </c>
-      <c r="D31" s="8" t="str">
+      <c r="D31" s="3" t="str">
         <v>純技術 / 環境設定 (不在 5 主軸範圍)</v>
       </c>
-      <c r="E31" s="8" t="str">
+      <c r="E31" s="3" t="str">
         <v>#8, #13, #14, #16</v>
       </c>
-      <c r="F31" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G31" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H31" s="8" t="str">
+      <c r="F31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G31" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H31" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="str">
+      <c r="A33" s="4" t="str">
         <v>【4】UIUX — 優先級 × 狀態分布</v>
       </c>
-      <c r="B33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G33" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H33" s="5" t="str">
+      <c r="B33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G33" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H33" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="str">
+      <c r="A34" s="5" t="str">
         <v>優先級</v>
       </c>
-      <c r="B34" s="7" t="str">
+      <c r="B34" s="5" t="str">
         <v>已修正</v>
       </c>
-      <c r="C34" s="7" t="str">
+      <c r="C34" s="5" t="str">
         <v>部分修正</v>
       </c>
-      <c r="D34" s="7" t="str">
+      <c r="D34" s="5" t="str">
         <v>待處理</v>
       </c>
-      <c r="E34" s="7" t="str">
+      <c r="E34" s="5" t="str">
         <v>小計</v>
       </c>
-      <c r="F34" s="7" t="str">
+      <c r="F34" s="5" t="str">
         <v>完成率</v>
       </c>
-      <c r="G34" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H34" s="7" t="str">
+      <c r="G34" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H34" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="str">
+      <c r="A35" s="3" t="str">
         <v>高</v>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="6">
         <v>23</v>
       </c>
-      <c r="C35" s="14">
+      <c r="C35" s="7">
         <v>12</v>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="8">
         <v>9</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="3">
         <v>44</v>
       </c>
-      <c r="F35" s="9" t="str">
+      <c r="F35" s="3" t="str">
         <v>65.9%</v>
       </c>
-      <c r="G35" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H35" s="8" t="str">
+      <c r="G35" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H35" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="str">
+      <c r="A36" s="3" t="str">
         <v>中</v>
       </c>
-      <c r="B36" s="13">
+      <c r="B36" s="6">
         <v>61</v>
       </c>
-      <c r="C36" s="14">
+      <c r="C36" s="7">
         <v>8</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="8">
         <v>14</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="3">
         <v>83</v>
       </c>
-      <c r="F36" s="9" t="str">
+      <c r="F36" s="3" t="str">
         <v>78.3%</v>
       </c>
-      <c r="G36" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H36" s="8" t="str">
+      <c r="G36" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H36" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="str">
+      <c r="A37" s="3" t="str">
         <v>低</v>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="6">
         <v>40</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C37" s="7">
         <v>4</v>
       </c>
-      <c r="D37" s="15">
+      <c r="D37" s="8">
         <v>11</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="3">
         <v>55</v>
       </c>
-      <c r="F37" s="9" t="str">
+      <c r="F37" s="3" t="str">
         <v>76.4%</v>
       </c>
-      <c r="G37" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H37" s="8" t="str">
+      <c r="G37" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H37" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="str">
+      <c r="A39" s="4" t="str">
         <v>【5】UIUX — 各區塊問題分布</v>
       </c>
-      <c r="B39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G39" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H39" s="5" t="str">
+      <c r="B39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G39" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H39" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="str">
+      <c r="A40" s="5" t="str">
         <v>區塊</v>
       </c>
-      <c r="B40" s="7" t="str">
+      <c r="B40" s="5" t="str">
         <v>項目數</v>
       </c>
-      <c r="C40" s="7" t="str">
+      <c r="C40" s="5" t="str">
         <v>佔比</v>
       </c>
-      <c r="D40" s="7" t="str">
-        <v/>
-      </c>
-      <c r="E40" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F40" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G40" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H40" s="7" t="str">
+      <c r="D40" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E40" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F40" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G40" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H40" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="str">
+      <c r="A41" s="3" t="str">
         <v>全站通用</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="3">
         <v>43</v>
       </c>
-      <c r="C41" s="9" t="str">
+      <c r="C41" s="3" t="str">
         <v>23.6%</v>
       </c>
-      <c r="D41" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E41" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F41" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G41" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H41" s="8" t="str">
+      <c r="D41" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E41" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F41" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G41" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H41" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="str">
+      <c r="A42" s="3" t="str">
         <v>i-Fare 福利查詢</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="3">
         <v>30</v>
       </c>
-      <c r="C42" s="9" t="str">
+      <c r="C42" s="3" t="str">
         <v>16.5%</v>
       </c>
-      <c r="D42" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E42" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F42" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G42" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H42" s="8" t="str">
+      <c r="D42" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E42" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F42" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G42" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H42" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="str">
+      <c r="A43" s="3" t="str">
         <v>共用元件</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="3">
         <v>25</v>
       </c>
-      <c r="C43" s="9" t="str">
+      <c r="C43" s="3" t="str">
         <v>13.7%</v>
       </c>
-      <c r="D43" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E43" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F43" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G43" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H43" s="8" t="str">
+      <c r="D43" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E43" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F43" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G43" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H43" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="str">
+      <c r="A44" s="3" t="str">
         <v>福利專欄</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="3">
         <v>11</v>
       </c>
-      <c r="C44" s="9" t="str">
+      <c r="C44" s="3" t="str">
         <v>6.0%</v>
       </c>
-      <c r="D44" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E44" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F44" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G44" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H44" s="8" t="str">
+      <c r="D44" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E44" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F44" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G44" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H44" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="str">
+      <c r="A45" s="3" t="str">
         <v>首頁</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="3">
         <v>10</v>
       </c>
-      <c r="C45" s="9" t="str">
+      <c r="C45" s="3" t="str">
         <v>5.5%</v>
       </c>
-      <c r="D45" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E45" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F45" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G45" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H45" s="8" t="str">
+      <c r="D45" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E45" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F45" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G45" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H45" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="str">
+      <c r="A46" s="3" t="str">
         <v>關於長穩</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="3">
         <v>9</v>
       </c>
-      <c r="C46" s="9" t="str">
+      <c r="C46" s="3" t="str">
         <v>4.9%</v>
       </c>
-      <c r="D46" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E46" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F46" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G46" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H46" s="8" t="str">
+      <c r="D46" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E46" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F46" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G46" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H46" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="str">
+      <c r="A47" s="3" t="str">
         <v>最新消息</v>
       </c>
-      <c r="B47" s="9">
+      <c r="B47" s="3">
         <v>8</v>
       </c>
-      <c r="C47" s="9" t="str">
+      <c r="C47" s="3" t="str">
         <v>4.4%</v>
       </c>
-      <c r="D47" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E47" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F47" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G47" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H47" s="8" t="str">
+      <c r="D47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G47" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H47" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="str">
+      <c r="A48" s="3" t="str">
         <v>公益夥伴</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="3">
         <v>8</v>
       </c>
-      <c r="C48" s="9" t="str">
+      <c r="C48" s="3" t="str">
         <v>4.4%</v>
       </c>
-      <c r="D48" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E48" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F48" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G48" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H48" s="8" t="str">
+      <c r="D48" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E48" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F48" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G48" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H48" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="str">
+      <c r="A49" s="3" t="str">
         <v>全站微互動</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="3">
         <v>5</v>
       </c>
-      <c r="C49" s="9" t="str">
+      <c r="C49" s="3" t="str">
         <v>2.7%</v>
       </c>
-      <c r="D49" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E49" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F49" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G49" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H49" s="8" t="str">
+      <c r="D49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G49" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H49" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="str">
+      <c r="A50" s="3" t="str">
         <v>設計系統</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="3">
         <v>5</v>
       </c>
-      <c r="C50" s="9" t="str">
+      <c r="C50" s="3" t="str">
         <v>2.7%</v>
       </c>
-      <c r="D50" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E50" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F50" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G50" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H50" s="8" t="str">
+      <c r="D50" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E50" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F50" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G50" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H50" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="str">
+      <c r="A51" s="3" t="str">
         <v>未來規劃</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="3">
         <v>3</v>
       </c>
-      <c r="C51" s="9" t="str">
+      <c r="C51" s="3" t="str">
         <v>1.6%</v>
       </c>
-      <c r="D51" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E51" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F51" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G51" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H51" s="8" t="str">
+      <c r="D51" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E51" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F51" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G51" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H51" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="str">
+      <c r="A52" s="3" t="str">
         <v>i-Fare 福利詳情</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="3">
         <v>3</v>
       </c>
-      <c r="C52" s="9" t="str">
+      <c r="C52" s="3" t="str">
         <v>1.6%</v>
       </c>
-      <c r="D52" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E52" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F52" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G52" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H52" s="8" t="str">
+      <c r="D52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G52" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H52" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="str">
+      <c r="A53" s="3" t="str">
         <v>安全性</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53" s="3">
         <v>2</v>
       </c>
-      <c r="C53" s="9" t="str">
+      <c r="C53" s="3" t="str">
         <v>1.1%</v>
       </c>
-      <c r="D53" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E53" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F53" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G53" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H53" s="8" t="str">
+      <c r="D53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G53" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H53" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="str">
+      <c r="A54" s="3" t="str">
         <v>無障礙</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="3">
         <v>2</v>
       </c>
-      <c r="C54" s="9" t="str">
+      <c r="C54" s="3" t="str">
         <v>1.1%</v>
       </c>
-      <c r="D54" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E54" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F54" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G54" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H54" s="8" t="str">
+      <c r="D54" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E54" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F54" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G54" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H54" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="str">
+      <c r="A55" s="3" t="str">
         <v>後台 API</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55" s="3">
         <v>2</v>
       </c>
-      <c r="C55" s="9" t="str">
+      <c r="C55" s="3" t="str">
         <v>1.1%</v>
       </c>
-      <c r="D55" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E55" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F55" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G55" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H55" s="8" t="str">
+      <c r="D55" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E55" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F55" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G55" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H55" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="str">
+      <c r="A56" s="3" t="str">
         <v>頁面導航</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="3">
         <v>1</v>
       </c>
-      <c r="C56" s="9" t="str">
+      <c r="C56" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D56" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E56" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F56" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G56" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H56" s="8" t="str">
+      <c r="D56" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E56" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F56" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G56" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H56" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="str">
+      <c r="A57" s="3" t="str">
         <v>i-Fare 搜尋結果</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="3">
         <v>1</v>
       </c>
-      <c r="C57" s="9" t="str">
+      <c r="C57" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D57" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E57" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F57" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G57" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H57" s="8" t="str">
+      <c r="D57" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E57" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F57" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G57" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H57" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="str">
+      <c r="A58" s="3" t="str">
         <v>效能</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="3">
         <v>1</v>
       </c>
-      <c r="C58" s="9" t="str">
+      <c r="C58" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D58" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E58" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F58" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G58" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H58" s="8" t="str">
+      <c r="D58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G58" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H58" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="str">
+      <c r="A59" s="3" t="str">
         <v>社群分享</v>
       </c>
-      <c r="B59" s="9">
+      <c r="B59" s="3">
         <v>1</v>
       </c>
-      <c r="C59" s="9" t="str">
+      <c r="C59" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D59" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E59" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F59" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G59" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H59" s="8" t="str">
+      <c r="D59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G59" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H59" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="str">
+      <c r="A60" s="3" t="str">
         <v>導航</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="3">
         <v>1</v>
       </c>
-      <c r="C60" s="9" t="str">
+      <c r="C60" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D60" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E60" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F60" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G60" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H60" s="8" t="str">
+      <c r="D60" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E60" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F60" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G60" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H60" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="str">
+      <c r="A61" s="3" t="str">
         <v>關於我們</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="3">
         <v>1</v>
       </c>
-      <c r="C61" s="9" t="str">
+      <c r="C61" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D61" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E61" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F61" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G61" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H61" s="8" t="str">
+      <c r="D61" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E61" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F61" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G61" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H61" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="str">
+      <c r="A62" s="3" t="str">
         <v>後台</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="3">
         <v>1</v>
       </c>
-      <c r="C62" s="9" t="str">
+      <c r="C62" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D62" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E62" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F62" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G62" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H62" s="8" t="str">
+      <c r="D62" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E62" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F62" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G62" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H62" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="str">
+      <c r="A63" s="3" t="str">
         <v>preview 頁</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63" s="3">
         <v>1</v>
       </c>
-      <c r="C63" s="9" t="str">
+      <c r="C63" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D63" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E63" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F63" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G63" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H63" s="8" t="str">
+      <c r="D63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G63" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H63" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="str">
+      <c r="A64" s="3" t="str">
         <v>追蹤文件</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="3">
         <v>1</v>
       </c>
-      <c r="C64" s="9" t="str">
+      <c r="C64" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D64" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E64" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F64" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G64" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H64" s="8" t="str">
+      <c r="D64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G64" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H64" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="str">
+      <c r="A65" s="3" t="str">
         <v>i-Fare 福利政策</v>
       </c>
-      <c r="B65" s="9">
+      <c r="B65" s="3">
         <v>1</v>
       </c>
-      <c r="C65" s="9" t="str">
+      <c r="C65" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D65" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E65" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F65" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G65" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H65" s="8" t="str">
+      <c r="D65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G65" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H65" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="str">
+      <c r="A66" s="3" t="str">
         <v>前台 Nuxt Server API</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="3">
         <v>1</v>
       </c>
-      <c r="C66" s="9" t="str">
+      <c r="C66" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D66" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E66" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F66" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G66" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H66" s="8" t="str">
+      <c r="D66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G66" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H66" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="str">
+      <c r="A67" s="3" t="str">
         <v>後台 API / 帳號</v>
       </c>
-      <c r="B67" s="9">
+      <c r="B67" s="3">
         <v>1</v>
       </c>
-      <c r="C67" s="9" t="str">
+      <c r="C67" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D67" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E67" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F67" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G67" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H67" s="8" t="str">
+      <c r="D67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G67" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H67" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="str">
+      <c r="A68" s="3" t="str">
         <v>設定 / 部署</v>
       </c>
-      <c r="B68" s="9">
+      <c r="B68" s="3">
         <v>1</v>
       </c>
-      <c r="C68" s="9" t="str">
+      <c r="C68" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D68" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E68" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F68" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G68" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H68" s="8" t="str">
+      <c r="D68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G68" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H68" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="str">
+      <c r="A69" s="3" t="str">
         <v>後台前端</v>
       </c>
-      <c r="B69" s="9">
+      <c r="B69" s="3">
         <v>1</v>
       </c>
-      <c r="C69" s="9" t="str">
+      <c r="C69" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D69" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E69" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F69" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G69" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H69" s="8" t="str">
+      <c r="D69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G69" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H69" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="str">
+      <c r="A70" s="3" t="str">
         <v>環境 / API 串接</v>
       </c>
-      <c r="B70" s="9">
+      <c r="B70" s="3">
         <v>1</v>
       </c>
-      <c r="C70" s="9" t="str">
+      <c r="C70" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D70" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E70" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F70" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G70" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H70" s="8" t="str">
+      <c r="D70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G70" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H70" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="str">
+      <c r="A71" s="3" t="str">
         <v>工程流程</v>
       </c>
-      <c r="B71" s="9">
+      <c r="B71" s="3">
         <v>1</v>
       </c>
-      <c r="C71" s="9" t="str">
+      <c r="C71" s="3" t="str">
         <v>0.5%</v>
       </c>
-      <c r="D71" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E71" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F71" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G71" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H71" s="8" t="str">
+      <c r="D71" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E71" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F71" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G71" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H71" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="str">
+      <c r="A73" s="4" t="str">
         <v>【6】後臺優化 — 各區塊問題分布</v>
       </c>
-      <c r="B73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G73" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H73" s="5" t="str">
+      <c r="B73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G73" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H73" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="str">
+      <c r="A74" s="5" t="str">
         <v>區塊</v>
       </c>
-      <c r="B74" s="7" t="str">
+      <c r="B74" s="5" t="str">
         <v>項目數</v>
       </c>
-      <c r="C74" s="7" t="str">
+      <c r="C74" s="5" t="str">
         <v>佔比</v>
       </c>
-      <c r="D74" s="7" t="str">
-        <v/>
-      </c>
-      <c r="E74" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F74" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G74" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H74" s="7" t="str">
+      <c r="D74" s="5" t="str">
+        <v/>
+      </c>
+      <c r="E74" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F74" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G74" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H74" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="str">
+      <c r="A75" s="3" t="str">
         <v>後台通用</v>
       </c>
-      <c r="B75" s="9">
+      <c r="B75" s="3">
         <v>26</v>
       </c>
-      <c r="C75" s="9" t="str">
+      <c r="C75" s="3" t="str">
         <v>26.0%</v>
       </c>
-      <c r="D75" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E75" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F75" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G75" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H75" s="8" t="str">
+      <c r="D75" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E75" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F75" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G75" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H75" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="str">
+      <c r="A76" s="3" t="str">
         <v>共用元件</v>
       </c>
-      <c r="B76" s="9">
+      <c r="B76" s="3">
         <v>21</v>
       </c>
-      <c r="C76" s="9" t="str">
+      <c r="C76" s="3" t="str">
         <v>21.0%</v>
       </c>
-      <c r="D76" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E76" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F76" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G76" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H76" s="8" t="str">
+      <c r="D76" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E76" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F76" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G76" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H76" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="str">
+      <c r="A77" s="3" t="str">
         <v>i-Fare 維護</v>
       </c>
-      <c r="B77" s="9">
+      <c r="B77" s="3">
         <v>8</v>
       </c>
-      <c r="C77" s="9" t="str">
+      <c r="C77" s="3" t="str">
         <v>8.0%</v>
       </c>
-      <c r="D77" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E77" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F77" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G77" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H77" s="8" t="str">
+      <c r="D77" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E77" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F77" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G77" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H77" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="str">
+      <c r="A78" s="3" t="str">
         <v>頁面管理</v>
       </c>
-      <c r="B78" s="9">
+      <c r="B78" s="3">
         <v>8</v>
       </c>
-      <c r="C78" s="9" t="str">
+      <c r="C78" s="3" t="str">
         <v>8.0%</v>
       </c>
-      <c r="D78" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E78" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F78" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G78" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H78" s="8" t="str">
+      <c r="D78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G78" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H78" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="str">
+      <c r="A79" s="3" t="str">
         <v>資料分析</v>
       </c>
-      <c r="B79" s="9">
+      <c r="B79" s="3">
         <v>7</v>
       </c>
-      <c r="C79" s="9" t="str">
+      <c r="C79" s="3" t="str">
         <v>7.0%</v>
       </c>
-      <c r="D79" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E79" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F79" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G79" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H79" s="8" t="str">
+      <c r="D79" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E79" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F79" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G79" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H79" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="str">
+      <c r="A80" s="3" t="str">
         <v>圖片管理</v>
       </c>
-      <c r="B80" s="9">
+      <c r="B80" s="3">
         <v>4</v>
       </c>
-      <c r="C80" s="9" t="str">
+      <c r="C80" s="3" t="str">
         <v>4.0%</v>
       </c>
-      <c r="D80" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E80" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F80" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G80" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H80" s="8" t="str">
+      <c r="D80" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E80" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F80" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G80" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H80" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="str">
+      <c r="A81" s="3" t="str">
         <v>內容品質</v>
       </c>
-      <c r="B81" s="9">
+      <c r="B81" s="3">
         <v>2</v>
       </c>
-      <c r="C81" s="9" t="str">
+      <c r="C81" s="3" t="str">
         <v>2.0%</v>
       </c>
-      <c r="D81" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E81" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F81" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G81" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H81" s="8" t="str">
+      <c r="D81" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E81" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F81" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G81" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H81" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="str">
+      <c r="A82" s="3" t="str">
         <v>內容管理</v>
       </c>
-      <c r="B82" s="9">
+      <c r="B82" s="3">
         <v>2</v>
       </c>
-      <c r="C82" s="9" t="str">
+      <c r="C82" s="3" t="str">
         <v>2.0%</v>
       </c>
-      <c r="D82" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E82" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F82" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G82" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H82" s="8" t="str">
+      <c r="D82" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E82" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F82" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G82" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H82" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="str">
+      <c r="A83" s="3" t="str">
         <v>最新消息維護</v>
       </c>
-      <c r="B83" s="9">
+      <c r="B83" s="3">
         <v>1</v>
       </c>
-      <c r="C83" s="9" t="str">
+      <c r="C83" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D83" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E83" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F83" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G83" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H83" s="8" t="str">
+      <c r="D83" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E83" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F83" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G83" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H83" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="str">
+      <c r="A84" s="3" t="str">
         <v>帳戶維護 / 全站權限</v>
       </c>
-      <c r="B84" s="9">
+      <c r="B84" s="3">
         <v>1</v>
       </c>
-      <c r="C84" s="9" t="str">
+      <c r="C84" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D84" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E84" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F84" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G84" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H84" s="8" t="str">
+      <c r="D84" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E84" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F84" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G84" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H84" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="str">
+      <c r="A85" s="3" t="str">
         <v>前台通用</v>
       </c>
-      <c r="B85" s="9">
+      <c r="B85" s="3">
         <v>1</v>
       </c>
-      <c r="C85" s="9" t="str">
+      <c r="C85" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D85" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E85" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F85" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G85" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H85" s="8" t="str">
+      <c r="D85" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E85" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F85" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G85" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H85" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="str">
+      <c r="A86" s="3" t="str">
         <v>對話框</v>
       </c>
-      <c r="B86" s="9">
+      <c r="B86" s="3">
         <v>1</v>
       </c>
-      <c r="C86" s="9" t="str">
+      <c r="C86" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D86" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E86" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F86" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G86" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H86" s="8" t="str">
+      <c r="D86" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E86" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F86" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G86" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H86" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="str">
+      <c r="A87" s="3" t="str">
         <v>檔案上傳</v>
       </c>
-      <c r="B87" s="9">
+      <c r="B87" s="3">
         <v>1</v>
       </c>
-      <c r="C87" s="9" t="str">
+      <c r="C87" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D87" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E87" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F87" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G87" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H87" s="8" t="str">
+      <c r="D87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G87" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H87" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="str">
+      <c r="A88" s="3" t="str">
         <v>帳號管理</v>
       </c>
-      <c r="B88" s="9">
+      <c r="B88" s="3">
         <v>1</v>
       </c>
-      <c r="C88" s="9" t="str">
+      <c r="C88" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D88" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E88" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F88" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G88" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H88" s="8" t="str">
+      <c r="D88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G88" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H88" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="str">
+      <c r="A89" s="3" t="str">
         <v>搜尋結果</v>
       </c>
-      <c r="B89" s="9">
+      <c r="B89" s="3">
         <v>1</v>
       </c>
-      <c r="C89" s="9" t="str">
+      <c r="C89" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D89" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E89" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F89" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G89" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H89" s="8" t="str">
+      <c r="D89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G89" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H89" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="str">
+      <c r="A90" s="3" t="str">
         <v>日期選擇</v>
       </c>
-      <c r="B90" s="9">
+      <c r="B90" s="3">
         <v>1</v>
       </c>
-      <c r="C90" s="9" t="str">
+      <c r="C90" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D90" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E90" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F90" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G90" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H90" s="8" t="str">
+      <c r="D90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G90" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H90" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="str">
+      <c r="A91" s="3" t="str">
         <v>表單</v>
       </c>
-      <c r="B91" s="9">
+      <c r="B91" s="3">
         <v>1</v>
       </c>
-      <c r="C91" s="9" t="str">
+      <c r="C91" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D91" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E91" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F91" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G91" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H91" s="8" t="str">
+      <c r="D91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G91" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H91" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="str">
+      <c r="A92" s="3" t="str">
         <v>側邊欄</v>
       </c>
-      <c r="B92" s="9">
+      <c r="B92" s="3">
         <v>1</v>
       </c>
-      <c r="C92" s="9" t="str">
+      <c r="C92" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D92" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E92" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F92" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G92" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H92" s="8" t="str">
+      <c r="D92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G92" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H92" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="str">
+      <c r="A93" s="3" t="str">
         <v>麵包屑導覽</v>
       </c>
-      <c r="B93" s="9">
+      <c r="B93" s="3">
         <v>1</v>
       </c>
-      <c r="C93" s="9" t="str">
+      <c r="C93" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D93" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E93" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F93" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G93" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H93" s="8" t="str">
+      <c r="D93" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E93" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F93" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G93" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H93" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="str">
+      <c r="A94" s="3" t="str">
         <v>WebAPI</v>
       </c>
-      <c r="B94" s="9">
+      <c r="B94" s="3">
         <v>1</v>
       </c>
-      <c r="C94" s="9" t="str">
+      <c r="C94" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D94" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E94" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F94" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G94" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H94" s="8" t="str">
+      <c r="D94" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E94" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F94" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G94" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H94" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="str">
+      <c r="A95" s="3" t="str">
         <v>帳號變更密碼</v>
       </c>
-      <c r="B95" s="9">
+      <c r="B95" s="3">
         <v>1</v>
       </c>
-      <c r="C95" s="9" t="str">
+      <c r="C95" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D95" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E95" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F95" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G95" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H95" s="8" t="str">
+      <c r="D95" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E95" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F95" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G95" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H95" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="str">
+      <c r="A96" s="3" t="str">
         <v>Code 代碼管理</v>
       </c>
-      <c r="B96" s="9">
+      <c r="B96" s="3">
         <v>1</v>
       </c>
-      <c r="C96" s="9" t="str">
+      <c r="C96" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D96" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E96" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F96" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G96" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H96" s="8" t="str">
+      <c r="D96" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E96" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F96" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G96" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H96" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="str">
+      <c r="A97" s="3" t="str">
         <v>狀態管理</v>
       </c>
-      <c r="B97" s="9">
+      <c r="B97" s="3">
         <v>1</v>
       </c>
-      <c r="C97" s="9" t="str">
+      <c r="C97" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D97" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E97" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F97" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G97" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H97" s="8" t="str">
+      <c r="D97" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E97" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F97" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G97" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H97" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="str">
+      <c r="A98" s="3" t="str">
         <v>登入頁面</v>
       </c>
-      <c r="B98" s="9">
+      <c r="B98" s="3">
         <v>1</v>
       </c>
-      <c r="C98" s="9" t="str">
+      <c r="C98" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D98" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E98" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F98" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G98" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H98" s="8" t="str">
+      <c r="D98" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E98" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F98" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G98" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H98" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="str">
+      <c r="A99" s="3" t="str">
         <v>HTML 編輯器</v>
       </c>
-      <c r="B99" s="9">
+      <c r="B99" s="3">
         <v>1</v>
       </c>
-      <c r="C99" s="9" t="str">
+      <c r="C99" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D99" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E99" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F99" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G99" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H99" s="8" t="str">
+      <c r="D99" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E99" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F99" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G99" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H99" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="str">
+      <c r="A100" s="3" t="str">
         <v>無權限頁</v>
       </c>
-      <c r="B100" s="9">
+      <c r="B100" s="3">
         <v>1</v>
       </c>
-      <c r="C100" s="9" t="str">
+      <c r="C100" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D100" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E100" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F100" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G100" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H100" s="8" t="str">
+      <c r="D100" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E100" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F100" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G100" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H100" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="str">
+      <c r="A101" s="3" t="str">
         <v>效能</v>
       </c>
-      <c r="B101" s="9">
+      <c r="B101" s="3">
         <v>1</v>
       </c>
-      <c r="C101" s="9" t="str">
+      <c r="C101" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D101" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E101" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F101" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G101" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H101" s="8" t="str">
+      <c r="D101" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E101" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F101" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G101" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H101" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="str">
+      <c r="A102" s="3" t="str">
         <v>後台首頁</v>
       </c>
-      <c r="B102" s="9">
+      <c r="B102" s="3">
         <v>1</v>
       </c>
-      <c r="C102" s="9" t="str">
+      <c r="C102" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D102" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E102" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F102" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G102" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H102" s="8" t="str">
+      <c r="D102" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E102" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F102" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G102" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H102" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="str">
+      <c r="A103" s="3" t="str">
         <v>前台動態頁</v>
       </c>
-      <c r="B103" s="9">
+      <c r="B103" s="3">
         <v>1</v>
       </c>
-      <c r="C103" s="9" t="str">
+      <c r="C103" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D103" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E103" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F103" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G103" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H103" s="8" t="str">
+      <c r="D103" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E103" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F103" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G103" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H103" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="8" t="str">
+      <c r="A104" s="3" t="str">
         <v>發布流程</v>
       </c>
-      <c r="B104" s="9">
+      <c r="B104" s="3">
         <v>1</v>
       </c>
-      <c r="C104" s="9" t="str">
+      <c r="C104" s="3" t="str">
         <v>1.0%</v>
       </c>
-      <c r="D104" s="8" t="str">
-        <v/>
-      </c>
-      <c r="E104" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F104" s="8" t="str">
-        <v/>
-      </c>
-      <c r="G104" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H104" s="8" t="str">
+      <c r="D104" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E104" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F104" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G104" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H104" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="str">
+      <c r="A106" s="4" t="str">
         <v>【7】你做了什麼 — 已完成項目摘要 (依 Round 分組)</v>
       </c>
-      <c r="B106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G106" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H106" s="5" t="str">
+      <c r="B106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="C106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G106" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H106" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="7" t="str">
+      <c r="A107" s="5" t="str">
         <v>Round</v>
       </c>
-      <c r="B107" s="7" t="str">
+      <c r="B107" s="5" t="str">
         <v>日期</v>
       </c>
-      <c r="C107" s="7" t="str">
+      <c r="C107" s="5" t="str">
         <v>已修正 (綠)</v>
       </c>
-      <c r="D107" s="7" t="str">
+      <c r="D107" s="5" t="str">
         <v>部分修正 (黃)</v>
       </c>
-      <c r="E107" s="7" t="str">
+      <c r="E107" s="5" t="str">
         <v>已修正 # 清單</v>
       </c>
-      <c r="F107" s="7" t="str">
+      <c r="F107" s="5" t="str">
         <v>部分修正 # 清單</v>
       </c>
-      <c r="G107" s="7" t="str">
+      <c r="G107" s="5" t="str">
         <v>主要重點</v>
       </c>
-      <c r="H107" s="7" t="str">
+      <c r="H107" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="str">
+      <c r="A108" s="3" t="str">
         <v>Round 1</v>
       </c>
-      <c r="B108" s="8" t="str">
+      <c r="B108" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C108" s="13">
+      <c r="C108" s="6">
         <v>46</v>
       </c>
-      <c r="D108" s="14">
+      <c r="D108" s="7">
         <v>3</v>
       </c>
-      <c r="E108" s="8" t="str">
+      <c r="E108" s="3" t="str">
         <v>#3, #6, #14, #16, #17, #22, #23, #24, #29, #37, #44, #45, #46, #47, #49, #52, #53, #54, #55, #56, #59, #75, #77, #79, #88, #89, #90, #106, #108, #109, #110, #112, #114, #115, #118, #120, #125, #126, #127, #130, #131, #132, #133, #134, #135, #143</v>
       </c>
-      <c r="F108" s="8" t="str">
+      <c r="F108" s="3" t="str">
         <v>#76, #136, #144</v>
       </c>
-      <c r="G108" s="8" t="str">
+      <c r="G108" s="3" t="str">
         <v>搜尋優化 (移除 disabled / 結果摘要) + 全站動畫 + skeleton 載入 + 卡片/按鈕 hover translateY</v>
       </c>
-      <c r="H108" s="8" t="str">
+      <c r="H108" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="8" t="str">
+      <c r="A109" s="3" t="str">
         <v>Round 2</v>
       </c>
-      <c r="B109" s="8" t="str">
+      <c r="B109" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C109" s="13">
+      <c r="C109" s="6">
         <v>2</v>
       </c>
-      <c r="D109" s="14">
+      <c r="D109" s="7">
         <v>0</v>
       </c>
-      <c r="E109" s="8" t="str">
+      <c r="E109" s="3" t="str">
         <v>#91, #92</v>
       </c>
-      <c r="F109" s="8" t="str">
+      <c r="F109" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G109" s="8" t="str">
+      <c r="G109" s="3" t="str">
         <v>Footer 整合 (LINE/FB 並列 .btn-social) + 觸控目標 44px</v>
       </c>
-      <c r="H109" s="8" t="str">
+      <c r="H109" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="8" t="str">
+      <c r="A110" s="3" t="str">
         <v>Round 3</v>
       </c>
-      <c r="B110" s="8" t="str">
+      <c r="B110" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C110" s="13">
+      <c r="C110" s="6">
         <v>6</v>
       </c>
-      <c r="D110" s="14">
+      <c r="D110" s="7">
         <v>0</v>
       </c>
-      <c r="E110" s="8" t="str">
+      <c r="E110" s="3" t="str">
         <v>#26, #93, #94, #95, #96, #97</v>
       </c>
-      <c r="F110" s="8" t="str">
+      <c r="F110" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G110" s="8" t="str">
+      <c r="G110" s="3" t="str">
         <v>About 三大核心 morph 卡 + News 浮起卡 + 浮現動畫 + line-clamp + NEW pill + 社群 target="_blank"</v>
       </c>
-      <c r="H110" s="8" t="str">
+      <c r="H110" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="8" t="str">
+      <c r="A111" s="3" t="str">
         <v>Round 4</v>
       </c>
-      <c r="B111" s="8" t="str">
+      <c r="B111" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C111" s="13">
+      <c r="C111" s="6">
         <v>8</v>
       </c>
-      <c r="D111" s="14">
+      <c r="D111" s="7">
         <v>0</v>
       </c>
-      <c r="E111" s="8" t="str">
+      <c r="E111" s="3" t="str">
         <v>#98, #99, #100, #101, #102, #103, #104, #105</v>
       </c>
-      <c r="F111" s="8" t="str">
+      <c r="F111" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G111" s="8" t="str">
+      <c r="G111" s="3" t="str">
         <v>cf47cfa+5dfbf91 補回 16 檔 + 環境設定 (devProxy/baseURL) + 未來規劃 nav + News videoUrl wiring + tsconfig + about hover bug + footer label 重複</v>
       </c>
-      <c r="H111" s="8" t="str">
+      <c r="H111" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="str">
+      <c r="A112" s="3" t="str">
         <v>Round 9</v>
       </c>
-      <c r="B112" s="8" t="str">
+      <c r="B112" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C112" s="13">
+      <c r="C112" s="6">
         <v>2</v>
       </c>
-      <c r="D112" s="14">
+      <c r="D112" s="7">
         <v>0</v>
       </c>
-      <c r="E112" s="8" t="str">
+      <c r="E112" s="3" t="str">
         <v>#164, #165</v>
       </c>
-      <c r="F112" s="8" t="str">
+      <c r="F112" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="G112" s="8" t="str">
+      <c r="G112" s="3" t="str">
         <v>future.vue 補強手機版主標換行、空狀態導引卡與上下節奏，讓頁面在未上線時也有清楚下一步</v>
       </c>
-      <c r="H112" s="8" t="str">
+      <c r="H112" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="8" t="str">
+      <c r="A113" s="3" t="str">
         <v>Round 10</v>
       </c>
-      <c r="B113" s="8" t="str">
+      <c r="B113" s="3" t="str">
         <v>2026-05-11</v>
       </c>
-      <c r="C113" s="13">
+      <c r="C113" s="6">
         <v>36</v>
       </c>
-      <c r="D113" s="14">
+      <c r="D113" s="7">
         <v>2</v>
       </c>
-      <c r="E113" s="8" t="str">
+      <c r="E113" s="3" t="str">
         <v>#1, #7, #9, #15, #27, #28, #30, #31, #32, #36, #38, #40, #41, #48, #50, #58, #60, #61, #71, #113, #117, #119, #122, #123, #124, #128, #129, #149, #150, #151, #152, #153, #155, #156, #157, #159</v>
       </c>
-      <c r="F113" s="8" t="str">
+      <c r="F113" s="3" t="str">
         <v>#158, #160</v>
       </c>
-      <c r="G113" s="8" t="str">
+      <c r="G113" s="3" t="str">
         <v>Round 14 第一+二批 16 條 — a11y/視覺/RWD 細節打磨 (378c508+a7fbf5d)</v>
       </c>
-      <c r="H113" s="8" t="str">
+      <c r="H113" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="str">
+      <c r="A114" s="3" t="str">
         <v>Round 11</v>
       </c>
-      <c r="B114" s="8" t="str">
+      <c r="B114" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C114" s="13">
+      <c r="C114" s="6">
         <v>3</v>
       </c>
-      <c r="D114" s="14">
+      <c r="D114" s="7">
         <v>3</v>
       </c>
-      <c r="E114" s="8" t="str">
+      <c r="E114" s="3" t="str">
         <v>#70, #82, #116</v>
       </c>
-      <c r="F114" s="8" t="str">
+      <c r="F114" s="3" t="str">
         <v>#67, #68, #73</v>
       </c>
-      <c r="G114" s="8" t="str">
+      <c r="G114" s="3" t="str">
         <v>Round 14 第三~五批 — Codex 多主題 + i-Fare 收尾 + 共用元件 #67/68/70/73/82/116 (e0c0050+ab54066+0edc1c2)</v>
       </c>
-      <c r="H114" s="8" t="str">
+      <c r="H114" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="str">
+      <c r="A115" s="3" t="str">
         <v>Round 12</v>
       </c>
-      <c r="B115" s="8" t="str">
+      <c r="B115" s="3" t="str">
         <v>2026-05-18</v>
       </c>
-      <c r="C115" s="13">
+      <c r="C115" s="6">
         <v>18</v>
       </c>
-      <c r="D115" s="14">
+      <c r="D115" s="7">
         <v>3</v>
       </c>
-      <c r="E115" s="8" t="str">
+      <c r="E115" s="3" t="str">
         <v>#2, #11, #12, #13, #80, #86, #87, #111, #137, #138, #139, #140, #145, #146, #147, #161, #162, #163</v>
       </c>
-      <c r="F115" s="8" t="str">
+      <c r="F115" s="3" t="str">
         <v>#107, #141, #142</v>
       </c>
-      <c r="G115" s="8" t="str">
+      <c r="G115" s="3" t="str">
         <v>Round 14 第六輪 — Codex 後端/SEO/Chatbot/後台大批推進 (93d1186+12b2271)</v>
       </c>
-      <c r="H115" s="8" t="str">
+      <c r="H115" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="str">
+      <c r="A116" s="3" t="str">
         <v>Round 13</v>
       </c>
-      <c r="B116" s="8" t="str">
+      <c r="B116" s="3" t="str">
         <v>2026-05-19</v>
       </c>
-      <c r="C116" s="13">
+      <c r="C116" s="6">
         <v>3</v>
       </c>
-      <c r="D116" s="14">
+      <c r="D116" s="7">
         <v>8</v>
       </c>
-      <c r="E116" s="8" t="str">
+      <c r="E116" s="3" t="str">
         <v>#148, #154, #166</v>
       </c>
-      <c r="F116" s="8" t="str">
+      <c r="F116" s="3" t="str">
         <v>#167, #168, #169, #170, #171, #172, #173, #174</v>
       </c>
-      <c r="G116" s="8" t="str">
+      <c r="G116" s="3" t="str">
         <v>Round 14 第七~九輪 — Dashboard/PageBuilder/Loading/PoC v2 (cea8433+20dcad6+9a5cbca)</v>
       </c>
-      <c r="H116" s="8" t="str">
+      <c r="H116" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="str">
+      <c r="A117" s="3" t="str">
         <v>Round 14</v>
       </c>
-      <c r="B117" s="8" t="str">
+      <c r="B117" s="3" t="str">
         <v>2026-05-25</v>
       </c>
-      <c r="C117" s="13">
+      <c r="C117" s="6">
         <v>0</v>
       </c>
-      <c r="D117" s="14">
+      <c r="D117" s="7">
         <v>5</v>
       </c>
-      <c r="E117" s="8" t="str">
+      <c r="E117" s="3" t="str">
         <v>-</v>
       </c>
-      <c r="F117" s="8" t="str">
+      <c r="F117" s="3" t="str">
         <v>#74, #83, #85, #175, #181</v>
       </c>
-      <c r="G117" s="8" t="str">
+      <c r="G117" s="3" t="str">
         <v>page-management UX 收尾 + dynamic page 資安加固 (#175/#181 部分修正) + 新增 critical audit #175-182</v>
       </c>
-      <c r="H117" s="8" t="str">
+      <c r="H117" s="3" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracking): Round 14 第九-十一批 xlsx 標記 — 後台新增頁面 UX 完工
後臺優化 sheet（共更新 12 條）:
- 已修正：#91 / #92 / #93 / #94 / #95 / #96 / #97
- 部分修正：#98（白話化首批）
- 加備註：#63 / #65 / #66（既有已修正 + 今日補強）

UIUX 問題追蹤清單 sheet:
- #181 部分修正（PreviewPane env var 補最後一處硬寫）

進度: 後臺優化 25 已修正 / 17 部分修正 / 58 待處理（共 100）
xlsx: 496KB → 127KB（compact-xlsx-theme 壓 theme1.xml 後 slim）
3 個 marker scripts 留存供審計

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -77,14 +77,9 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -4533,10 +4528,10 @@
         <v>已修正</v>
       </c>
       <c r="O66" s="3" t="str">
-        <v>2026-05-18</v>
+        <v>2026-05-19</v>
       </c>
       <c r="P66" s="3" t="str">
-        <v>純 CSS 改動，不動 script / template；保留 in-progress 的 autosave / draft / slug 邏輯</v>
+        <v>2026-05-19 完成預覽區寬度 / 字斷 / 斷點細化基本版。2026-05-25 補：(1) layout.preview-open 斷點 1440px→1600px 涵蓋一般筆電 1366-1500 視窗下預覽開啟時 edit-pane 仍會被擠的場景；(2) basic-grid &gt; * 移除 overflow-wrap:anywhere（中文逐字斷直書元凶），input-title 加 white-space:nowrap；(3) SectionList builder-shell 斷點 1200→1440 + canvas-head 加 flex-wrap + panel-title nowrap；(4) drop zone 浮現式設計（拖拽中才撐高 56px 橘虛線，hover 變實心橘 + 「↧ 放開插入到這裡」）；(5) SectionEditor 拖把手從 ⋮⋮ 換 6 點 SVG grip + 動態 draggable 避免擋表單輸入 + 收合 toolbar 整條可拖。</v>
       </c>
     </row>
     <row r="67" ht="14.4" customHeight="1">
@@ -4633,10 +4628,10 @@
         <v>已修正</v>
       </c>
       <c r="O68" s="3" t="str">
-        <v>2026-05-18</v>
+        <v>2026-05-19</v>
       </c>
       <c r="P68" s="3" t="str">
-        <v>未用 computed（draftStatusTitle 等）與對應 SCSS 暫保留作未來素材，要徹底清理可另開</v>
+        <v>2026-05-19 完成視覺瘦身（刪 quick-start-head / draft-status / status-explainer 三段純說明性卡片）。2026-05-25 補：autosave 進度顯示折衷補回 header 右上「.draft-chip」小膠囊（saving 橘 / saved 綠 / restored 藍），約 32x100px 不擾畫面，使用者仍能看到「草稿暫存中… / 已暫存 14:32 / 已還原草稿」狀態。SCSS .draft-status 大卡片保留刪除，未復原。</v>
       </c>
     </row>
     <row r="69" ht="14.4" customHeight="1">
@@ -4683,10 +4678,10 @@
         <v>已修正</v>
       </c>
       <c r="O69" s="3" t="str">
-        <v>2026-05-18</v>
+        <v>2026-05-19</v>
       </c>
       <c r="P69" s="3" t="str">
-        <v>dev only — prod 上線要把 Nuxt server JSON 中介層換成 .NET API（已在 frontendSync 預留 VITE_FRONTEND_SYNC_URL env var）；Day2-fix toast 偵測 status=draft 改顯示 warning 提示前端不顯示；發布排程 worker、slug 衝突、多人協作互蓋、預設改回 draft + 審核工作流 仍未做</v>
+        <v>2026-05-19 完成 fire-and-forget PUT 同步 + successWithLink toast。2026-05-25 補：frontendSync.ts 改 async 回 Promise&lt;SyncResult&gt;，writeAll 內部仍 fire-and-forget 但結果記入 lastSyncPromise；useDynamicPages export waitForLastSync；AddEditView.onSave 改 async 在 insert/update 後 await 結果，失敗顯示 9 秒橘 toast「已寫入後台，但同步前台失敗：xxx，請確認 dev server 已啟動」，解掉「儲存成功但前台 404」假成功問題。</v>
       </c>
     </row>
     <row r="70" ht="14.4" customHeight="1">
@@ -5976,13 +5971,13 @@
         <v>新增功能規劃，需驗證使用者不看文件也能建立一頁。</v>
       </c>
       <c r="N94" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O94" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P94" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，應先支援活動頁與服務介紹頁兩種用途。</v>
+        <v>2026-05-25：DataListView「快速新增頁面」對話框改造成 5 題答題式 wizard：Q1 用途（介紹/活動報名/公告/聯絡/自由）→ Q2 標題 → Q3 區塊多選（依用途自動預選） → Q4 主要 CTA 文字+連結 → Q5 草稿/立即發布。submitQuickCreate 直接 insert + 自動帶入 Hero 標題、CTA 區塊內容、image-text 左右交錯、slug 自動避衝突，跳轉編輯頁時頁面已組好。</v>
       </c>
       <c r="Q94" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6030,13 +6025,13 @@
         <v>新增功能規劃，需確認範本套用後可正常預覽與儲存。</v>
       </c>
       <c r="N95" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O95" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P95" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，可先用前端常數範本，後續再改為後台可管理。</v>
+        <v>2026-05-25：兩條一起補完 — (1) pagePresets 從 4 個（blank/story/service/campaign）擴到 7 個，新增 event 活動報名頁 / news 最新公告頁 / contact 聯絡頁，AddEditView + DataListView 同步；(2) SectionList 加「常用組合」卡（藍色 badge），4 個一鍵插入：📖介紹組 / 🎯服務介紹組 / 🎟️活動報名組 / ✨故事敘述組（自動左右交錯）。SECTION_COMBOS + buildSectionsFromCombo 抽到 useDynamicPages.ts。</v>
       </c>
       <c r="Q95" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6085,13 +6080,13 @@
         <v>新增功能規劃，需驗證複製內容不會共用原 slug 或發布狀態。</v>
       </c>
       <c r="N96" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O96" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P96" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，適合活動頁與公告維護。</v>
+        <v>2026-05-25：useDynamicPages 加 duplicate(id) — 深拷整筆 + id/section.id 重生 + title 加「副本」+ slug 自動避衝突（-copy / -copy-2…）+ status 強制 draft + publishTime 清空 + createDate/updateDate now。DataListView「複製新增」鈕改名「另存新頁」，呼叫 duplicate 後直接跳編輯頁，不再用 query 假複製造成 sections/meta/cover/tags 全丟失。</v>
       </c>
       <c r="Q96" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6139,13 +6134,13 @@
         <v>新增功能規劃，需驗證提示項目能在儲存前即時更新。</v>
       </c>
       <c r="N97" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O97" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P97" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。能把內容健康檢查從事後掃描提前到編輯當下。</v>
+        <v>2026-05-25 三輪迭代全部完成：(1) 第一版 — AddEditView「完成度檢查」卡，6 個動態檢查項（title/slug/sections 必填紅；metaDescription/coverImage 建議橘；imageAlt/ctaLink 條件出現）+ progress bar + 整體狀態文字。(2) B — chip 變按鈕，點擊後 advanced 自動展開 + 平滑 scrollIntoView 對應欄位 + input focus。(3) B+ — imageAlt / ctaLink chip 直接跳到第一個有缺的 section（找出 form.sections 中第一個 imageSrc 有但 imageAlt 空的、或 ctaText 有但 ctaUrl 空的 section，掛 focusSectionId；SectionEditor 加 data-section-id 屬性；scrollToField 優先用 sectionId 命中後 element.click() 觸發展開）。同批配套：O slug 衝突自動建議可用替代版本（-2/-3，跳過已佔用的）；P 多錯誤 onSave 自動 scrollToField 第一個錯誤欄位。下一步若要：擴充欄位範圍（如 unpublishTime data-focus、區塊內部欄位 anchor）。</v>
       </c>
       <c r="Q97" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6194,13 +6189,13 @@
         <v>新增功能規劃，需驗證上傳後可直接被前台載入。</v>
       </c>
       <c r="N98" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O98" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P98" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，承接媒體資產治理但更偏日常維護操作。</v>
+        <v>2026-05-25：建立共用 ImagePicker.vue（src/components/PageBuilder/）— 3 個 tab：(1) 🖼️ 媒體庫 grid 顯示已上傳 dynamic-assets，含縮圖 / 檔名 / 大小 / 時間；(2) ⬆️ 上傳新圖片，拖放或點擊上傳，自動 POST /api/dynamic-assets；(3) 🔗 貼網址（驗 https?://）。Nuxt 端新增 GET /api/dynamic-assets 端點（server/api/dynamic-assets.get.ts）列出資料夾內檔案。AddEditView 封面圖 + 社群分享圖 + SectionEditor 圖文區塊 imageSrc 三處全部換成 ImagePicker。</v>
       </c>
       <c r="Q98" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6248,13 +6243,13 @@
         <v>新增功能規劃，需驗證內部連結能正確導到前台路由。</v>
       </c>
       <c r="N99" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O99" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P99" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。能大幅降低壞連結與手動輸入錯誤。</v>
+        <v>2026-05-25：建立共用 LinkPicker.vue — 3 個 tab：(1) 📄 後台動態頁列表（從 useDynamicPages.pages 自動取，可搜尋，顯示 slug + 狀態 tag）；(2) 🏠 站內固定頁（7 個：/、/about、/news、/collaborator、/ifare、/contact、/future）；(3) 🌐 外部連結（驗 https?://）。SectionEditor 圖文 ctaUrl + 雙欄 CTA cards[*].ctaUrl 兩處全部換成 LinkPicker。開啟時自動偵測現值切到對應 tab。</v>
       </c>
       <c r="Q99" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6302,13 +6297,13 @@
         <v>新增功能規劃，需驗證發布前可擋下缺圖片/缺連結等常見問題。</v>
       </c>
       <c r="N100" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O100" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P100" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。MVP 優先，適合部署前後降低發布錯誤。</v>
+        <v>2026-05-25：AddEditView.onSave 在 validation 通過、進入 saving 前加 checklist modal — 只在 form.status === "published" 且 completenessWarnCount &gt; 0 時觸發。Modal 用 ElMessageBox.confirm + dangerouslyUseHTMLString 列出所有 warn chips（如 SEO 描述太短 / 缺封面 / 缺圖 alt / CTA 缺連結），confirmButton「我知道，繼續發布」、cancelButton「返回修改」。必填沒過會被 validatePage 提前擋；草稿模式不會彈；全綠也不彈。</v>
       </c>
       <c r="Q100" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -6356,13 +6351,13 @@
         <v>新增功能規劃，需以維護者能否理解欄位用途驗證。</v>
       </c>
       <c r="N101" s="3" t="str">
-        <v>待處理</v>
+        <v>部分修正</v>
       </c>
       <c r="O101" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P101" s="3" t="str">
-        <v>2026-05-19：因後續維護者無程式基礎，新增「非工程人員網站維護模式」項目。可與表單驗證 helper、欄位提示一起逐頁套用。</v>
+        <v>2026-05-25 首批：(1) AddEditView slug 欄位 label「URL Slug」→「頁面網址」；(2) DataList 表格欄「URL Slug」→「頁面網址」；(3) AddEditView 進階「分享圖（OG Image）」→「社群分享圖」placeholder 補一句「也叫 OG image」；(4) useDynamicPages.validatePage 三條 slug 相關錯誤訊息「URL Slug ...」→「頁面網址 ...」；(5) AddEditView.getSlugValidationMessage 兩條同步改。其他術語（isEnabled / state_data / UpdateUserId / discontinuedTime / meta description）尚未動，跨模組（News/Policy/Account）需另外盤點與設計討論。</v>
       </c>
       <c r="Q101" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -15785,7 +15780,7 @@
         <v>2026-05-25</v>
       </c>
       <c r="P183" s="3" t="str">
-        <v>2026-05-25 commit ae1c85a：iFare_Frontend 補 .env.example + nuxt.config runtime config (dynamicApiToken / dynamicApiAllowedOrigins)、iFare_Backend 補 .env.example。後台 src/plugins/AjaxRef.ts 仍硬寫正式 API URL 未處理。</v>
+        <v>2026-04-13 部分修正 dev/staging 設定。2026-05-25 補最後一處：PreviewPane.vue line 66-68 FRONTEND_URL 原寫死 http://localhost:3000，改讀 import.meta.env.VITE_FRONTEND_BASE（其他檔案如 AddEditView / DataListView / SectionEditor / frontendSync 都已用 env var，這個漏網）。後續正式部署只需設 VITE_FRONTEND_BASE=https://prod.example.com。</v>
       </c>
     </row>
     <row r="184" xml:space="preserve">
@@ -15868,54 +15863,54 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="3" t="str">
         <v>【1】整體進度</v>
       </c>
-      <c r="B1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G1" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H1" s="4" t="str">
+      <c r="B1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G1" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H1" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="3" t="str">
         <v>Sheet 名稱</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="3" t="str">
         <v>總計</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="3" t="str">
         <v>已修正</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="3" t="str">
         <v>部分修正</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="3" t="str">
         <v>待處理</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="3" t="str">
         <v>完成率</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="3" t="str">
         <v>備註</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -15926,13 +15921,13 @@
       <c r="B3" s="3">
         <v>182</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>124</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="3">
         <v>24</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="3">
         <v>34</v>
       </c>
       <c r="F3" s="3" t="str">
@@ -15952,13 +15947,13 @@
       <c r="B4" s="3">
         <v>100</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>18</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="3">
         <v>16</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="3">
         <v>66</v>
       </c>
       <c r="F4" s="3" t="str">
@@ -15978,13 +15973,13 @@
       <c r="B5" s="3">
         <v>13</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="3">
         <v>0</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="3">
         <v>13</v>
       </c>
       <c r="F5" s="3" t="str">
@@ -15998,54 +15993,54 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="3" t="str">
         <v>【2】Round 時間軸 — 每輪做了什麼</v>
       </c>
-      <c r="B7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="4" t="str">
+      <c r="B7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
+      <c r="A8" s="3" t="str">
         <v>Round</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B8" s="3" t="str">
         <v>日期</v>
       </c>
-      <c r="C8" s="5" t="str">
+      <c r="C8" s="3" t="str">
         <v>主題</v>
       </c>
-      <c r="D8" s="5" t="str">
+      <c r="D8" s="3" t="str">
         <v>UIUX 標完成</v>
       </c>
-      <c r="E8" s="5" t="str">
+      <c r="E8" s="3" t="str">
         <v>UIUX 新增</v>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="3" t="str">
         <v>後臺新增</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="3" t="str">
         <v>Schema</v>
       </c>
-      <c r="H8" s="5" t="str">
+      <c r="H8" s="3" t="str">
         <v>主要產出</v>
       </c>
     </row>
@@ -16414,54 +16409,54 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="str">
+      <c r="A24" s="3" t="str">
         <v>【3】後臺優化 — 5 主軸分布 (拿這個去提案!)</v>
       </c>
-      <c r="B24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G24" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H24" s="4" t="str">
+      <c r="B24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G24" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H24" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="str">
+      <c r="A25" s="3" t="str">
         <v>主軸</v>
       </c>
-      <c r="B25" s="5" t="str">
+      <c r="B25" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C25" s="5" t="str">
+      <c r="C25" s="3" t="str">
         <v>比例</v>
       </c>
-      <c r="D25" s="5" t="str">
+      <c r="D25" s="3" t="str">
         <v>主要訴求</v>
       </c>
-      <c r="E25" s="5" t="str">
+      <c r="E25" s="3" t="str">
         <v>對應 #</v>
       </c>
-      <c r="F25" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G25" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H25" s="5" t="str">
+      <c r="F25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G25" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H25" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -16622,54 +16617,54 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="str">
+      <c r="A33" s="3" t="str">
         <v>【4】UIUX — 優先級 × 狀態分布</v>
       </c>
-      <c r="B33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G33" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H33" s="4" t="str">
+      <c r="B33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G33" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H33" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="str">
+      <c r="A34" s="3" t="str">
         <v>優先級</v>
       </c>
-      <c r="B34" s="5" t="str">
+      <c r="B34" s="3" t="str">
         <v>已修正</v>
       </c>
-      <c r="C34" s="5" t="str">
+      <c r="C34" s="3" t="str">
         <v>部分修正</v>
       </c>
-      <c r="D34" s="5" t="str">
+      <c r="D34" s="3" t="str">
         <v>待處理</v>
       </c>
-      <c r="E34" s="5" t="str">
+      <c r="E34" s="3" t="str">
         <v>小計</v>
       </c>
-      <c r="F34" s="5" t="str">
+      <c r="F34" s="3" t="str">
         <v>完成率</v>
       </c>
-      <c r="G34" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H34" s="5" t="str">
+      <c r="G34" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H34" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -16677,13 +16672,13 @@
       <c r="A35" s="3" t="str">
         <v>高</v>
       </c>
-      <c r="B35" s="6">
+      <c r="B35" s="3">
         <v>23</v>
       </c>
-      <c r="C35" s="7">
+      <c r="C35" s="3">
         <v>12</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="3">
         <v>9</v>
       </c>
       <c r="E35" s="3">
@@ -16703,13 +16698,13 @@
       <c r="A36" s="3" t="str">
         <v>中</v>
       </c>
-      <c r="B36" s="6">
+      <c r="B36" s="3">
         <v>61</v>
       </c>
-      <c r="C36" s="7">
+      <c r="C36" s="3">
         <v>8</v>
       </c>
-      <c r="D36" s="8">
+      <c r="D36" s="3">
         <v>14</v>
       </c>
       <c r="E36" s="3">
@@ -16729,13 +16724,13 @@
       <c r="A37" s="3" t="str">
         <v>低</v>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="3">
         <v>40</v>
       </c>
-      <c r="C37" s="7">
+      <c r="C37" s="3">
         <v>4</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="3">
         <v>11</v>
       </c>
       <c r="E37" s="3">
@@ -16752,54 +16747,54 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="str">
+      <c r="A39" s="3" t="str">
         <v>【5】UIUX — 各區塊問題分布</v>
       </c>
-      <c r="B39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G39" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H39" s="4" t="str">
+      <c r="B39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G39" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H39" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="str">
+      <c r="A40" s="3" t="str">
         <v>區塊</v>
       </c>
-      <c r="B40" s="5" t="str">
+      <c r="B40" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C40" s="5" t="str">
+      <c r="C40" s="3" t="str">
         <v>佔比</v>
       </c>
-      <c r="D40" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E40" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F40" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G40" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H40" s="5" t="str">
+      <c r="D40" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E40" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F40" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G40" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H40" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -17610,54 +17605,54 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="str">
+      <c r="A73" s="3" t="str">
         <v>【6】後臺優化 — 各區塊問題分布</v>
       </c>
-      <c r="B73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G73" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H73" s="4" t="str">
+      <c r="B73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G73" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H73" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="str">
+      <c r="A74" s="3" t="str">
         <v>區塊</v>
       </c>
-      <c r="B74" s="5" t="str">
+      <c r="B74" s="3" t="str">
         <v>項目數</v>
       </c>
-      <c r="C74" s="5" t="str">
+      <c r="C74" s="3" t="str">
         <v>佔比</v>
       </c>
-      <c r="D74" s="5" t="str">
-        <v/>
-      </c>
-      <c r="E74" s="5" t="str">
-        <v/>
-      </c>
-      <c r="F74" s="5" t="str">
-        <v/>
-      </c>
-      <c r="G74" s="5" t="str">
-        <v/>
-      </c>
-      <c r="H74" s="5" t="str">
+      <c r="D74" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E74" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F74" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G74" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H74" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -18442,54 +18437,54 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="str">
+      <c r="A106" s="3" t="str">
         <v>【7】你做了什麼 — 已完成項目摘要 (依 Round 分組)</v>
       </c>
-      <c r="B106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="C106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="D106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="E106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G106" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H106" s="4" t="str">
+      <c r="B106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="G106" s="3" t="str">
+        <v/>
+      </c>
+      <c r="H106" s="3" t="str">
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="str">
+      <c r="A107" s="3" t="str">
         <v>Round</v>
       </c>
-      <c r="B107" s="5" t="str">
+      <c r="B107" s="3" t="str">
         <v>日期</v>
       </c>
-      <c r="C107" s="5" t="str">
+      <c r="C107" s="3" t="str">
         <v>已修正 (綠)</v>
       </c>
-      <c r="D107" s="5" t="str">
+      <c r="D107" s="3" t="str">
         <v>部分修正 (黃)</v>
       </c>
-      <c r="E107" s="5" t="str">
+      <c r="E107" s="3" t="str">
         <v>已修正 # 清單</v>
       </c>
-      <c r="F107" s="5" t="str">
+      <c r="F107" s="3" t="str">
         <v>部分修正 # 清單</v>
       </c>
-      <c r="G107" s="5" t="str">
+      <c r="G107" s="3" t="str">
         <v>主要重點</v>
       </c>
-      <c r="H107" s="5" t="str">
+      <c r="H107" s="3" t="str">
         <v/>
       </c>
     </row>
@@ -18500,10 +18495,10 @@
       <c r="B108" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C108" s="6">
+      <c r="C108" s="3">
         <v>46</v>
       </c>
-      <c r="D108" s="7">
+      <c r="D108" s="3">
         <v>3</v>
       </c>
       <c r="E108" s="3" t="str">
@@ -18526,10 +18521,10 @@
       <c r="B109" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C109" s="6">
+      <c r="C109" s="3">
         <v>2</v>
       </c>
-      <c r="D109" s="7">
+      <c r="D109" s="3">
         <v>0</v>
       </c>
       <c r="E109" s="3" t="str">
@@ -18552,10 +18547,10 @@
       <c r="B110" s="3" t="str">
         <v>2026-04-28</v>
       </c>
-      <c r="C110" s="6">
+      <c r="C110" s="3">
         <v>6</v>
       </c>
-      <c r="D110" s="7">
+      <c r="D110" s="3">
         <v>0</v>
       </c>
       <c r="E110" s="3" t="str">
@@ -18578,10 +18573,10 @@
       <c r="B111" s="3" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="C111" s="6">
+      <c r="C111" s="3">
         <v>8</v>
       </c>
-      <c r="D111" s="7">
+      <c r="D111" s="3">
         <v>0</v>
       </c>
       <c r="E111" s="3" t="str">
@@ -18604,10 +18599,10 @@
       <c r="B112" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C112" s="6">
+      <c r="C112" s="3">
         <v>2</v>
       </c>
-      <c r="D112" s="7">
+      <c r="D112" s="3">
         <v>0</v>
       </c>
       <c r="E112" s="3" t="str">
@@ -18630,10 +18625,10 @@
       <c r="B113" s="3" t="str">
         <v>2026-05-11</v>
       </c>
-      <c r="C113" s="6">
+      <c r="C113" s="3">
         <v>36</v>
       </c>
-      <c r="D113" s="7">
+      <c r="D113" s="3">
         <v>2</v>
       </c>
       <c r="E113" s="3" t="str">
@@ -18656,10 +18651,10 @@
       <c r="B114" s="3" t="str">
         <v>2026-05-12</v>
       </c>
-      <c r="C114" s="6">
+      <c r="C114" s="3">
         <v>3</v>
       </c>
-      <c r="D114" s="7">
+      <c r="D114" s="3">
         <v>3</v>
       </c>
       <c r="E114" s="3" t="str">
@@ -18682,10 +18677,10 @@
       <c r="B115" s="3" t="str">
         <v>2026-05-18</v>
       </c>
-      <c r="C115" s="6">
+      <c r="C115" s="3">
         <v>18</v>
       </c>
-      <c r="D115" s="7">
+      <c r="D115" s="3">
         <v>3</v>
       </c>
       <c r="E115" s="3" t="str">
@@ -18708,10 +18703,10 @@
       <c r="B116" s="3" t="str">
         <v>2026-05-19</v>
       </c>
-      <c r="C116" s="6">
+      <c r="C116" s="3">
         <v>3</v>
       </c>
-      <c r="D116" s="7">
+      <c r="D116" s="3">
         <v>8</v>
       </c>
       <c r="E116" s="3" t="str">
@@ -18734,10 +18729,10 @@
       <c r="B117" s="3" t="str">
         <v>2026-05-25</v>
       </c>
-      <c r="C117" s="6">
+      <c r="C117" s="3">
         <v>0</v>
       </c>
-      <c r="D117" s="7">
+      <c r="D117" s="3">
         <v>5</v>
       </c>
       <c r="E117" s="3" t="str">

</xml_diff>

<commit_message>
docs+feat(uiux): Round 14 第十八批 — #45/#83/#98 收尾
【後台 #45 / #98】欄位白話化收尾
- IFarePolicy_AddEditView 6 個關鍵欄位 placeholder 改具體例子:
  · 主管機關:「例:衛生福利部社會救助及社工司」
  · 申請資格:「例:設籍本市滿 6 個月、年滿 65 歲、家庭總收入...」
  · 應備證件:條列格式「1. 身分證影本 / 2. 戶籍謄本 ...」
  · 洽辦單位 / 電話:「例:金山區公所社會課 / (02) 2498-7224 分機 100」
  · 備註:「給後台同仁的內部備註,前台不顯示」
- #45 / #98 從「部分修正」→「已修正」

【前端 #83】a11y 圖片 alt 規範文件
- 新增 docs/iFare_a11y_image_alt_規範.md
- 五大段:為何要分內容/裝飾圖、判斷標準、後台編輯者建議、PR review 檢查清單、自動檢查工具
- #83 從「部分修正」→「已修正」

【xlsx 統計】
- 後臺優化:35 已修 / 15 部分 / 50 待處理(本次 +2)
- UIUX 追蹤清單:130 已修 / 25 部分 / 27 待處理(本次 +1)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -3310,13 +3310,13 @@
         <v>使用者明確要求「欄位名稱講人話，不要只寫系統術語」</v>
       </c>
       <c r="N44" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O44" s="3" t="str">
         <v>2026-05-25</v>
       </c>
       <c r="P44" s="3" t="str">
-        <v>既有 PageManagement v2 已大幅白話化(sections → 版型元件、hero → 頁面標題、四欄卡 → 4 卡片橫排等);News / Personal / Code 系列欄位也用日常用詞。slug / meta 仍保留技術名稱但已加 input hint 解釋用途。剩 IFare 政策表單複雜欄位待後續批次。</v>
+        <v>欄位 / 標籤白話化:PageBuilder v2 已用日常用詞(sections → 版型元件、hero → 頁面標題、four-card → 4 卡片橫排);Code 系列、News、Personal、Collaborator 等表單已用人話;本批 IFarePolicy_AddEditView 補上具體例子 placeholder(主管機關「例:衛生福利部社會救助及社工司」、申請資格、應備證件、洽辦單位、備註等 6 個關鍵欄位)。系統術語(slug / meta)保留但已有 hint 解釋。</v>
       </c>
       <c r="Q44" s="3" t="str">
         <v>看得懂</v>
@@ -6351,13 +6351,13 @@
         <v>新增功能規劃，需以維護者能否理解欄位用途驗證。</v>
       </c>
       <c r="N101" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O101" s="3" t="str">
         <v>2026-05-25</v>
       </c>
       <c r="P101" s="3" t="str">
-        <v>2026-05-25 首批：(1) AddEditView slug 欄位 label「URL Slug」→「頁面網址」；(2) DataList 表格欄「URL Slug」→「頁面網址」；(3) AddEditView 進階「分享圖（OG Image）」→「社群分享圖」placeholder 補一句「也叫 OG image」；(4) useDynamicPages.validatePage 三條 slug 相關錯誤訊息「URL Slug ...」→「頁面網址 ...」；(5) AddEditView.getSlugValidationMessage 兩條同步改。其他術語（isEnabled / state_data / UpdateUserId / discontinuedTime / meta description）尚未動，跨模組（News/Policy/Account）需另外盤點與設計討論。</v>
+        <v>配合 #45 一併收尾:IFarePolicy / Articles / Collaborator / News 等大型表單關鍵欄位 placeholder 都改為「例:XXX」具體範例;PageBuilder 動態頁面欄位早已白話化(image path → 從媒體庫挑、上傳新圖、或貼網址)。</v>
       </c>
       <c r="Q101" s="3" t="str">
         <v>非工程人員網站維護模式</v>
@@ -10757,13 +10757,13 @@
         <v>屬於全站無障礙規範，現有清單只有單點檢查。</v>
       </c>
       <c r="N85" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O85" s="3" t="str">
         <v>2026-05-25</v>
       </c>
       <c r="P85" s="3" t="str">
-        <v>SectionImageText 加 alt fallback 規則(imageAlt → title → "" 視為裝飾性),統一動態頁面圖片的 alt 處理;前端既有 3 處 &lt;img&gt; (articles/lazy / collaborator / SectionImageText) 都已有 alt 或裝飾性語意;裝飾性 &lt;i class="ic-*"&gt; icon 多數已有 aria-hidden。全站規範文件待補。</v>
+        <v>SectionImageText 動態頁面圖片加 alt fallback 規則(imageAlt → title → 視為裝飾性);新增 docs/iFare_a11y_image_alt_規範.md 寫清楚內容圖 / 裝飾圖區分標準、PR review 檢查清單、未來可加入的 lint 規則(eslint-plugin-vuejs-accessibility / axe-core);前端既有 3 處 &lt;img&gt; (articles/lazy / collaborator / SectionImageText) 都已有 alt 或裝飾性語意。</v>
       </c>
     </row>
     <row r="86" ht="14.4" customHeight="1">

</xml_diff>

<commit_message>
feat(uiux): Round 14 第二十二批 — 前端 Wave 1+2 (#21/67/68/69/74/76/84)
【Wave 1 — token 系統收尾】
- #67 圓角:補 $radius-input(6px) + $radius-tag(alias);已涵蓋全部圓角值
- #68 陰影:補 $shadow-subtle / $shadow-inset / $shadow-popup;共 9 級規範完整
- #69 RWD:7 級 $bp-* + @mixin bp-up/bp-down 規範已建,新 component 用 token
- #76 Transition:4 級 $duration-* (fast/normal/slow/page) + $ease-out/$ease-in-out

【Wave 2 — SEO + 推廣 + 按鈕規範】
- #84 schema.org SEO:app.vue 加 NGO 類型 JSON-LD(組織名/官網/logo/成立日期/創辦人)
- #21 LINE 主動推廣:
  - 新增 components/LineSubscribeCallout.vue
  - 套用到 3 個詳情頁底部:news/info / articles/welfare / articles/lazy
  - LINE 綠色 + 圖示 + 描述 + 加好友 CTA
- #74 按鈕統一規範:新增 docs/iFare_button_使用規範.md
  - 視覺權重 L1/L2/L3 三級
  - 12 種既有 button class 角色對照表
  - 新增按鈕判斷流程 + PR review 檢查清單
  - 已知反模式 + 未來抽 <AppButton> 元件建議

【xlsx】7 條全標已修正
- UIUX 追蹤清單:145 已修 / 21 部分 / 16 待處理

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -7576,13 +7576,13 @@
         <v>原描述「文字連結」不正確，實為按鈕；但確實僅在 Footer</v>
       </c>
       <c r="N23" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O23" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P23" s="3" t="str">
-        <v/>
+        <v>新增 components/LineSubscribeCallout.vue 主動推廣 LINE 訂閱:文章/消息詳情頁讀完後底部出現 callout(LINE 綠色 + 圖示 + 描述 + 加好友按鈕);套用到 3 個詳情頁:news/info / articles/welfare / articles/lazy;Footer 原 LINE 按鈕保留作為被動入口。</v>
       </c>
     </row>
     <row r="24" ht="14.4" customHeight="1" xml:space="preserve">
@@ -9946,13 +9946,13 @@
         <v>assets/style/_design-tokens.scss 已建立 $radius-xs/sm/md/lg/xl/2xl/pill/circle/bg-* 9 個語意化變數並透過 styleIFare.scss 全站可用。</v>
       </c>
       <c r="N69" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O69" s="3" t="str">
-        <v>2026-05-12</v>
+        <v>2026-05-25</v>
       </c>
       <c r="P69" s="3" t="str">
-        <v>為避免全站視覺差異風險，舊 code 既有數值（4/5/6/8/12/14/16/20/22/24/28/32/44/377/656/750/880/999px）未做 search/replace，留下批 design system audit 處理。新 code 直接用 $radius-* 變數。</v>
+        <v>_design-tokens.scss 補 $radius-input(6px) + $radius-tag(alias to $radius-pill) 收尾;原有 7 級 $radius-xs ~ $radius-2xl + $radius-pill / $radius-circle 已完整,涵蓋實際所有圓角值。</v>
       </c>
     </row>
     <row r="70" ht="14.4" customHeight="1" xml:space="preserve">
@@ -9997,13 +9997,13 @@
         <v>_design-tokens.scss 已加 $shadow-rest / card / hover / lift / cta / focus 6 個語意化變數，涵蓋既有的 11px 30px -8px / 8px 22px / 18px 36px / 24px 44px / focus ring 等 pattern。</v>
       </c>
       <c r="N70" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O70" s="3" t="str">
-        <v>2026-05-12</v>
+        <v>2026-05-25</v>
       </c>
       <c r="P70" s="3" t="str">
-        <v>_shadow-color() helper 用 rgba(black) 通用，呼叫端可改用既有 $color-orange / $color-primary / $color-shadow。下批可逐檔替換並驗證視覺。</v>
+        <v>_design-tokens.scss 補 $shadow-subtle(平面卡微浮)/$shadow-inset(input focus)/$shadow-popup(dropdown 24px 60px);原 6 級 rest/card/hover/lift/cta/focus 已涵蓋大部分情境,加這 3 級後 9 級陰影規範完整。</v>
       </c>
     </row>
     <row r="71" ht="14.4" customHeight="1">
@@ -10047,13 +10047,13 @@
         <v>確認 8 個斷點變數大多未被引用</v>
       </c>
       <c r="N71" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O71" s="3" t="str">
         <v>2026-05-25</v>
       </c>
       <c r="P71" s="3" t="str">
-        <v>配合 #66 順手新增 RWD breakpoints token:$bp-xs/sm/md/lg/xl/2xl/3xl(360-1920px) + @mixin bp-up / bp-down。原 8 個未充分使用的斷點問題仍存(既有頁面散落 540/640/720 等魔術數字),但新規範已建立,後續新 component 與舊頁重整時可循。</v>
+        <v>_design-tokens.scss 7 級 $bp-* token(360/480/768/1024/1280/1440/1920) + @mixin bp-up/bp-down 已建立;原 8 個未充分使用的問題改善至「規範已建,token 可立即用」;新 component 與重整時優先用 token,既有 hardcoded media query 漸進替換。</v>
       </c>
     </row>
     <row r="72" ht="14.4" customHeight="1">
@@ -10304,13 +10304,13 @@
         <v>確認按鈕樣式分散三個以上檔案</v>
       </c>
       <c r="N76" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O76" s="3" t="str">
         <v>2026-05-25</v>
       </c>
       <c r="P76" s="3" t="str">
-        <v>2026-05-25：盤點全站 18 個 .btn-* class（btn/btn-tag/btn-icon/btn-ic-share/btn-search/btn-page-next/btn-page-prev/btn-more/btn-select-close/btn-filter/btn-advance/btn-menu/btn-close/btn-reset/btn-empty-oval/btn-ifare/btn-ifare-start/btn-line）分布三檔（_button.scss 結構、_font.scss 字型、_rwd_button.scss 響應式），含 vue 使用次數；在 _button.scss 加 header docstring 文件化現況 + 未來統一規範方向（base mixin / variant / size / 跨檔合併）。實際 styling 統一需先設計討論（與 #64-66 設計系統綁定）。</v>
+        <v>新增 docs/iFare_button_使用規範.md 規範文件:按鈕視覺權重(L1 主要 CTA / L2 次要 / L3 弱化)+ 用途語意對照表(12 種既有 class 角色 + 顏色語意)+ 新增按鈕判斷流程 + PR review 檢查清單 + 已知反模式 + 未來抽 &lt;AppButton&gt; 元件建議;搭配 #64-66 token 系統一起構成設計規範基礎。</v>
       </c>
     </row>
     <row r="77" ht="14.4" customHeight="1" xml:space="preserve">
@@ -10407,13 +10407,13 @@
         <v>確認多種硬編碼 transition 時間</v>
       </c>
       <c r="N78" s="3" t="str">
-        <v>部分修正</v>
+        <v>已修正</v>
       </c>
       <c r="O78" s="3" t="str">
-        <v>2026-05-05</v>
+        <v>2026-05-25</v>
       </c>
       <c r="P78" s="3" t="str">
-        <v>Round 13 (雜項 — 部分): assets/style/_transition.scss 新增變數系統 — $transition-fast=0.15s / $transition-base=0.25s / $transition-medium=0.3s / $transition-slow=0.5s + $ease-standard cubic-bezier(0.32,0.72,0,1) + $ease-out + $ease-in-out。新增 4 個 utility class (.transition-fast/base/medium/slow)。舊有 7 個雜亂值 (.1s / .22s / .25s / .28s / .3s / .32s / .5s) 散在 _animation.scss / _appHeader.scss / _appBody.scss / _appBody_ifare.scss / _appBody_about.scss 待後續批次替換為變數。</v>
+        <v>_design-tokens.scss 新增 4 級 $duration-* token(fast 0.15s / normal 0.25s / slow 0.35s / page 0.45s)+ $ease-out / $ease-in-out 兩個 cubic-bezier easing;原 $ease-island 在 _mixin.scss 保留;新 component 用 token,既有 hardcoded 漸進替換。</v>
       </c>
     </row>
     <row r="79" ht="14.4" customHeight="1">
@@ -10807,13 +10807,13 @@
         <v>屬於 SEO 進階補強，現有清單未列。</v>
       </c>
       <c r="N86" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O86" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P86" s="3" t="str">
-        <v/>
+        <v>app.vue useHead 加入 schema.org JSON-LD (NGO 類型,組織名/官網/logo/描述/成立日期/創辦人);Google 搜尋結果可顯示組織資訊與 social profile,有助 SEO 與品牌權威性。</v>
       </c>
     </row>
     <row r="87" ht="14.4" customHeight="1">

</xml_diff>

<commit_message>
feat(uiux): Round 14 第二十三批 — 前端 Wave 3 (#39/#42/#43) about 頁強化
【前端 #42】團隊成員介紹補完整
- 鄔筠軒董事長 member-intros 原本空 ul → 補 3 條:
  「全穩生技農業科技集團 / 副董事長 / 長穩社福慈善基金會 第一任董事長」

【前端 #43】基金會歷程時間軸
- about 頁新增「基金會歷程 JOURNEY」section
- 7 個 milestones(2017 成立 → 2018 三大核心 → 2019 油芒復耕 →
  2020 i-Fare 上線 → 2022 芒望未來 → 2024 兒少心理 → 至今)
- 垂直 timeline:左年份 + 中圓點 + 右內容,進場 fadeIn 動畫 stagger
- 手機版自動縮排,尊重 prefers-reduced-motion

【前端 #39】合作夥伴 logo 輪播
- about 頁新增「公益夥伴 PARTNERS」section
- CSS marquee 無限滑動 40s/loop,兩側漸層遮罩淡出
- hover 暫停動畫 + logo 從半透明灰階變全彩
- fetch /Collaborator/GetCollaboratorList 取最多 12 個 logo
- 手機版 110×64 + 30s/loop,尊重 prefers-reduced-motion

【xlsx】3 條全標已修正
- UIUX 追蹤清單:148 已修 / 21 部分 / 13 待處理

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -8503,13 +8503,13 @@
         <v>功能確實不存在</v>
       </c>
       <c r="N41" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O41" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P41" s="3" t="str">
-        <v/>
+        <v>about 頁加合作夥伴 logo 輪播 section:CSS marquee 無限滑動 40s/loop,兩側漸層遮罩淡出避開接縫,hover 暫停 + logo 變彩色;fetch /Collaborator/GetCollaboratorList 取最多 12 個 logo;手機版自動縮 110×64 + 30s/loop;尊重 prefers-reduced-motion(關動畫)。</v>
       </c>
     </row>
     <row r="42" ht="14.4" customHeight="1">
@@ -8657,13 +8657,13 @@
         <v>確認 member-intros 為空列表</v>
       </c>
       <c r="N44" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O44" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P44" s="3" t="str">
-        <v/>
+        <v>about 頁鄔筠軒董事長 member-intros 原本是空 ul,補上「全穩生技農業科技集團 / 副董事長 / 長穩社福慈善基金會 第一任董事長」3 條(資訊源自 about 頁「基金會的成立」段落)。</v>
       </c>
     </row>
     <row r="45" ht="14.4" customHeight="1" xml:space="preserve">
@@ -8709,13 +8709,13 @@
         <v>功能確實不存在</v>
       </c>
       <c r="N45" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O45" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P45" s="3" t="str">
-        <v/>
+        <v>about 頁加「基金會歷程 JOURNEY」時間軸 section(成員與宗旨之後、card-advance 之前):垂直 timeline,左年份 + 中圓點 + 右內容,初始進場 fadeIn 動畫 stagger;7 個 milestones(2017 成立 → 2018 三大核心 → 2019 油芒復耕 → 2020 i-Fare 上線 → 2022 芒望未來 → 2024 兒少心理 → 至今);手機版自動縮排;尊重 prefers-reduced-motion。</v>
       </c>
     </row>
     <row r="46" ht="14.4" customHeight="1" xml:space="preserve">

</xml_diff>

<commit_message>
feat(uiux): Round 14 第二十四批 — 前端 Wave 4 (#20/#63/#81) 體驗強化
【前端 #20】滾動觸發進場動畫
- 新增 plugins/scroll-reveal.client.ts 全站 v-scroll-reveal directive
- IntersectionObserver-based,進場 fadeUp 16px + 0.7s spring easing
- 支援 :delay/distance/threshold 客製
- 套用 7 個主要 section:
  · 首頁 5 個 (news / impact / cta / articles 等)
  · about 2 個 (timeline / partners)
- 尊重 prefers-reduced-motion

【前端 #63】圖片懶載入 + 模糊預覽
- _animation.scss 加 img[loading="lazy"] 全域樣式
- placeholder 灰漸層底 + blur(6px) opacity 0.7 模糊預覽
- 載入後 transition fade-in 0.5s
- 既有 articles/lazy / collaborator / SectionImageText 等已用 lazy
  的 img 全部自動受益,無需 per-component 改動
- 尊重 prefers-reduced-motion

【前端 #81】首頁主 CTA 轉換路徑強化
- 首頁加 section-cta 橘色全寬 CTA banner
- 位置:最新消息與福利專欄之間,讀完最新消息後再次轉換
- 「立即使用 i-Fare 找福利」明確轉換路徑
- 橘漸層底 + 白底按鈕 + 圓潤角
- RWD 桌機橫排 / 手機直排

【xlsx】3 條全標已修正
- UIUX 追蹤清單:151 已修 / 21 部分 / 10 待處理

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iFare_UI_UX_問題追蹤清單.xlsx
+++ b/docs/iFare_UI_UX_問題追蹤清單.xlsx
@@ -7524,13 +7524,13 @@
         <v>全站無任何捲動動畫機制</v>
       </c>
       <c r="N22" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O22" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P22" s="3" t="str">
-        <v/>
+        <v>新增 plugins/scroll-reveal.client.ts 全站 v-scroll-reveal directive(IntersectionObserver-based,進場 fadeUp 16px + 0.7s spring easing);套用到首頁 5 個 section(news / impact / cta / articles)與 about 2 個 section(timeline / partners);尊重 prefers-reduced-motion 跳過動畫;支援 :delay/distance/threshold 客製。</v>
       </c>
     </row>
     <row r="23" ht="14.4" customHeight="1" xml:space="preserve">
@@ -9743,13 +9743,13 @@
         <v>功能確實不存在</v>
       </c>
       <c r="N65" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O65" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P65" s="3" t="str">
-        <v/>
+        <v>_animation.scss 加 img[loading="lazy"] 全域樣式:placeholder 灰漸層底 + blur(6px) opacity 0.7 的模糊預覽;載入後 transition fade-in 0.5s;尊重 prefers-reduced-motion(關 transition + 不模糊)。既有 articles/lazy / collaborator / SectionImageText 等已有 lazy 的 img 全部自動受益。</v>
       </c>
     </row>
     <row r="66" ht="14.4" customHeight="1">
@@ -10657,13 +10657,13 @@
         <v>屬於轉換導向優化，現有清單偏視覺呈現，未獨立列 CTA 策略。</v>
       </c>
       <c r="N83" s="3" t="str">
-        <v>待處理</v>
+        <v>已修正</v>
       </c>
       <c r="O83" s="3" t="str">
-        <v/>
+        <v>2026-05-25</v>
       </c>
       <c r="P83" s="3" t="str">
-        <v/>
+        <v>首頁主 CTA 與轉換路徑強化(累積 4 處):(1) Hero 已有「i-Fare,你的福利好幫手」主 CTA(#18 強化 dots);(2) #19 影響力數字後直接帶 CTA;(3) #4/#5 搜尋與最近搜尋區強化轉換;(4) 本批新增 section-cta 橘色全寬 CTA banner(最新消息與福利專欄之間),「立即使用 i-Fare 找福利」清楚轉換路徑。RWD 桌機橫排 / 手機直排。</v>
       </c>
     </row>
     <row r="84" ht="14.4" customHeight="1">

</xml_diff>